<commit_message>
- fixed using filters on Reports page - tuned query and mapping
</commit_message>
<xml_diff>
--- a/api/templates/results_dr_tb_10a/en.xlsx
+++ b/api/templates/results_dr_tb_10a/en.xlsx
@@ -2735,6 +2735,452 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="6" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="6" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
@@ -2787,14 +3233,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="30" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2804,22 +3242,6 @@
     <xf numFmtId="0" fontId="30" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
@@ -2828,531 +3250,97 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="56" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="57" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="57" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="56" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="76" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="52" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="52" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="51" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="58" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
@@ -3370,64 +3358,76 @@
       <alignment horizontal="left" shrinkToFit="1"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="76" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="57" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="57" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="57" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="53" fillId="6" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="53" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="53" fillId="6" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
   </cellXfs>
@@ -3887,26 +3887,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="165" t="s">
+      <c r="A1" s="232" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="165"/>
-      <c r="C1" s="165"/>
-      <c r="D1" s="165"/>
-      <c r="E1" s="165"/>
-      <c r="F1" s="165"/>
-      <c r="G1" s="165"/>
-      <c r="H1" s="165"/>
-      <c r="I1" s="165"/>
-      <c r="J1" s="165"/>
-      <c r="K1" s="165"/>
-      <c r="L1" s="165"/>
-      <c r="M1" s="165"/>
-      <c r="N1" s="165"/>
-      <c r="O1" s="165"/>
-      <c r="P1" s="165"/>
-      <c r="Q1" s="165"/>
-      <c r="R1" s="165"/>
+      <c r="B1" s="232"/>
+      <c r="C1" s="232"/>
+      <c r="D1" s="232"/>
+      <c r="E1" s="232"/>
+      <c r="F1" s="232"/>
+      <c r="G1" s="232"/>
+      <c r="H1" s="232"/>
+      <c r="I1" s="232"/>
+      <c r="J1" s="232"/>
+      <c r="K1" s="232"/>
+      <c r="L1" s="232"/>
+      <c r="M1" s="232"/>
+      <c r="N1" s="232"/>
+      <c r="O1" s="232"/>
+      <c r="P1" s="232"/>
+      <c r="Q1" s="232"/>
+      <c r="R1" s="232"/>
       <c r="S1" s="2" t="s">
         <v>70</v>
       </c>
@@ -3916,54 +3916,54 @@
       <c r="X1" s="1"/>
     </row>
     <row r="2" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="165" t="s">
+      <c r="A2" s="232" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="165"/>
-      <c r="C2" s="165"/>
-      <c r="D2" s="165"/>
-      <c r="E2" s="165"/>
-      <c r="F2" s="165"/>
-      <c r="G2" s="165"/>
-      <c r="H2" s="165"/>
-      <c r="I2" s="165"/>
-      <c r="J2" s="165"/>
-      <c r="K2" s="165"/>
-      <c r="L2" s="165"/>
-      <c r="M2" s="165"/>
-      <c r="N2" s="165"/>
-      <c r="O2" s="165"/>
-      <c r="P2" s="165"/>
-      <c r="Q2" s="165"/>
-      <c r="R2" s="165"/>
-      <c r="S2" s="165"/>
-      <c r="T2" s="165"/>
-      <c r="U2" s="165"/>
+      <c r="B2" s="232"/>
+      <c r="C2" s="232"/>
+      <c r="D2" s="232"/>
+      <c r="E2" s="232"/>
+      <c r="F2" s="232"/>
+      <c r="G2" s="232"/>
+      <c r="H2" s="232"/>
+      <c r="I2" s="232"/>
+      <c r="J2" s="232"/>
+      <c r="K2" s="232"/>
+      <c r="L2" s="232"/>
+      <c r="M2" s="232"/>
+      <c r="N2" s="232"/>
+      <c r="O2" s="232"/>
+      <c r="P2" s="232"/>
+      <c r="Q2" s="232"/>
+      <c r="R2" s="232"/>
+      <c r="S2" s="232"/>
+      <c r="T2" s="232"/>
+      <c r="U2" s="232"/>
       <c r="V2" s="1"/>
       <c r="W2" s="1"/>
       <c r="X2" s="1"/>
     </row>
     <row r="3" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="165" t="s">
+      <c r="A3" s="232" t="s">
         <v>80</v>
       </c>
-      <c r="B3" s="165"/>
-      <c r="C3" s="165"/>
-      <c r="D3" s="165"/>
-      <c r="E3" s="165"/>
-      <c r="F3" s="165"/>
-      <c r="G3" s="165"/>
-      <c r="H3" s="165"/>
-      <c r="I3" s="165"/>
-      <c r="J3" s="165"/>
-      <c r="K3" s="165"/>
-      <c r="L3" s="165"/>
-      <c r="M3" s="165"/>
-      <c r="N3" s="165"/>
-      <c r="O3" s="165"/>
-      <c r="P3" s="165"/>
-      <c r="Q3" s="165"/>
-      <c r="R3" s="165"/>
+      <c r="B3" s="232"/>
+      <c r="C3" s="232"/>
+      <c r="D3" s="232"/>
+      <c r="E3" s="232"/>
+      <c r="F3" s="232"/>
+      <c r="G3" s="232"/>
+      <c r="H3" s="232"/>
+      <c r="I3" s="232"/>
+      <c r="J3" s="232"/>
+      <c r="K3" s="232"/>
+      <c r="L3" s="232"/>
+      <c r="M3" s="232"/>
+      <c r="N3" s="232"/>
+      <c r="O3" s="232"/>
+      <c r="P3" s="232"/>
+      <c r="Q3" s="232"/>
+      <c r="R3" s="232"/>
       <c r="S3" s="43"/>
       <c r="T3" s="43"/>
       <c r="U3" s="43"/>
@@ -3972,29 +3972,29 @@
       <c r="X3" s="1"/>
     </row>
     <row r="4" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="177" t="s">
+      <c r="A4" s="244" t="s">
         <v>72</v>
       </c>
-      <c r="B4" s="177"/>
-      <c r="C4" s="177"/>
-      <c r="D4" s="177"/>
-      <c r="E4" s="177"/>
-      <c r="F4" s="177"/>
-      <c r="G4" s="177"/>
-      <c r="H4" s="177"/>
-      <c r="I4" s="177"/>
-      <c r="J4" s="177"/>
-      <c r="K4" s="177"/>
-      <c r="L4" s="177"/>
-      <c r="M4" s="177"/>
-      <c r="N4" s="177"/>
-      <c r="O4" s="177"/>
-      <c r="P4" s="177"/>
-      <c r="Q4" s="177"/>
-      <c r="R4" s="177"/>
-      <c r="S4" s="177"/>
-      <c r="T4" s="177"/>
-      <c r="U4" s="177"/>
+      <c r="B4" s="244"/>
+      <c r="C4" s="244"/>
+      <c r="D4" s="244"/>
+      <c r="E4" s="244"/>
+      <c r="F4" s="244"/>
+      <c r="G4" s="244"/>
+      <c r="H4" s="244"/>
+      <c r="I4" s="244"/>
+      <c r="J4" s="244"/>
+      <c r="K4" s="244"/>
+      <c r="L4" s="244"/>
+      <c r="M4" s="244"/>
+      <c r="N4" s="244"/>
+      <c r="O4" s="244"/>
+      <c r="P4" s="244"/>
+      <c r="Q4" s="244"/>
+      <c r="R4" s="244"/>
+      <c r="S4" s="244"/>
+      <c r="T4" s="244"/>
+      <c r="U4" s="244"/>
       <c r="V4" s="4"/>
       <c r="W4" s="4"/>
       <c r="X4" s="4"/>
@@ -4030,11 +4030,11 @@
         <v>87</v>
       </c>
       <c r="B6" s="5"/>
-      <c r="C6" s="141"/>
-      <c r="D6" s="141"/>
-      <c r="E6" s="141"/>
-      <c r="F6" s="141"/>
-      <c r="G6" s="141"/>
+      <c r="C6" s="255"/>
+      <c r="D6" s="255"/>
+      <c r="E6" s="255"/>
+      <c r="F6" s="255"/>
+      <c r="G6" s="255"/>
       <c r="I6" s="1"/>
       <c r="J6" s="7" t="s">
         <v>16</v>
@@ -4043,11 +4043,8 @@
       <c r="M6" s="62" t="s">
         <v>14</v>
       </c>
-      <c r="N6" s="215" t="str">
-        <f>IF(L6="","",VLOOKUP(L6,#REF!,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="O6" s="215"/>
+      <c r="N6" s="317"/>
+      <c r="O6" s="317"/>
       <c r="P6" s="8" t="s">
         <v>15</v>
       </c>
@@ -4058,11 +4055,11 @@
         <v>9</v>
       </c>
       <c r="B7" s="5"/>
-      <c r="C7" s="142"/>
-      <c r="D7" s="142"/>
-      <c r="E7" s="142"/>
-      <c r="F7" s="142"/>
-      <c r="G7" s="142"/>
+      <c r="C7" s="256"/>
+      <c r="D7" s="256"/>
+      <c r="E7" s="256"/>
+      <c r="F7" s="256"/>
+      <c r="G7" s="256"/>
       <c r="I7" s="6"/>
       <c r="J7" s="9" t="s">
         <v>69</v>
@@ -4070,36 +4067,36 @@
       <c r="K7" s="9"/>
       <c r="L7" s="9"/>
       <c r="M7" s="9"/>
-      <c r="N7" s="147"/>
-      <c r="O7" s="147"/>
-      <c r="P7" s="147"/>
-      <c r="Q7" s="147"/>
-      <c r="R7" s="147"/>
-      <c r="S7" s="147"/>
+      <c r="N7" s="261"/>
+      <c r="O7" s="261"/>
+      <c r="P7" s="261"/>
+      <c r="Q7" s="261"/>
+      <c r="R7" s="261"/>
+      <c r="S7" s="261"/>
     </row>
     <row r="8" spans="1:603" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="5"/>
-      <c r="C8" s="143"/>
-      <c r="D8" s="143"/>
-      <c r="E8" s="143"/>
-      <c r="F8" s="143"/>
-      <c r="G8" s="143"/>
+      <c r="C8" s="257"/>
+      <c r="D8" s="257"/>
+      <c r="E8" s="257"/>
+      <c r="F8" s="257"/>
+      <c r="G8" s="257"/>
       <c r="I8" s="6"/>
       <c r="J8" s="9" t="s">
         <v>68</v>
       </c>
       <c r="K8" s="9"/>
       <c r="L8" s="9"/>
-      <c r="M8" s="147"/>
-      <c r="N8" s="147"/>
-      <c r="O8" s="147"/>
-      <c r="P8" s="147"/>
-      <c r="Q8" s="147"/>
-      <c r="R8" s="147"/>
-      <c r="S8" s="147"/>
+      <c r="M8" s="261"/>
+      <c r="N8" s="261"/>
+      <c r="O8" s="261"/>
+      <c r="P8" s="261"/>
+      <c r="Q8" s="261"/>
+      <c r="R8" s="261"/>
+      <c r="S8" s="261"/>
     </row>
     <row r="9" spans="1:603" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="J9" s="9" t="s">
@@ -4107,8 +4104,8 @@
       </c>
       <c r="K9" s="9"/>
       <c r="L9" s="9"/>
-      <c r="M9" s="148"/>
-      <c r="N9" s="148"/>
+      <c r="M9" s="262"/>
+      <c r="N9" s="262"/>
       <c r="O9" s="64"/>
       <c r="P9" s="63"/>
     </row>
@@ -4116,16 +4113,16 @@
       <c r="J10" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="K10" s="149"/>
-      <c r="L10" s="149"/>
+      <c r="K10" s="263"/>
+      <c r="L10" s="263"/>
       <c r="M10" s="10"/>
       <c r="N10" s="11"/>
       <c r="O10" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="Q10" s="150"/>
-      <c r="R10" s="150"/>
-      <c r="S10" s="150"/>
+      <c r="Q10" s="264"/>
+      <c r="R10" s="264"/>
+      <c r="S10" s="264"/>
       <c r="T10" s="19"/>
     </row>
     <row r="11" spans="1:603" s="11" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4729,27 +4726,27 @@
       <c r="WE11" s="24"/>
     </row>
     <row r="12" spans="1:603" s="25" customFormat="1" ht="13.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="230" t="s">
+      <c r="A12" s="188" t="s">
         <v>74</v>
       </c>
-      <c r="B12" s="231"/>
-      <c r="C12" s="232"/>
-      <c r="D12" s="217" t="s">
+      <c r="B12" s="189"/>
+      <c r="C12" s="190"/>
+      <c r="D12" s="175" t="s">
         <v>85</v>
       </c>
-      <c r="E12" s="217"/>
-      <c r="F12" s="217"/>
-      <c r="G12" s="217"/>
+      <c r="E12" s="175"/>
+      <c r="F12" s="175"/>
+      <c r="G12" s="175"/>
       <c r="H12" s="67">
         <f>D26+E39</f>
         <v>0</v>
       </c>
       <c r="I12" s="24"/>
-      <c r="J12" s="314" t="s">
+      <c r="J12" s="251" t="s">
         <v>137</v>
       </c>
-      <c r="K12" s="314"/>
-      <c r="L12" s="314"/>
+      <c r="K12" s="251"/>
+      <c r="L12" s="251"/>
       <c r="M12" s="140"/>
       <c r="N12" s="24"/>
       <c r="O12" s="24"/>
@@ -5343,45 +5340,45 @@
       <c r="WE12" s="24"/>
     </row>
     <row r="13" spans="1:603" s="24" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="233"/>
-      <c r="B13" s="234"/>
-      <c r="C13" s="235"/>
-      <c r="D13" s="218" t="s">
+      <c r="A13" s="191"/>
+      <c r="B13" s="192"/>
+      <c r="C13" s="193"/>
+      <c r="D13" s="176" t="s">
         <v>77</v>
       </c>
-      <c r="E13" s="218"/>
-      <c r="F13" s="218"/>
-      <c r="G13" s="218"/>
+      <c r="E13" s="176"/>
+      <c r="F13" s="176"/>
+      <c r="G13" s="176"/>
       <c r="H13" s="68">
         <f>U26</f>
         <v>0</v>
       </c>
-      <c r="J13" s="314" t="s">
+      <c r="J13" s="251" t="s">
         <v>139</v>
       </c>
-      <c r="K13" s="314"/>
-      <c r="L13" s="314"/>
+      <c r="K13" s="251"/>
+      <c r="L13" s="251"/>
       <c r="M13" s="140"/>
     </row>
     <row r="14" spans="1:603" s="24" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="236"/>
-      <c r="B14" s="237"/>
-      <c r="C14" s="238"/>
-      <c r="D14" s="219" t="s">
+      <c r="A14" s="194"/>
+      <c r="B14" s="195"/>
+      <c r="C14" s="196"/>
+      <c r="D14" s="177" t="s">
         <v>3</v>
       </c>
-      <c r="E14" s="219"/>
-      <c r="F14" s="219"/>
-      <c r="G14" s="219"/>
+      <c r="E14" s="177"/>
+      <c r="F14" s="177"/>
+      <c r="G14" s="177"/>
       <c r="H14" s="69">
         <f>H12+H13</f>
         <v>0</v>
       </c>
-      <c r="J14" s="315" t="s">
+      <c r="J14" s="252" t="s">
         <v>138</v>
       </c>
-      <c r="K14" s="316"/>
-      <c r="L14" s="317"/>
+      <c r="K14" s="253"/>
+      <c r="L14" s="254"/>
       <c r="M14" s="140"/>
     </row>
     <row r="15" spans="1:603" s="25" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6592,11 +6589,11 @@
       <c r="WE16" s="24"/>
     </row>
     <row r="17" spans="1:603" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="253" t="s">
+      <c r="A17" s="151" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="254"/>
-      <c r="C17" s="254"/>
+      <c r="B17" s="152"/>
+      <c r="C17" s="152"/>
       <c r="D17" s="70">
         <f>D29+E41-D32-E43</f>
         <v>0</v>
@@ -6610,22 +6607,22 @@
         <v>0</v>
       </c>
       <c r="G17" s="24"/>
-      <c r="H17" s="223" t="s">
+      <c r="H17" s="181" t="s">
         <v>66</v>
       </c>
-      <c r="I17" s="223"/>
-      <c r="J17" s="223"/>
-      <c r="K17" s="223"/>
-      <c r="L17" s="224" t="s">
+      <c r="I17" s="181"/>
+      <c r="J17" s="181"/>
+      <c r="K17" s="181"/>
+      <c r="L17" s="182" t="s">
         <v>83</v>
       </c>
-      <c r="M17" s="225"/>
-      <c r="N17" s="226"/>
-      <c r="O17" s="227" t="s">
+      <c r="M17" s="183"/>
+      <c r="N17" s="184"/>
+      <c r="O17" s="185" t="s">
         <v>73</v>
       </c>
-      <c r="P17" s="228"/>
-      <c r="Q17" s="229"/>
+      <c r="P17" s="186"/>
+      <c r="Q17" s="187"/>
       <c r="R17" s="55" t="s">
         <v>3</v>
       </c>
@@ -7205,11 +7202,11 @@
       <c r="WE17" s="24"/>
     </row>
     <row r="18" spans="1:603" s="11" customFormat="1" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="253" t="s">
+      <c r="A18" s="151" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="254"/>
-      <c r="C18" s="254"/>
+      <c r="B18" s="152"/>
+      <c r="C18" s="152"/>
       <c r="D18" s="72">
         <f>D32+E43</f>
         <v>0</v>
@@ -7223,10 +7220,10 @@
         <v>0</v>
       </c>
       <c r="G18" s="24"/>
-      <c r="H18" s="223"/>
-      <c r="I18" s="223"/>
-      <c r="J18" s="223"/>
-      <c r="K18" s="223"/>
+      <c r="H18" s="181"/>
+      <c r="I18" s="181"/>
+      <c r="J18" s="181"/>
+      <c r="K18" s="181"/>
       <c r="L18" s="56"/>
       <c r="M18" s="57"/>
       <c r="N18" s="57"/>
@@ -7813,11 +7810,11 @@
       <c r="WE18" s="24"/>
     </row>
     <row r="19" spans="1:603" s="11" customFormat="1" ht="13.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="253" t="s">
+      <c r="A19" s="151" t="s">
         <v>65</v>
       </c>
-      <c r="B19" s="254"/>
-      <c r="C19" s="254"/>
+      <c r="B19" s="152"/>
+      <c r="C19" s="152"/>
       <c r="D19" s="51"/>
       <c r="E19" s="59"/>
       <c r="F19" s="71">
@@ -8412,11 +8409,11 @@
       <c r="WE19" s="24"/>
     </row>
     <row r="20" spans="1:603" s="11" customFormat="1" ht="13.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="239" t="s">
+      <c r="A20" s="197" t="s">
         <v>114</v>
       </c>
-      <c r="B20" s="240"/>
-      <c r="C20" s="240"/>
+      <c r="B20" s="198"/>
+      <c r="C20" s="198"/>
       <c r="D20" s="74">
         <f>H12-D29-E41</f>
         <v>0</v>
@@ -9620,45 +9617,45 @@
       <c r="E22" s="37"/>
     </row>
     <row r="23" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="266" t="s">
+      <c r="A23" s="164" t="s">
         <v>1</v>
       </c>
-      <c r="B23" s="262" t="s">
+      <c r="B23" s="160" t="s">
         <v>86</v>
       </c>
-      <c r="C23" s="263"/>
-      <c r="D23" s="264"/>
-      <c r="E23" s="163" t="s">
+      <c r="C23" s="161"/>
+      <c r="D23" s="162"/>
+      <c r="E23" s="271" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="164"/>
-      <c r="G23" s="164"/>
-      <c r="H23" s="164"/>
-      <c r="I23" s="164"/>
-      <c r="J23" s="164"/>
-      <c r="K23" s="164"/>
-      <c r="L23" s="164"/>
-      <c r="M23" s="164"/>
-      <c r="N23" s="164"/>
-      <c r="O23" s="164"/>
-      <c r="P23" s="164"/>
-      <c r="Q23" s="164"/>
-      <c r="R23" s="164"/>
-      <c r="S23" s="164"/>
-      <c r="T23" s="164"/>
-      <c r="U23" s="151" t="s">
+      <c r="F23" s="272"/>
+      <c r="G23" s="272"/>
+      <c r="H23" s="272"/>
+      <c r="I23" s="272"/>
+      <c r="J23" s="272"/>
+      <c r="K23" s="272"/>
+      <c r="L23" s="272"/>
+      <c r="M23" s="272"/>
+      <c r="N23" s="272"/>
+      <c r="O23" s="272"/>
+      <c r="P23" s="272"/>
+      <c r="Q23" s="272"/>
+      <c r="R23" s="272"/>
+      <c r="S23" s="272"/>
+      <c r="T23" s="272"/>
+      <c r="U23" s="265" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="24" spans="1:603" ht="66.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="267"/>
+      <c r="A24" s="165"/>
       <c r="B24" s="100" t="s">
         <v>46</v>
       </c>
       <c r="C24" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="D24" s="260" t="s">
+      <c r="D24" s="158" t="s">
         <v>81</v>
       </c>
       <c r="E24" s="20" t="s">
@@ -9685,31 +9682,31 @@
       <c r="L24" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="M24" s="185" t="s">
+      <c r="M24" s="201" t="s">
         <v>34</v>
       </c>
-      <c r="N24" s="185"/>
-      <c r="O24" s="185"/>
-      <c r="P24" s="185" t="s">
+      <c r="N24" s="201"/>
+      <c r="O24" s="201"/>
+      <c r="P24" s="201" t="s">
         <v>36</v>
       </c>
-      <c r="Q24" s="185"/>
-      <c r="R24" s="185"/>
-      <c r="S24" s="187" t="s">
+      <c r="Q24" s="201"/>
+      <c r="R24" s="201"/>
+      <c r="S24" s="230" t="s">
         <v>38</v>
       </c>
-      <c r="T24" s="187"/>
-      <c r="U24" s="152"/>
+      <c r="T24" s="230"/>
+      <c r="U24" s="266"/>
     </row>
     <row r="25" spans="1:603" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="268"/>
+      <c r="A25" s="166"/>
       <c r="B25" s="52" t="s">
         <v>18</v>
       </c>
       <c r="C25" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="D25" s="261"/>
+      <c r="D25" s="159"/>
       <c r="E25" s="52" t="s">
         <v>23</v>
       </c>
@@ -9734,297 +9731,297 @@
       <c r="L25" s="53" t="s">
         <v>37</v>
       </c>
-      <c r="M25" s="186" t="s">
+      <c r="M25" s="202" t="s">
         <v>39</v>
       </c>
-      <c r="N25" s="186"/>
-      <c r="O25" s="186"/>
-      <c r="P25" s="186" t="s">
+      <c r="N25" s="202"/>
+      <c r="O25" s="202"/>
+      <c r="P25" s="202" t="s">
         <v>78</v>
       </c>
-      <c r="Q25" s="186"/>
-      <c r="R25" s="186"/>
-      <c r="S25" s="186" t="s">
+      <c r="Q25" s="202"/>
+      <c r="R25" s="202"/>
+      <c r="S25" s="202" t="s">
         <v>79</v>
       </c>
-      <c r="T25" s="186"/>
-      <c r="U25" s="153"/>
+      <c r="T25" s="202"/>
+      <c r="U25" s="267"/>
     </row>
     <row r="26" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="178" t="s">
+      <c r="A26" s="245" t="s">
         <v>76</v>
       </c>
-      <c r="B26" s="255"/>
-      <c r="C26" s="172"/>
-      <c r="D26" s="167">
+      <c r="B26" s="153"/>
+      <c r="C26" s="239"/>
+      <c r="D26" s="234">
         <f>B26+C26</f>
         <v>0</v>
       </c>
-      <c r="E26" s="181"/>
-      <c r="F26" s="154"/>
-      <c r="G26" s="154"/>
-      <c r="H26" s="154"/>
-      <c r="I26" s="154"/>
-      <c r="J26" s="154"/>
-      <c r="K26" s="154"/>
-      <c r="L26" s="154"/>
-      <c r="M26" s="190" t="s">
+      <c r="E26" s="248"/>
+      <c r="F26" s="219"/>
+      <c r="G26" s="219"/>
+      <c r="H26" s="219"/>
+      <c r="I26" s="219"/>
+      <c r="J26" s="219"/>
+      <c r="K26" s="219"/>
+      <c r="L26" s="219"/>
+      <c r="M26" s="226" t="s">
         <v>40</v>
       </c>
-      <c r="N26" s="191"/>
+      <c r="N26" s="227"/>
       <c r="O26" s="54"/>
-      <c r="P26" s="190" t="s">
+      <c r="P26" s="226" t="s">
         <v>40</v>
       </c>
-      <c r="Q26" s="191"/>
+      <c r="Q26" s="227"/>
       <c r="R26" s="54"/>
-      <c r="S26" s="188">
+      <c r="S26" s="231">
         <f>M40+M41+M42+N40+N41+N42+O40+O41</f>
         <v>0</v>
       </c>
-      <c r="T26" s="188"/>
-      <c r="U26" s="156">
+      <c r="T26" s="231"/>
+      <c r="U26" s="268">
         <f>E26+F26+G26+H26+I26+J26+K26+L26+O26+O27+O28+R26+R27+R28+S26</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="179"/>
-      <c r="B27" s="256"/>
-      <c r="C27" s="173"/>
-      <c r="D27" s="168"/>
-      <c r="E27" s="182"/>
-      <c r="F27" s="155"/>
-      <c r="G27" s="155"/>
-      <c r="H27" s="155"/>
-      <c r="I27" s="155"/>
-      <c r="J27" s="155"/>
-      <c r="K27" s="155"/>
-      <c r="L27" s="155"/>
-      <c r="M27" s="159" t="s">
+      <c r="A27" s="246"/>
+      <c r="B27" s="154"/>
+      <c r="C27" s="240"/>
+      <c r="D27" s="235"/>
+      <c r="E27" s="249"/>
+      <c r="F27" s="203"/>
+      <c r="G27" s="203"/>
+      <c r="H27" s="203"/>
+      <c r="I27" s="203"/>
+      <c r="J27" s="203"/>
+      <c r="K27" s="203"/>
+      <c r="L27" s="203"/>
+      <c r="M27" s="199" t="s">
         <v>13</v>
       </c>
-      <c r="N27" s="160"/>
+      <c r="N27" s="200"/>
       <c r="O27" s="49"/>
-      <c r="P27" s="159" t="s">
+      <c r="P27" s="199" t="s">
         <v>13</v>
       </c>
-      <c r="Q27" s="160"/>
+      <c r="Q27" s="200"/>
       <c r="R27" s="49"/>
-      <c r="S27" s="189"/>
-      <c r="T27" s="189"/>
-      <c r="U27" s="157"/>
+      <c r="S27" s="223"/>
+      <c r="T27" s="223"/>
+      <c r="U27" s="269"/>
     </row>
     <row r="28" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="179"/>
-      <c r="B28" s="257"/>
-      <c r="C28" s="174"/>
-      <c r="D28" s="169"/>
-      <c r="E28" s="182"/>
-      <c r="F28" s="155"/>
-      <c r="G28" s="155"/>
-      <c r="H28" s="155"/>
-      <c r="I28" s="155"/>
-      <c r="J28" s="155"/>
-      <c r="K28" s="155"/>
-      <c r="L28" s="155"/>
-      <c r="M28" s="159" t="s">
+      <c r="A28" s="246"/>
+      <c r="B28" s="155"/>
+      <c r="C28" s="241"/>
+      <c r="D28" s="236"/>
+      <c r="E28" s="249"/>
+      <c r="F28" s="203"/>
+      <c r="G28" s="203"/>
+      <c r="H28" s="203"/>
+      <c r="I28" s="203"/>
+      <c r="J28" s="203"/>
+      <c r="K28" s="203"/>
+      <c r="L28" s="203"/>
+      <c r="M28" s="199" t="s">
         <v>49</v>
       </c>
-      <c r="N28" s="160"/>
+      <c r="N28" s="200"/>
       <c r="O28" s="49"/>
-      <c r="P28" s="159" t="s">
+      <c r="P28" s="199" t="s">
         <v>49</v>
       </c>
-      <c r="Q28" s="160"/>
+      <c r="Q28" s="200"/>
       <c r="R28" s="49"/>
-      <c r="S28" s="189"/>
-      <c r="T28" s="189"/>
-      <c r="U28" s="157"/>
+      <c r="S28" s="223"/>
+      <c r="T28" s="223"/>
+      <c r="U28" s="269"/>
     </row>
     <row r="29" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="179" t="s">
+      <c r="A29" s="246" t="s">
         <v>4</v>
       </c>
-      <c r="B29" s="258"/>
-      <c r="C29" s="175"/>
-      <c r="D29" s="170">
+      <c r="B29" s="156"/>
+      <c r="C29" s="242"/>
+      <c r="D29" s="237">
         <f>B29+C29</f>
         <v>0</v>
       </c>
-      <c r="E29" s="182"/>
-      <c r="F29" s="155"/>
-      <c r="G29" s="155"/>
-      <c r="H29" s="155"/>
-      <c r="I29" s="155"/>
-      <c r="J29" s="155"/>
-      <c r="K29" s="155"/>
-      <c r="L29" s="155"/>
-      <c r="M29" s="159" t="s">
+      <c r="E29" s="249"/>
+      <c r="F29" s="203"/>
+      <c r="G29" s="203"/>
+      <c r="H29" s="203"/>
+      <c r="I29" s="203"/>
+      <c r="J29" s="203"/>
+      <c r="K29" s="203"/>
+      <c r="L29" s="203"/>
+      <c r="M29" s="199" t="s">
         <v>40</v>
       </c>
-      <c r="N29" s="160"/>
+      <c r="N29" s="200"/>
       <c r="O29" s="49"/>
-      <c r="P29" s="159" t="s">
+      <c r="P29" s="199" t="s">
         <v>40</v>
       </c>
-      <c r="Q29" s="160"/>
+      <c r="Q29" s="200"/>
       <c r="R29" s="49"/>
-      <c r="S29" s="189">
+      <c r="S29" s="223">
         <f>P40+P41+P42+Q40+Q41+Q42+R40+R41</f>
         <v>0</v>
       </c>
-      <c r="T29" s="189"/>
-      <c r="U29" s="157">
+      <c r="T29" s="223"/>
+      <c r="U29" s="269">
         <f>E29+F29+G29+H29+I29+J29+K29+L29+O29+O30+O31+R29+R30+R31+S29</f>
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="179"/>
-      <c r="B30" s="256"/>
-      <c r="C30" s="173"/>
-      <c r="D30" s="168"/>
-      <c r="E30" s="182"/>
-      <c r="F30" s="155"/>
-      <c r="G30" s="155"/>
-      <c r="H30" s="155"/>
-      <c r="I30" s="155"/>
-      <c r="J30" s="155"/>
-      <c r="K30" s="155"/>
-      <c r="L30" s="155"/>
-      <c r="M30" s="159" t="s">
+      <c r="A30" s="246"/>
+      <c r="B30" s="154"/>
+      <c r="C30" s="240"/>
+      <c r="D30" s="235"/>
+      <c r="E30" s="249"/>
+      <c r="F30" s="203"/>
+      <c r="G30" s="203"/>
+      <c r="H30" s="203"/>
+      <c r="I30" s="203"/>
+      <c r="J30" s="203"/>
+      <c r="K30" s="203"/>
+      <c r="L30" s="203"/>
+      <c r="M30" s="199" t="s">
         <v>13</v>
       </c>
-      <c r="N30" s="160"/>
+      <c r="N30" s="200"/>
       <c r="O30" s="49"/>
-      <c r="P30" s="159" t="s">
+      <c r="P30" s="199" t="s">
         <v>13</v>
       </c>
-      <c r="Q30" s="160"/>
+      <c r="Q30" s="200"/>
       <c r="R30" s="49"/>
-      <c r="S30" s="189"/>
-      <c r="T30" s="189"/>
-      <c r="U30" s="157"/>
+      <c r="S30" s="223"/>
+      <c r="T30" s="223"/>
+      <c r="U30" s="269"/>
     </row>
     <row r="31" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="179"/>
-      <c r="B31" s="257"/>
-      <c r="C31" s="174"/>
-      <c r="D31" s="169"/>
-      <c r="E31" s="182"/>
-      <c r="F31" s="155"/>
-      <c r="G31" s="155"/>
-      <c r="H31" s="155"/>
-      <c r="I31" s="155"/>
-      <c r="J31" s="155"/>
-      <c r="K31" s="155"/>
-      <c r="L31" s="155"/>
-      <c r="M31" s="159" t="s">
+      <c r="A31" s="246"/>
+      <c r="B31" s="155"/>
+      <c r="C31" s="241"/>
+      <c r="D31" s="236"/>
+      <c r="E31" s="249"/>
+      <c r="F31" s="203"/>
+      <c r="G31" s="203"/>
+      <c r="H31" s="203"/>
+      <c r="I31" s="203"/>
+      <c r="J31" s="203"/>
+      <c r="K31" s="203"/>
+      <c r="L31" s="203"/>
+      <c r="M31" s="199" t="s">
         <v>49</v>
       </c>
-      <c r="N31" s="160"/>
+      <c r="N31" s="200"/>
       <c r="O31" s="49"/>
-      <c r="P31" s="159" t="s">
+      <c r="P31" s="199" t="s">
         <v>49</v>
       </c>
-      <c r="Q31" s="160"/>
+      <c r="Q31" s="200"/>
       <c r="R31" s="49"/>
-      <c r="S31" s="189"/>
-      <c r="T31" s="189"/>
-      <c r="U31" s="157"/>
+      <c r="S31" s="223"/>
+      <c r="T31" s="223"/>
+      <c r="U31" s="269"/>
     </row>
     <row r="32" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="179" t="s">
+      <c r="A32" s="246" t="s">
         <v>5</v>
       </c>
-      <c r="B32" s="258"/>
-      <c r="C32" s="175"/>
-      <c r="D32" s="170">
+      <c r="B32" s="156"/>
+      <c r="C32" s="242"/>
+      <c r="D32" s="237">
         <f>B32+C32</f>
         <v>0</v>
       </c>
-      <c r="E32" s="182"/>
-      <c r="F32" s="155"/>
-      <c r="G32" s="155"/>
-      <c r="H32" s="155"/>
-      <c r="I32" s="155"/>
-      <c r="J32" s="155"/>
-      <c r="K32" s="155"/>
-      <c r="L32" s="155"/>
-      <c r="M32" s="159" t="s">
+      <c r="E32" s="249"/>
+      <c r="F32" s="203"/>
+      <c r="G32" s="203"/>
+      <c r="H32" s="203"/>
+      <c r="I32" s="203"/>
+      <c r="J32" s="203"/>
+      <c r="K32" s="203"/>
+      <c r="L32" s="203"/>
+      <c r="M32" s="199" t="s">
         <v>40</v>
       </c>
-      <c r="N32" s="160"/>
+      <c r="N32" s="200"/>
       <c r="O32" s="49"/>
-      <c r="P32" s="159" t="s">
+      <c r="P32" s="199" t="s">
         <v>40</v>
       </c>
-      <c r="Q32" s="160"/>
+      <c r="Q32" s="200"/>
       <c r="R32" s="49"/>
-      <c r="S32" s="189">
+      <c r="S32" s="223">
         <f>S40+S41+S42+T40+T41+T42+U40+U41</f>
         <v>0</v>
       </c>
-      <c r="T32" s="189"/>
-      <c r="U32" s="157">
+      <c r="T32" s="223"/>
+      <c r="U32" s="269">
         <f>E32+F32+G32+H32+I32+J32+K32+L32+O32+O33+O34+R32+R33+R34+S32</f>
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:24" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="179"/>
-      <c r="B33" s="256"/>
-      <c r="C33" s="173"/>
-      <c r="D33" s="168"/>
-      <c r="E33" s="182"/>
-      <c r="F33" s="155"/>
-      <c r="G33" s="155"/>
-      <c r="H33" s="155"/>
-      <c r="I33" s="155"/>
-      <c r="J33" s="155"/>
-      <c r="K33" s="155"/>
-      <c r="L33" s="155"/>
-      <c r="M33" s="159" t="s">
+      <c r="A33" s="246"/>
+      <c r="B33" s="154"/>
+      <c r="C33" s="240"/>
+      <c r="D33" s="235"/>
+      <c r="E33" s="249"/>
+      <c r="F33" s="203"/>
+      <c r="G33" s="203"/>
+      <c r="H33" s="203"/>
+      <c r="I33" s="203"/>
+      <c r="J33" s="203"/>
+      <c r="K33" s="203"/>
+      <c r="L33" s="203"/>
+      <c r="M33" s="199" t="s">
         <v>13</v>
       </c>
-      <c r="N33" s="160"/>
+      <c r="N33" s="200"/>
       <c r="O33" s="49"/>
-      <c r="P33" s="159" t="s">
+      <c r="P33" s="199" t="s">
         <v>13</v>
       </c>
-      <c r="Q33" s="160"/>
+      <c r="Q33" s="200"/>
       <c r="R33" s="49"/>
-      <c r="S33" s="189"/>
-      <c r="T33" s="189"/>
-      <c r="U33" s="157"/>
+      <c r="S33" s="223"/>
+      <c r="T33" s="223"/>
+      <c r="U33" s="269"/>
     </row>
     <row r="34" spans="1:24" ht="13.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="180"/>
-      <c r="B34" s="259"/>
-      <c r="C34" s="176"/>
-      <c r="D34" s="171"/>
-      <c r="E34" s="183"/>
-      <c r="F34" s="184"/>
-      <c r="G34" s="184"/>
-      <c r="H34" s="184"/>
-      <c r="I34" s="184"/>
-      <c r="J34" s="184"/>
-      <c r="K34" s="184"/>
-      <c r="L34" s="184"/>
-      <c r="M34" s="161" t="s">
+      <c r="A34" s="247"/>
+      <c r="B34" s="157"/>
+      <c r="C34" s="243"/>
+      <c r="D34" s="238"/>
+      <c r="E34" s="250"/>
+      <c r="F34" s="204"/>
+      <c r="G34" s="204"/>
+      <c r="H34" s="204"/>
+      <c r="I34" s="204"/>
+      <c r="J34" s="204"/>
+      <c r="K34" s="204"/>
+      <c r="L34" s="204"/>
+      <c r="M34" s="228" t="s">
         <v>49</v>
       </c>
-      <c r="N34" s="162"/>
+      <c r="N34" s="229"/>
       <c r="O34" s="50"/>
-      <c r="P34" s="161" t="s">
+      <c r="P34" s="228" t="s">
         <v>49</v>
       </c>
-      <c r="Q34" s="162"/>
+      <c r="Q34" s="229"/>
       <c r="R34" s="50"/>
-      <c r="S34" s="214"/>
-      <c r="T34" s="214"/>
-      <c r="U34" s="158"/>
+      <c r="S34" s="224"/>
+      <c r="T34" s="224"/>
+      <c r="U34" s="270"/>
     </row>
     <row r="35" spans="1:24" ht="4.6500000000000004" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="36" spans="1:24" ht="13.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -10036,30 +10033,30 @@
       <c r="D36" s="2"/>
     </row>
     <row r="37" spans="1:24" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="220" t="s">
+      <c r="A37" s="178" t="s">
         <v>45</v>
       </c>
-      <c r="B37" s="221"/>
-      <c r="C37" s="221"/>
-      <c r="D37" s="221"/>
-      <c r="E37" s="222"/>
+      <c r="B37" s="179"/>
+      <c r="C37" s="179"/>
+      <c r="D37" s="179"/>
+      <c r="E37" s="180"/>
       <c r="F37" s="18"/>
       <c r="G37" s="18"/>
       <c r="H37" s="18"/>
-      <c r="J37" s="199" t="s">
+      <c r="J37" s="207" t="s">
         <v>50</v>
       </c>
-      <c r="K37" s="200"/>
-      <c r="L37" s="200"/>
-      <c r="M37" s="200"/>
-      <c r="N37" s="200"/>
-      <c r="O37" s="200"/>
-      <c r="P37" s="200"/>
-      <c r="Q37" s="200"/>
-      <c r="R37" s="200"/>
-      <c r="S37" s="200"/>
-      <c r="T37" s="200"/>
-      <c r="U37" s="201"/>
+      <c r="K37" s="208"/>
+      <c r="L37" s="208"/>
+      <c r="M37" s="208"/>
+      <c r="N37" s="208"/>
+      <c r="O37" s="208"/>
+      <c r="P37" s="208"/>
+      <c r="Q37" s="208"/>
+      <c r="R37" s="208"/>
+      <c r="S37" s="208"/>
+      <c r="T37" s="208"/>
+      <c r="U37" s="209"/>
     </row>
     <row r="38" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="14"/>
@@ -10075,44 +10072,44 @@
       <c r="E38" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="J38" s="202" t="s">
+      <c r="J38" s="210" t="s">
         <v>2</v>
       </c>
-      <c r="K38" s="203"/>
-      <c r="L38" s="204"/>
-      <c r="M38" s="197" t="s">
+      <c r="K38" s="211"/>
+      <c r="L38" s="212"/>
+      <c r="M38" s="205" t="s">
         <v>6</v>
       </c>
-      <c r="N38" s="197"/>
-      <c r="O38" s="197"/>
-      <c r="P38" s="197" t="s">
+      <c r="N38" s="205"/>
+      <c r="O38" s="205"/>
+      <c r="P38" s="205" t="s">
         <v>4</v>
       </c>
-      <c r="Q38" s="197"/>
-      <c r="R38" s="197"/>
-      <c r="S38" s="197" t="s">
+      <c r="Q38" s="205"/>
+      <c r="R38" s="205"/>
+      <c r="S38" s="205" t="s">
         <v>5</v>
       </c>
-      <c r="T38" s="197"/>
-      <c r="U38" s="198"/>
+      <c r="T38" s="205"/>
+      <c r="U38" s="206"/>
     </row>
     <row r="39" spans="1:24" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="242" t="s">
+      <c r="A39" s="169" t="s">
         <v>42</v>
       </c>
-      <c r="B39" s="192"/>
-      <c r="C39" s="192"/>
-      <c r="D39" s="192"/>
-      <c r="E39" s="194">
+      <c r="B39" s="172"/>
+      <c r="C39" s="172"/>
+      <c r="D39" s="172"/>
+      <c r="E39" s="171">
         <f>B39+C39+D39</f>
         <v>0</v>
       </c>
-      <c r="F39" s="196"/>
-      <c r="G39" s="196"/>
-      <c r="H39" s="241"/>
-      <c r="J39" s="205"/>
-      <c r="K39" s="206"/>
-      <c r="L39" s="207"/>
+      <c r="F39" s="168"/>
+      <c r="G39" s="168"/>
+      <c r="H39" s="167"/>
+      <c r="J39" s="213"/>
+      <c r="K39" s="214"/>
+      <c r="L39" s="215"/>
       <c r="M39" s="44" t="s">
         <v>51</v>
       </c>
@@ -10142,19 +10139,19 @@
       </c>
     </row>
     <row r="40" spans="1:24" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="242"/>
-      <c r="B40" s="216"/>
-      <c r="C40" s="216"/>
-      <c r="D40" s="216"/>
-      <c r="E40" s="194"/>
-      <c r="F40" s="196"/>
-      <c r="G40" s="196"/>
-      <c r="H40" s="241"/>
-      <c r="J40" s="208" t="s">
+      <c r="A40" s="169"/>
+      <c r="B40" s="174"/>
+      <c r="C40" s="174"/>
+      <c r="D40" s="174"/>
+      <c r="E40" s="171"/>
+      <c r="F40" s="168"/>
+      <c r="G40" s="168"/>
+      <c r="H40" s="167"/>
+      <c r="J40" s="216" t="s">
         <v>53</v>
       </c>
-      <c r="K40" s="209"/>
-      <c r="L40" s="210"/>
+      <c r="K40" s="217"/>
+      <c r="L40" s="218"/>
       <c r="M40" s="38"/>
       <c r="N40" s="38"/>
       <c r="O40" s="38"/>
@@ -10166,24 +10163,24 @@
       <c r="U40" s="39"/>
     </row>
     <row r="41" spans="1:24" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="242" t="s">
+      <c r="A41" s="169" t="s">
         <v>43</v>
       </c>
-      <c r="B41" s="192"/>
-      <c r="C41" s="192"/>
-      <c r="D41" s="192"/>
-      <c r="E41" s="194">
+      <c r="B41" s="172"/>
+      <c r="C41" s="172"/>
+      <c r="D41" s="172"/>
+      <c r="E41" s="171">
         <f>B41+C41+D41</f>
         <v>0</v>
       </c>
-      <c r="F41" s="196"/>
-      <c r="G41" s="196"/>
-      <c r="H41" s="241"/>
-      <c r="J41" s="208" t="s">
+      <c r="F41" s="168"/>
+      <c r="G41" s="168"/>
+      <c r="H41" s="167"/>
+      <c r="J41" s="216" t="s">
         <v>54</v>
       </c>
-      <c r="K41" s="209"/>
-      <c r="L41" s="210"/>
+      <c r="K41" s="217"/>
+      <c r="L41" s="218"/>
       <c r="M41" s="38"/>
       <c r="N41" s="38"/>
       <c r="O41" s="38"/>
@@ -10195,19 +10192,19 @@
       <c r="U41" s="39"/>
     </row>
     <row r="42" spans="1:24" ht="13.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="242"/>
-      <c r="B42" s="216"/>
-      <c r="C42" s="216"/>
-      <c r="D42" s="216"/>
-      <c r="E42" s="194"/>
-      <c r="F42" s="196"/>
-      <c r="G42" s="196"/>
-      <c r="H42" s="241"/>
-      <c r="J42" s="211" t="s">
+      <c r="A42" s="169"/>
+      <c r="B42" s="174"/>
+      <c r="C42" s="174"/>
+      <c r="D42" s="174"/>
+      <c r="E42" s="171"/>
+      <c r="F42" s="168"/>
+      <c r="G42" s="168"/>
+      <c r="H42" s="167"/>
+      <c r="J42" s="220" t="s">
         <v>55</v>
       </c>
-      <c r="K42" s="212"/>
-      <c r="L42" s="213"/>
+      <c r="K42" s="221"/>
+      <c r="L42" s="222"/>
       <c r="M42" s="40"/>
       <c r="N42" s="40"/>
       <c r="O42" s="41"/>
@@ -10219,19 +10216,19 @@
       <c r="U42" s="42"/>
     </row>
     <row r="43" spans="1:24" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="242" t="s">
+      <c r="A43" s="169" t="s">
         <v>44</v>
       </c>
-      <c r="B43" s="192"/>
-      <c r="C43" s="192"/>
-      <c r="D43" s="192"/>
-      <c r="E43" s="194">
+      <c r="B43" s="172"/>
+      <c r="C43" s="172"/>
+      <c r="D43" s="172"/>
+      <c r="E43" s="171">
         <f>B43+C43+D43</f>
         <v>0</v>
       </c>
-      <c r="F43" s="196"/>
-      <c r="G43" s="196"/>
-      <c r="H43" s="241"/>
+      <c r="F43" s="168"/>
+      <c r="G43" s="168"/>
+      <c r="H43" s="167"/>
       <c r="J43" s="15" t="s">
         <v>56</v>
       </c>
@@ -10251,25 +10248,25 @@
       <c r="X43" s="16"/>
     </row>
     <row r="44" spans="1:24" ht="13.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="269"/>
-      <c r="B44" s="193"/>
-      <c r="C44" s="193"/>
-      <c r="D44" s="193"/>
-      <c r="E44" s="195"/>
-      <c r="F44" s="196"/>
-      <c r="G44" s="196"/>
-      <c r="H44" s="241"/>
+      <c r="A44" s="170"/>
+      <c r="B44" s="173"/>
+      <c r="C44" s="173"/>
+      <c r="D44" s="173"/>
+      <c r="E44" s="225"/>
+      <c r="F44" s="168"/>
+      <c r="G44" s="168"/>
+      <c r="H44" s="167"/>
     </row>
     <row r="45" spans="1:24" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
-      <c r="F45" s="252" t="s">
+      <c r="F45" s="150" t="s">
         <v>115</v>
       </c>
-      <c r="G45" s="252"/>
-      <c r="H45" s="252"/>
+      <c r="G45" s="150"/>
+      <c r="H45" s="150"/>
       <c r="L45" s="16" t="s">
         <v>57</v>
       </c>
@@ -10277,97 +10274,213 @@
       <c r="N45" s="16"/>
       <c r="O45" s="16"/>
       <c r="P45" s="16"/>
-      <c r="Q45" s="146"/>
-      <c r="R45" s="146"/>
-      <c r="S45" s="146"/>
-      <c r="T45" s="146"/>
-      <c r="U45" s="146"/>
+      <c r="Q45" s="260"/>
+      <c r="R45" s="260"/>
+      <c r="S45" s="260"/>
+      <c r="T45" s="260"/>
+      <c r="U45" s="260"/>
     </row>
     <row r="46" spans="1:24" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="265"/>
+      <c r="A46" s="163"/>
       <c r="B46" s="48"/>
       <c r="C46" s="48"/>
       <c r="D46" s="48"/>
-      <c r="E46" s="243"/>
-      <c r="F46" s="244"/>
-      <c r="G46" s="244"/>
-      <c r="H46" s="244"/>
-      <c r="I46" s="244"/>
-      <c r="J46" s="245"/>
+      <c r="E46" s="141"/>
+      <c r="F46" s="142"/>
+      <c r="G46" s="142"/>
+      <c r="H46" s="142"/>
+      <c r="I46" s="142"/>
+      <c r="J46" s="143"/>
       <c r="K46" s="16"/>
       <c r="L46" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M46" s="146"/>
-      <c r="N46" s="146"/>
-      <c r="O46" s="146"/>
-      <c r="P46" s="146"/>
+      <c r="M46" s="260"/>
+      <c r="N46" s="260"/>
+      <c r="O46" s="260"/>
+      <c r="P46" s="260"/>
       <c r="Q46" s="16"/>
       <c r="R46" s="16"/>
     </row>
     <row r="47" spans="1:24" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="265"/>
+      <c r="A47" s="163"/>
       <c r="B47" s="48"/>
       <c r="C47" s="48"/>
       <c r="D47" s="48"/>
-      <c r="E47" s="246"/>
-      <c r="F47" s="247"/>
-      <c r="G47" s="247"/>
-      <c r="H47" s="247"/>
-      <c r="I47" s="247"/>
-      <c r="J47" s="248"/>
+      <c r="E47" s="144"/>
+      <c r="F47" s="145"/>
+      <c r="G47" s="145"/>
+      <c r="H47" s="145"/>
+      <c r="I47" s="145"/>
+      <c r="J47" s="146"/>
       <c r="K47" s="16"/>
       <c r="L47" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="M47" s="145"/>
-      <c r="N47" s="145"/>
-      <c r="O47" s="145"/>
-      <c r="P47" s="145"/>
+      <c r="M47" s="259"/>
+      <c r="N47" s="259"/>
+      <c r="O47" s="259"/>
+      <c r="P47" s="259"/>
       <c r="Q47" s="16"/>
       <c r="R47" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="S47" s="144"/>
-      <c r="T47" s="144"/>
+      <c r="S47" s="258"/>
+      <c r="T47" s="258"/>
     </row>
     <row r="48" spans="1:24" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="241"/>
+      <c r="A48" s="167"/>
       <c r="B48" s="47"/>
       <c r="C48" s="47"/>
       <c r="D48" s="47"/>
-      <c r="E48" s="246"/>
-      <c r="F48" s="247"/>
-      <c r="G48" s="247"/>
-      <c r="H48" s="247"/>
-      <c r="I48" s="247"/>
-      <c r="J48" s="248"/>
+      <c r="E48" s="144"/>
+      <c r="F48" s="145"/>
+      <c r="G48" s="145"/>
+      <c r="H48" s="145"/>
+      <c r="I48" s="145"/>
+      <c r="J48" s="146"/>
       <c r="K48" s="16"/>
       <c r="L48" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="M48" s="166"/>
-      <c r="N48" s="166"/>
-      <c r="O48" s="166"/>
-      <c r="P48" s="166"/>
+      <c r="M48" s="233"/>
+      <c r="N48" s="233"/>
+      <c r="O48" s="233"/>
+      <c r="P48" s="233"/>
       <c r="Q48" s="16"/>
       <c r="R48" s="16"/>
     </row>
     <row r="49" spans="1:11" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="241"/>
+      <c r="A49" s="167"/>
       <c r="B49" s="47"/>
       <c r="C49" s="47"/>
       <c r="D49" s="47"/>
-      <c r="E49" s="249"/>
-      <c r="F49" s="250"/>
-      <c r="G49" s="250"/>
-      <c r="H49" s="250"/>
-      <c r="I49" s="250"/>
-      <c r="J49" s="251"/>
+      <c r="E49" s="147"/>
+      <c r="F49" s="148"/>
+      <c r="G49" s="148"/>
+      <c r="H49" s="148"/>
+      <c r="I49" s="148"/>
+      <c r="J49" s="149"/>
       <c r="K49" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="140">
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="S47:T47"/>
+    <mergeCell ref="M47:P47"/>
+    <mergeCell ref="M46:P46"/>
+    <mergeCell ref="Q45:U45"/>
+    <mergeCell ref="N7:S7"/>
+    <mergeCell ref="M8:S8"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="Q10:S10"/>
+    <mergeCell ref="U23:U25"/>
+    <mergeCell ref="I26:I28"/>
+    <mergeCell ref="U26:U28"/>
+    <mergeCell ref="U29:U31"/>
+    <mergeCell ref="U32:U34"/>
+    <mergeCell ref="L26:L28"/>
+    <mergeCell ref="L29:L31"/>
+    <mergeCell ref="M33:N33"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="E23:T23"/>
+    <mergeCell ref="K26:K28"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="M48:P48"/>
+    <mergeCell ref="D26:D28"/>
+    <mergeCell ref="D29:D31"/>
+    <mergeCell ref="D32:D34"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="C29:C31"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="A4:U4"/>
+    <mergeCell ref="A2:U2"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="A29:A31"/>
+    <mergeCell ref="A32:A34"/>
+    <mergeCell ref="E26:E28"/>
+    <mergeCell ref="E29:E31"/>
+    <mergeCell ref="E32:E34"/>
+    <mergeCell ref="F26:F28"/>
+    <mergeCell ref="G32:G34"/>
+    <mergeCell ref="J29:J31"/>
+    <mergeCell ref="K29:K31"/>
+    <mergeCell ref="J12:L12"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="P24:R24"/>
+    <mergeCell ref="S25:T25"/>
+    <mergeCell ref="P34:Q34"/>
+    <mergeCell ref="P30:Q30"/>
+    <mergeCell ref="P31:Q31"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="S24:T24"/>
+    <mergeCell ref="S26:T28"/>
+    <mergeCell ref="M26:N26"/>
+    <mergeCell ref="P28:Q28"/>
+    <mergeCell ref="P29:Q29"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="D43:D44"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="F29:F31"/>
+    <mergeCell ref="P26:Q26"/>
+    <mergeCell ref="P33:Q33"/>
+    <mergeCell ref="K32:K34"/>
+    <mergeCell ref="F32:F34"/>
+    <mergeCell ref="G29:G31"/>
+    <mergeCell ref="S38:U38"/>
+    <mergeCell ref="J37:U37"/>
+    <mergeCell ref="J38:L39"/>
+    <mergeCell ref="J40:L40"/>
+    <mergeCell ref="J41:L41"/>
+    <mergeCell ref="J32:J34"/>
+    <mergeCell ref="G26:G28"/>
+    <mergeCell ref="J26:J28"/>
+    <mergeCell ref="J42:L42"/>
+    <mergeCell ref="M38:O38"/>
+    <mergeCell ref="P38:R38"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="I29:I31"/>
+    <mergeCell ref="I32:I34"/>
+    <mergeCell ref="M27:N27"/>
+    <mergeCell ref="P32:Q32"/>
+    <mergeCell ref="H26:H28"/>
+    <mergeCell ref="H29:H31"/>
+    <mergeCell ref="S29:T31"/>
+    <mergeCell ref="S32:T34"/>
+    <mergeCell ref="N6:O6"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="D39:D40"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="D41:D42"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="D13:G13"/>
+    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="H17:K18"/>
+    <mergeCell ref="L17:N17"/>
+    <mergeCell ref="O17:Q17"/>
+    <mergeCell ref="A12:C14"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="P27:Q27"/>
+    <mergeCell ref="M24:O24"/>
+    <mergeCell ref="M25:O25"/>
+    <mergeCell ref="P25:R25"/>
+    <mergeCell ref="L32:L34"/>
+    <mergeCell ref="H39:H40"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="A41:A42"/>
     <mergeCell ref="E46:J49"/>
     <mergeCell ref="F45:H45"/>
     <mergeCell ref="A17:C17"/>
@@ -10392,125 +10505,9 @@
     <mergeCell ref="G41:G42"/>
     <mergeCell ref="H41:H42"/>
     <mergeCell ref="B43:B44"/>
-    <mergeCell ref="N6:O6"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="D39:D40"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="D41:D42"/>
-    <mergeCell ref="D12:G12"/>
-    <mergeCell ref="D13:G13"/>
-    <mergeCell ref="D14:G14"/>
-    <mergeCell ref="A37:E37"/>
-    <mergeCell ref="H17:K18"/>
-    <mergeCell ref="L17:N17"/>
-    <mergeCell ref="O17:Q17"/>
-    <mergeCell ref="A12:C14"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="P27:Q27"/>
-    <mergeCell ref="M24:O24"/>
-    <mergeCell ref="M25:O25"/>
-    <mergeCell ref="P25:R25"/>
-    <mergeCell ref="L32:L34"/>
-    <mergeCell ref="H39:H40"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="S38:U38"/>
-    <mergeCell ref="J37:U37"/>
-    <mergeCell ref="J38:L39"/>
-    <mergeCell ref="J40:L40"/>
-    <mergeCell ref="J41:L41"/>
-    <mergeCell ref="J32:J34"/>
-    <mergeCell ref="G26:G28"/>
-    <mergeCell ref="J26:J28"/>
-    <mergeCell ref="J42:L42"/>
-    <mergeCell ref="M38:O38"/>
-    <mergeCell ref="P38:R38"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="I29:I31"/>
-    <mergeCell ref="I32:I34"/>
-    <mergeCell ref="M27:N27"/>
-    <mergeCell ref="P32:Q32"/>
-    <mergeCell ref="H26:H28"/>
-    <mergeCell ref="H29:H31"/>
-    <mergeCell ref="S29:T31"/>
-    <mergeCell ref="S32:T34"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="D43:D44"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="H32:H34"/>
-    <mergeCell ref="F29:F31"/>
-    <mergeCell ref="P26:Q26"/>
-    <mergeCell ref="P33:Q33"/>
-    <mergeCell ref="K32:K34"/>
-    <mergeCell ref="F32:F34"/>
-    <mergeCell ref="G29:G31"/>
-    <mergeCell ref="P24:R24"/>
-    <mergeCell ref="S25:T25"/>
-    <mergeCell ref="P34:Q34"/>
-    <mergeCell ref="P30:Q30"/>
-    <mergeCell ref="P31:Q31"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="S24:T24"/>
-    <mergeCell ref="S26:T28"/>
-    <mergeCell ref="M26:N26"/>
-    <mergeCell ref="P28:Q28"/>
-    <mergeCell ref="P29:Q29"/>
-    <mergeCell ref="A1:R1"/>
-    <mergeCell ref="M48:P48"/>
-    <mergeCell ref="D26:D28"/>
-    <mergeCell ref="D29:D31"/>
-    <mergeCell ref="D32:D34"/>
-    <mergeCell ref="C26:C28"/>
-    <mergeCell ref="C29:C31"/>
-    <mergeCell ref="C32:C34"/>
-    <mergeCell ref="A4:U4"/>
-    <mergeCell ref="A2:U2"/>
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="A29:A31"/>
-    <mergeCell ref="A32:A34"/>
-    <mergeCell ref="E26:E28"/>
-    <mergeCell ref="E29:E31"/>
-    <mergeCell ref="E32:E34"/>
-    <mergeCell ref="F26:F28"/>
-    <mergeCell ref="G32:G34"/>
-    <mergeCell ref="J29:J31"/>
-    <mergeCell ref="K29:K31"/>
-    <mergeCell ref="J12:L12"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="S47:T47"/>
-    <mergeCell ref="M47:P47"/>
-    <mergeCell ref="M46:P46"/>
-    <mergeCell ref="Q45:U45"/>
-    <mergeCell ref="N7:S7"/>
-    <mergeCell ref="M8:S8"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="K10:L10"/>
-    <mergeCell ref="Q10:S10"/>
-    <mergeCell ref="U23:U25"/>
-    <mergeCell ref="I26:I28"/>
-    <mergeCell ref="U26:U28"/>
-    <mergeCell ref="U29:U31"/>
-    <mergeCell ref="U32:U34"/>
-    <mergeCell ref="L26:L28"/>
-    <mergeCell ref="L29:L31"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="M34:N34"/>
-    <mergeCell ref="E23:T23"/>
-    <mergeCell ref="K26:K28"/>
-    <mergeCell ref="M32:N32"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Date Format:_x000a_DD/MM/YYYY" sqref="S47 P9"/>
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E26:L34 M40:U42 B39:D44 L18:N18 R26:R34 O26:O34 C26:C34 B26:B28 B32:B34">
       <formula1>0</formula1>
@@ -10523,6 +10520,9 @@
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B29:B31">
       <formula1>0</formula1>
       <formula2>999999</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L6">
+      <formula1>"January, February, March, April, May, June, July, August, September, October, November, December"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.21" right="0.17" top="0.47" bottom="0.22" header="0.23" footer="0.16"/>
@@ -11439,23 +11439,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:42" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="271" t="s">
+      <c r="A1" s="274" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="271"/>
-      <c r="C1" s="271"/>
-      <c r="D1" s="271"/>
-      <c r="E1" s="271"/>
-      <c r="F1" s="271"/>
-      <c r="G1" s="271"/>
-      <c r="H1" s="271"/>
-      <c r="I1" s="271"/>
-      <c r="J1" s="271"/>
-      <c r="K1" s="271"/>
-      <c r="L1" s="271"/>
-      <c r="M1" s="271"/>
-      <c r="N1" s="271"/>
-      <c r="O1" s="271"/>
+      <c r="B1" s="274"/>
+      <c r="C1" s="274"/>
+      <c r="D1" s="274"/>
+      <c r="E1" s="274"/>
+      <c r="F1" s="274"/>
+      <c r="G1" s="274"/>
+      <c r="H1" s="274"/>
+      <c r="I1" s="274"/>
+      <c r="J1" s="274"/>
+      <c r="K1" s="274"/>
+      <c r="L1" s="274"/>
+      <c r="M1" s="274"/>
+      <c r="N1" s="274"/>
+      <c r="O1" s="274"/>
       <c r="P1" s="76"/>
       <c r="Q1" s="76"/>
       <c r="R1" s="76"/>
@@ -11485,23 +11485,23 @@
       <c r="AP1" s="76"/>
     </row>
     <row r="2" spans="1:42" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="271" t="s">
+      <c r="A2" s="274" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="271"/>
-      <c r="C2" s="271"/>
-      <c r="D2" s="271"/>
-      <c r="E2" s="271"/>
-      <c r="F2" s="271"/>
-      <c r="G2" s="271"/>
-      <c r="H2" s="271"/>
-      <c r="I2" s="271"/>
-      <c r="J2" s="271"/>
-      <c r="K2" s="271"/>
-      <c r="L2" s="271"/>
-      <c r="M2" s="271"/>
-      <c r="N2" s="271"/>
-      <c r="O2" s="271"/>
+      <c r="B2" s="274"/>
+      <c r="C2" s="274"/>
+      <c r="D2" s="274"/>
+      <c r="E2" s="274"/>
+      <c r="F2" s="274"/>
+      <c r="G2" s="274"/>
+      <c r="H2" s="274"/>
+      <c r="I2" s="274"/>
+      <c r="J2" s="274"/>
+      <c r="K2" s="274"/>
+      <c r="L2" s="274"/>
+      <c r="M2" s="274"/>
+      <c r="N2" s="274"/>
+      <c r="O2" s="274"/>
       <c r="P2" s="76"/>
       <c r="Q2" s="76"/>
       <c r="R2" s="76"/>
@@ -11531,23 +11531,23 @@
       <c r="AP2" s="76"/>
     </row>
     <row r="3" spans="1:42" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="271" t="s">
+      <c r="A3" s="274" t="s">
         <v>90</v>
       </c>
-      <c r="B3" s="271"/>
-      <c r="C3" s="271"/>
-      <c r="D3" s="271"/>
-      <c r="E3" s="271"/>
-      <c r="F3" s="271"/>
-      <c r="G3" s="271"/>
-      <c r="H3" s="271"/>
-      <c r="I3" s="271"/>
-      <c r="J3" s="271"/>
-      <c r="K3" s="271"/>
-      <c r="L3" s="271"/>
-      <c r="M3" s="271"/>
-      <c r="N3" s="271"/>
-      <c r="O3" s="271"/>
+      <c r="B3" s="274"/>
+      <c r="C3" s="274"/>
+      <c r="D3" s="274"/>
+      <c r="E3" s="274"/>
+      <c r="F3" s="274"/>
+      <c r="G3" s="274"/>
+      <c r="H3" s="274"/>
+      <c r="I3" s="274"/>
+      <c r="J3" s="274"/>
+      <c r="K3" s="274"/>
+      <c r="L3" s="274"/>
+      <c r="M3" s="274"/>
+      <c r="N3" s="274"/>
+      <c r="O3" s="274"/>
       <c r="P3" s="76"/>
       <c r="Q3" s="76"/>
       <c r="R3" s="76"/>
@@ -11577,23 +11577,23 @@
       <c r="AP3" s="76"/>
     </row>
     <row r="4" spans="1:42" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="271" t="s">
+      <c r="A4" s="274" t="s">
         <v>91</v>
       </c>
-      <c r="B4" s="271"/>
-      <c r="C4" s="271"/>
-      <c r="D4" s="271"/>
-      <c r="E4" s="271"/>
-      <c r="F4" s="271"/>
-      <c r="G4" s="271"/>
-      <c r="H4" s="271"/>
-      <c r="I4" s="271"/>
-      <c r="J4" s="271"/>
-      <c r="K4" s="271"/>
-      <c r="L4" s="271"/>
-      <c r="M4" s="271"/>
-      <c r="N4" s="271"/>
-      <c r="O4" s="271"/>
+      <c r="B4" s="274"/>
+      <c r="C4" s="274"/>
+      <c r="D4" s="274"/>
+      <c r="E4" s="274"/>
+      <c r="F4" s="274"/>
+      <c r="G4" s="274"/>
+      <c r="H4" s="274"/>
+      <c r="I4" s="274"/>
+      <c r="J4" s="274"/>
+      <c r="K4" s="274"/>
+      <c r="L4" s="274"/>
+      <c r="M4" s="274"/>
+      <c r="N4" s="274"/>
+      <c r="O4" s="274"/>
       <c r="P4" s="76"/>
       <c r="Q4" s="76"/>
       <c r="R4" s="76"/>
@@ -11623,23 +11623,23 @@
       <c r="AP4" s="76"/>
     </row>
     <row r="5" spans="1:42" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="271" t="s">
+      <c r="A5" s="274" t="s">
         <v>92</v>
       </c>
-      <c r="B5" s="271"/>
-      <c r="C5" s="271"/>
-      <c r="D5" s="271"/>
-      <c r="E5" s="271"/>
-      <c r="F5" s="271"/>
-      <c r="G5" s="271"/>
-      <c r="H5" s="271"/>
-      <c r="I5" s="271"/>
-      <c r="J5" s="271"/>
-      <c r="K5" s="271"/>
-      <c r="L5" s="271"/>
-      <c r="M5" s="271"/>
-      <c r="N5" s="271"/>
-      <c r="O5" s="271"/>
+      <c r="B5" s="274"/>
+      <c r="C5" s="274"/>
+      <c r="D5" s="274"/>
+      <c r="E5" s="274"/>
+      <c r="F5" s="274"/>
+      <c r="G5" s="274"/>
+      <c r="H5" s="274"/>
+      <c r="I5" s="274"/>
+      <c r="J5" s="274"/>
+      <c r="K5" s="274"/>
+      <c r="L5" s="274"/>
+      <c r="M5" s="274"/>
+      <c r="N5" s="274"/>
+      <c r="O5" s="274"/>
     </row>
     <row r="6" spans="1:42" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="7" spans="1:42" x14ac:dyDescent="0.3">
@@ -11651,12 +11651,12 @@
       <c r="A8" s="86" t="s">
         <v>94</v>
       </c>
-      <c r="D8" s="272" t="str">
+      <c r="D8" s="275" t="str">
         <f>IF('DR-TB 10A'!C8="","",'DR-TB 10A'!C8)</f>
         <v/>
       </c>
-      <c r="E8" s="272"/>
-      <c r="F8" s="272"/>
+      <c r="E8" s="275"/>
+      <c r="F8" s="275"/>
       <c r="G8" s="85"/>
       <c r="H8" s="79" t="s">
         <v>95</v>
@@ -12031,23 +12031,23 @@
       <c r="C29" s="80"/>
     </row>
     <row r="30" spans="1:15" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="270" t="s">
+      <c r="A30" s="273" t="s">
         <v>109</v>
       </c>
-      <c r="B30" s="270"/>
-      <c r="C30" s="270"/>
-      <c r="D30" s="270"/>
-      <c r="E30" s="270"/>
-      <c r="F30" s="270"/>
-      <c r="G30" s="270"/>
-      <c r="H30" s="270"/>
-      <c r="I30" s="270"/>
-      <c r="J30" s="270"/>
-      <c r="K30" s="270"/>
-      <c r="L30" s="270"/>
-      <c r="M30" s="270"/>
-      <c r="N30" s="270"/>
-      <c r="O30" s="270"/>
+      <c r="B30" s="273"/>
+      <c r="C30" s="273"/>
+      <c r="D30" s="273"/>
+      <c r="E30" s="273"/>
+      <c r="F30" s="273"/>
+      <c r="G30" s="273"/>
+      <c r="H30" s="273"/>
+      <c r="I30" s="273"/>
+      <c r="J30" s="273"/>
+      <c r="K30" s="273"/>
+      <c r="L30" s="273"/>
+      <c r="M30" s="273"/>
+      <c r="N30" s="273"/>
+      <c r="O30" s="273"/>
     </row>
     <row r="31" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="81" t="s">
@@ -12130,78 +12130,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" s="65" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="307" t="s">
+      <c r="A1" s="280" t="s">
         <v>136</v>
       </c>
-      <c r="B1" s="307"/>
-      <c r="C1" s="307"/>
-      <c r="D1" s="307"/>
-      <c r="E1" s="307"/>
-      <c r="F1" s="307"/>
-      <c r="G1" s="307"/>
-      <c r="H1" s="307"/>
-      <c r="I1" s="307"/>
-      <c r="J1" s="307"/>
-      <c r="K1" s="307"/>
-      <c r="L1" s="307"/>
-      <c r="M1" s="307"/>
-      <c r="N1" s="307"/>
-      <c r="O1" s="307"/>
-      <c r="P1" s="306" t="s">
+      <c r="B1" s="280"/>
+      <c r="C1" s="280"/>
+      <c r="D1" s="280"/>
+      <c r="E1" s="280"/>
+      <c r="F1" s="280"/>
+      <c r="G1" s="280"/>
+      <c r="H1" s="280"/>
+      <c r="I1" s="280"/>
+      <c r="J1" s="280"/>
+      <c r="K1" s="280"/>
+      <c r="L1" s="280"/>
+      <c r="M1" s="280"/>
+      <c r="N1" s="280"/>
+      <c r="O1" s="280"/>
+      <c r="P1" s="281" t="s">
         <v>135</v>
       </c>
-      <c r="Q1" s="306"/>
-      <c r="R1" s="306"/>
-      <c r="S1" s="306"/>
+      <c r="Q1" s="281"/>
+      <c r="R1" s="281"/>
+      <c r="S1" s="281"/>
       <c r="T1" s="130"/>
       <c r="U1" s="130"/>
     </row>
     <row r="2" spans="1:21" s="65" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A2" s="307" t="s">
+      <c r="A2" s="280" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="307"/>
-      <c r="C2" s="307"/>
-      <c r="D2" s="307"/>
-      <c r="E2" s="307"/>
-      <c r="F2" s="307"/>
-      <c r="G2" s="307"/>
-      <c r="H2" s="307"/>
-      <c r="I2" s="307"/>
-      <c r="J2" s="307"/>
-      <c r="K2" s="307"/>
-      <c r="L2" s="307"/>
-      <c r="M2" s="307"/>
-      <c r="N2" s="307"/>
-      <c r="O2" s="307"/>
-      <c r="P2" s="307"/>
-      <c r="Q2" s="307"/>
-      <c r="R2" s="307"/>
-      <c r="S2" s="307"/>
-      <c r="T2" s="307"/>
-      <c r="U2" s="307"/>
+      <c r="B2" s="280"/>
+      <c r="C2" s="280"/>
+      <c r="D2" s="280"/>
+      <c r="E2" s="280"/>
+      <c r="F2" s="280"/>
+      <c r="G2" s="280"/>
+      <c r="H2" s="280"/>
+      <c r="I2" s="280"/>
+      <c r="J2" s="280"/>
+      <c r="K2" s="280"/>
+      <c r="L2" s="280"/>
+      <c r="M2" s="280"/>
+      <c r="N2" s="280"/>
+      <c r="O2" s="280"/>
+      <c r="P2" s="280"/>
+      <c r="Q2" s="280"/>
+      <c r="R2" s="280"/>
+      <c r="S2" s="280"/>
+      <c r="T2" s="280"/>
+      <c r="U2" s="280"/>
     </row>
     <row r="3" spans="1:21" s="65" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A3" s="307" t="s">
+      <c r="A3" s="280" t="s">
         <v>118</v>
       </c>
-      <c r="B3" s="307"/>
-      <c r="C3" s="307"/>
-      <c r="D3" s="307"/>
-      <c r="E3" s="307"/>
-      <c r="F3" s="307"/>
-      <c r="G3" s="307"/>
-      <c r="H3" s="307"/>
-      <c r="I3" s="307"/>
-      <c r="J3" s="307"/>
-      <c r="K3" s="307"/>
-      <c r="L3" s="307"/>
-      <c r="M3" s="307"/>
-      <c r="N3" s="307"/>
-      <c r="O3" s="307"/>
-      <c r="P3" s="307"/>
-      <c r="Q3" s="307"/>
-      <c r="R3" s="307"/>
+      <c r="B3" s="280"/>
+      <c r="C3" s="280"/>
+      <c r="D3" s="280"/>
+      <c r="E3" s="280"/>
+      <c r="F3" s="280"/>
+      <c r="G3" s="280"/>
+      <c r="H3" s="280"/>
+      <c r="I3" s="280"/>
+      <c r="J3" s="280"/>
+      <c r="K3" s="280"/>
+      <c r="L3" s="280"/>
+      <c r="M3" s="280"/>
+      <c r="N3" s="280"/>
+      <c r="O3" s="280"/>
+      <c r="P3" s="280"/>
+      <c r="Q3" s="280"/>
+      <c r="R3" s="280"/>
       <c r="S3" s="131"/>
       <c r="T3" s="131"/>
       <c r="U3" s="131"/>
@@ -12230,29 +12230,29 @@
       <c r="U4" s="131"/>
     </row>
     <row r="5" spans="1:21" s="65" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A5" s="306" t="s">
+      <c r="A5" s="281" t="s">
         <v>119</v>
       </c>
-      <c r="B5" s="306"/>
-      <c r="C5" s="306"/>
-      <c r="D5" s="306"/>
-      <c r="E5" s="306"/>
-      <c r="F5" s="306"/>
-      <c r="G5" s="306"/>
-      <c r="H5" s="306"/>
-      <c r="I5" s="306"/>
-      <c r="J5" s="306"/>
-      <c r="K5" s="306"/>
-      <c r="L5" s="306"/>
-      <c r="M5" s="306"/>
-      <c r="N5" s="306"/>
-      <c r="O5" s="306"/>
-      <c r="P5" s="306"/>
-      <c r="Q5" s="306"/>
-      <c r="R5" s="306"/>
-      <c r="S5" s="306"/>
-      <c r="T5" s="306"/>
-      <c r="U5" s="306"/>
+      <c r="B5" s="281"/>
+      <c r="C5" s="281"/>
+      <c r="D5" s="281"/>
+      <c r="E5" s="281"/>
+      <c r="F5" s="281"/>
+      <c r="G5" s="281"/>
+      <c r="H5" s="281"/>
+      <c r="I5" s="281"/>
+      <c r="J5" s="281"/>
+      <c r="K5" s="281"/>
+      <c r="L5" s="281"/>
+      <c r="M5" s="281"/>
+      <c r="N5" s="281"/>
+      <c r="O5" s="281"/>
+      <c r="P5" s="281"/>
+      <c r="Q5" s="281"/>
+      <c r="R5" s="281"/>
+      <c r="S5" s="281"/>
+      <c r="T5" s="281"/>
+      <c r="U5" s="281"/>
     </row>
     <row r="6" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="103"/>
@@ -12282,14 +12282,14 @@
         <v>87</v>
       </c>
       <c r="B7" s="104"/>
-      <c r="C7" s="309">
+      <c r="C7" s="291">
         <f>'DR-TB 10A'!C6:G6</f>
         <v>0</v>
       </c>
-      <c r="D7" s="309"/>
-      <c r="E7" s="309"/>
-      <c r="F7" s="309"/>
-      <c r="G7" s="309"/>
+      <c r="D7" s="291"/>
+      <c r="E7" s="291"/>
+      <c r="F7" s="291"/>
+      <c r="G7" s="291"/>
       <c r="H7" s="101"/>
       <c r="I7" s="104"/>
       <c r="J7" s="107" t="s">
@@ -12303,11 +12303,11 @@
       <c r="M7" s="108" t="s">
         <v>14</v>
       </c>
-      <c r="N7" s="308" t="str">
+      <c r="N7" s="290">
         <f>'DR-TB 10A'!N6:O6</f>
-        <v/>
-      </c>
-      <c r="O7" s="308"/>
+        <v>0</v>
+      </c>
+      <c r="O7" s="290"/>
       <c r="P7" s="109" t="s">
         <v>15</v>
       </c>
@@ -12325,14 +12325,14 @@
         <v>9</v>
       </c>
       <c r="B8" s="104"/>
-      <c r="C8" s="293">
+      <c r="C8" s="300">
         <f>'DR-TB 10A'!C7:G7</f>
         <v>0</v>
       </c>
-      <c r="D8" s="293"/>
-      <c r="E8" s="293"/>
-      <c r="F8" s="293"/>
-      <c r="G8" s="293"/>
+      <c r="D8" s="300"/>
+      <c r="E8" s="300"/>
+      <c r="F8" s="300"/>
+      <c r="G8" s="300"/>
       <c r="H8" s="101"/>
       <c r="I8" s="110"/>
       <c r="J8" s="124" t="s">
@@ -12341,12 +12341,12 @@
       <c r="K8" s="123"/>
       <c r="L8" s="123"/>
       <c r="M8" s="123"/>
-      <c r="N8" s="299"/>
-      <c r="O8" s="299"/>
-      <c r="P8" s="299"/>
-      <c r="Q8" s="299"/>
-      <c r="R8" s="299"/>
-      <c r="S8" s="299"/>
+      <c r="N8" s="296"/>
+      <c r="O8" s="296"/>
+      <c r="P8" s="296"/>
+      <c r="Q8" s="296"/>
+      <c r="R8" s="296"/>
+      <c r="S8" s="296"/>
       <c r="T8" s="101"/>
       <c r="U8" s="101"/>
     </row>
@@ -12355,14 +12355,14 @@
         <v>10</v>
       </c>
       <c r="B9" s="104"/>
-      <c r="C9" s="295">
+      <c r="C9" s="301">
         <f>'DR-TB 10A'!C8:G8</f>
         <v>0</v>
       </c>
-      <c r="D9" s="295"/>
-      <c r="E9" s="295"/>
-      <c r="F9" s="295"/>
-      <c r="G9" s="295"/>
+      <c r="D9" s="301"/>
+      <c r="E9" s="301"/>
+      <c r="F9" s="301"/>
+      <c r="G9" s="301"/>
       <c r="H9" s="101"/>
       <c r="I9" s="110"/>
       <c r="J9" s="110" t="s">
@@ -12370,13 +12370,13 @@
       </c>
       <c r="K9" s="110"/>
       <c r="L9" s="110"/>
-      <c r="M9" s="299"/>
-      <c r="N9" s="299"/>
-      <c r="O9" s="299"/>
-      <c r="P9" s="299"/>
-      <c r="Q9" s="299"/>
-      <c r="R9" s="299"/>
-      <c r="S9" s="299"/>
+      <c r="M9" s="296"/>
+      <c r="N9" s="296"/>
+      <c r="O9" s="296"/>
+      <c r="P9" s="296"/>
+      <c r="Q9" s="296"/>
+      <c r="R9" s="296"/>
+      <c r="S9" s="296"/>
       <c r="T9" s="101"/>
       <c r="U9" s="101"/>
     </row>
@@ -12395,8 +12395,8 @@
       </c>
       <c r="K10" s="110"/>
       <c r="L10" s="110"/>
-      <c r="M10" s="300"/>
-      <c r="N10" s="300"/>
+      <c r="M10" s="297"/>
+      <c r="N10" s="297"/>
       <c r="O10" s="111"/>
       <c r="P10" s="102"/>
       <c r="Q10" s="101"/>
@@ -12418,17 +12418,17 @@
       <c r="J11" s="112" t="s">
         <v>75</v>
       </c>
-      <c r="K11" s="301"/>
-      <c r="L11" s="301"/>
+      <c r="K11" s="298"/>
+      <c r="L11" s="298"/>
       <c r="M11" s="112"/>
       <c r="N11" s="113"/>
       <c r="O11" s="110" t="s">
         <v>12</v>
       </c>
       <c r="P11" s="101"/>
-      <c r="Q11" s="302"/>
-      <c r="R11" s="302"/>
-      <c r="S11" s="302"/>
+      <c r="Q11" s="299"/>
+      <c r="R11" s="299"/>
+      <c r="S11" s="299"/>
       <c r="T11" s="106"/>
       <c r="U11" s="101"/>
     </row>
@@ -12456,34 +12456,34 @@
       <c r="U12" s="101"/>
     </row>
     <row r="13" spans="1:21" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="273" t="s">
+      <c r="A13" s="303" t="s">
         <v>121</v>
       </c>
-      <c r="B13" s="296" t="s">
+      <c r="B13" s="302" t="s">
         <v>122</v>
       </c>
-      <c r="C13" s="296"/>
-      <c r="D13" s="296" t="s">
+      <c r="C13" s="302"/>
+      <c r="D13" s="302" t="s">
         <v>123</v>
       </c>
-      <c r="E13" s="296"/>
+      <c r="E13" s="302"/>
       <c r="F13" s="101"/>
       <c r="G13" s="101"/>
-      <c r="H13" s="276" t="s">
+      <c r="H13" s="305" t="s">
         <v>124</v>
       </c>
-      <c r="I13" s="277"/>
-      <c r="J13" s="277"/>
-      <c r="K13" s="278"/>
-      <c r="L13" s="282" t="s">
+      <c r="I13" s="306"/>
+      <c r="J13" s="306"/>
+      <c r="K13" s="307"/>
+      <c r="L13" s="311" t="s">
         <v>125</v>
       </c>
-      <c r="M13" s="282"/>
-      <c r="N13" s="282"/>
-      <c r="O13" s="283" t="s">
+      <c r="M13" s="311"/>
+      <c r="N13" s="311"/>
+      <c r="O13" s="312" t="s">
         <v>3</v>
       </c>
-      <c r="P13" s="284"/>
+      <c r="P13" s="313"/>
       <c r="Q13" s="106"/>
       <c r="R13" s="101"/>
       <c r="S13" s="101"/>
@@ -12491,25 +12491,25 @@
       <c r="U13" s="101"/>
     </row>
     <row r="14" spans="1:21" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="274"/>
-      <c r="B14" s="297"/>
-      <c r="C14" s="298"/>
-      <c r="D14" s="297"/>
-      <c r="E14" s="298"/>
+      <c r="A14" s="304"/>
+      <c r="B14" s="282"/>
+      <c r="C14" s="283"/>
+      <c r="D14" s="282"/>
+      <c r="E14" s="283"/>
       <c r="F14" s="101"/>
       <c r="G14" s="101"/>
-      <c r="H14" s="279"/>
-      <c r="I14" s="280"/>
-      <c r="J14" s="280"/>
-      <c r="K14" s="281"/>
+      <c r="H14" s="308"/>
+      <c r="I14" s="309"/>
+      <c r="J14" s="309"/>
+      <c r="K14" s="310"/>
       <c r="L14" s="136"/>
       <c r="M14" s="137"/>
       <c r="N14" s="138"/>
-      <c r="O14" s="285">
+      <c r="O14" s="314">
         <f>L14+M14+N14</f>
         <v>0</v>
       </c>
-      <c r="P14" s="286"/>
+      <c r="P14" s="315"/>
       <c r="Q14" s="106"/>
       <c r="R14" s="101"/>
       <c r="S14" s="101"/>
@@ -12563,21 +12563,21 @@
       <c r="U16" s="118"/>
     </row>
     <row r="17" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="291"/>
-      <c r="B17" s="291"/>
+      <c r="A17" s="316"/>
+      <c r="B17" s="316"/>
       <c r="C17" s="287" t="s">
         <v>126</v>
       </c>
       <c r="D17" s="287"/>
       <c r="E17" s="287"/>
-      <c r="F17" s="305" t="s">
+      <c r="F17" s="294" t="s">
         <v>127</v>
       </c>
-      <c r="G17" s="305"/>
-      <c r="H17" s="305"/>
-      <c r="I17" s="305"/>
-      <c r="J17" s="305"/>
-      <c r="K17" s="305"/>
+      <c r="G17" s="294"/>
+      <c r="H17" s="294"/>
+      <c r="I17" s="294"/>
+      <c r="J17" s="294"/>
+      <c r="K17" s="294"/>
       <c r="L17" s="287" t="s">
         <v>128</v>
       </c>
@@ -12589,32 +12589,32 @@
       <c r="R17" s="101"/>
       <c r="S17" s="101"/>
       <c r="T17" s="101"/>
-      <c r="U17" s="303"/>
+      <c r="U17" s="292"/>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A18" s="291"/>
-      <c r="B18" s="291"/>
-      <c r="C18" s="294" t="s">
+      <c r="A18" s="316"/>
+      <c r="B18" s="316"/>
+      <c r="C18" s="295" t="s">
         <v>129</v>
       </c>
-      <c r="D18" s="294" t="s">
+      <c r="D18" s="295" t="s">
         <v>130</v>
       </c>
-      <c r="E18" s="294" t="s">
+      <c r="E18" s="295" t="s">
         <v>3</v>
       </c>
-      <c r="F18" s="305" t="s">
+      <c r="F18" s="294" t="s">
         <v>129</v>
       </c>
-      <c r="G18" s="305"/>
-      <c r="H18" s="305" t="s">
+      <c r="G18" s="294"/>
+      <c r="H18" s="294" t="s">
         <v>130</v>
       </c>
-      <c r="I18" s="305"/>
-      <c r="J18" s="305" t="s">
+      <c r="I18" s="294"/>
+      <c r="J18" s="294" t="s">
         <v>3</v>
       </c>
-      <c r="K18" s="305"/>
+      <c r="K18" s="294"/>
       <c r="L18" s="287" t="s">
         <v>129</v>
       </c>
@@ -12623,159 +12623,159 @@
         <v>130</v>
       </c>
       <c r="O18" s="287"/>
-      <c r="P18" s="294" t="s">
+      <c r="P18" s="295" t="s">
         <v>3</v>
       </c>
-      <c r="Q18" s="294"/>
+      <c r="Q18" s="295"/>
       <c r="R18" s="101"/>
       <c r="S18" s="101"/>
       <c r="T18" s="101"/>
-      <c r="U18" s="303"/>
+      <c r="U18" s="292"/>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A19" s="291"/>
-      <c r="B19" s="291"/>
-      <c r="C19" s="294"/>
-      <c r="D19" s="294"/>
-      <c r="E19" s="294"/>
-      <c r="F19" s="305"/>
-      <c r="G19" s="305"/>
-      <c r="H19" s="305"/>
-      <c r="I19" s="305"/>
-      <c r="J19" s="305"/>
-      <c r="K19" s="305"/>
+      <c r="A19" s="316"/>
+      <c r="B19" s="316"/>
+      <c r="C19" s="295"/>
+      <c r="D19" s="295"/>
+      <c r="E19" s="295"/>
+      <c r="F19" s="294"/>
+      <c r="G19" s="294"/>
+      <c r="H19" s="294"/>
+      <c r="I19" s="294"/>
+      <c r="J19" s="294"/>
+      <c r="K19" s="294"/>
       <c r="L19" s="287"/>
       <c r="M19" s="287"/>
       <c r="N19" s="287"/>
       <c r="O19" s="287"/>
-      <c r="P19" s="294"/>
-      <c r="Q19" s="294"/>
+      <c r="P19" s="295"/>
+      <c r="Q19" s="295"/>
       <c r="R19" s="101"/>
       <c r="S19" s="101"/>
       <c r="T19" s="101"/>
-      <c r="U19" s="303"/>
+      <c r="U19" s="292"/>
     </row>
     <row r="20" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="287" t="s">
         <v>131</v>
       </c>
       <c r="B20" s="287"/>
-      <c r="C20" s="292"/>
-      <c r="D20" s="292"/>
-      <c r="E20" s="275">
+      <c r="C20" s="288"/>
+      <c r="D20" s="288"/>
+      <c r="E20" s="286">
         <f>C20+D20</f>
         <v>0</v>
       </c>
       <c r="F20" s="289"/>
       <c r="G20" s="289"/>
-      <c r="H20" s="290"/>
-      <c r="I20" s="290"/>
-      <c r="J20" s="288">
+      <c r="H20" s="278"/>
+      <c r="I20" s="278"/>
+      <c r="J20" s="279">
         <f>F20+H20</f>
         <v>0</v>
       </c>
-      <c r="K20" s="288"/>
-      <c r="L20" s="275">
+      <c r="K20" s="279"/>
+      <c r="L20" s="286">
         <f>C20+F20</f>
         <v>0</v>
       </c>
-      <c r="M20" s="275"/>
-      <c r="N20" s="275">
+      <c r="M20" s="286"/>
+      <c r="N20" s="286">
         <f>D20+H20</f>
         <v>0</v>
       </c>
-      <c r="O20" s="275"/>
-      <c r="P20" s="275">
+      <c r="O20" s="286"/>
+      <c r="P20" s="286">
         <f>L20+N20</f>
         <v>0</v>
       </c>
-      <c r="Q20" s="275"/>
+      <c r="Q20" s="286"/>
       <c r="R20" s="101"/>
       <c r="S20" s="101"/>
       <c r="T20" s="101"/>
-      <c r="U20" s="304"/>
+      <c r="U20" s="293"/>
     </row>
     <row r="21" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="287"/>
       <c r="B21" s="287"/>
-      <c r="C21" s="292"/>
-      <c r="D21" s="292"/>
-      <c r="E21" s="275"/>
+      <c r="C21" s="288"/>
+      <c r="D21" s="288"/>
+      <c r="E21" s="286"/>
       <c r="F21" s="289"/>
       <c r="G21" s="289"/>
-      <c r="H21" s="290"/>
-      <c r="I21" s="290"/>
-      <c r="J21" s="288"/>
-      <c r="K21" s="288"/>
-      <c r="L21" s="275"/>
-      <c r="M21" s="275"/>
-      <c r="N21" s="275"/>
-      <c r="O21" s="275"/>
-      <c r="P21" s="275"/>
-      <c r="Q21" s="275"/>
+      <c r="H21" s="278"/>
+      <c r="I21" s="278"/>
+      <c r="J21" s="279"/>
+      <c r="K21" s="279"/>
+      <c r="L21" s="286"/>
+      <c r="M21" s="286"/>
+      <c r="N21" s="286"/>
+      <c r="O21" s="286"/>
+      <c r="P21" s="286"/>
+      <c r="Q21" s="286"/>
       <c r="R21" s="101"/>
       <c r="S21" s="101"/>
       <c r="T21" s="101"/>
-      <c r="U21" s="304"/>
+      <c r="U21" s="293"/>
     </row>
     <row r="22" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="287"/>
       <c r="B22" s="287"/>
-      <c r="C22" s="292"/>
-      <c r="D22" s="292"/>
-      <c r="E22" s="275"/>
+      <c r="C22" s="288"/>
+      <c r="D22" s="288"/>
+      <c r="E22" s="286"/>
       <c r="F22" s="289"/>
       <c r="G22" s="289"/>
-      <c r="H22" s="290"/>
-      <c r="I22" s="290"/>
-      <c r="J22" s="288"/>
-      <c r="K22" s="288"/>
-      <c r="L22" s="275"/>
-      <c r="M22" s="275"/>
-      <c r="N22" s="275"/>
-      <c r="O22" s="275"/>
-      <c r="P22" s="275"/>
-      <c r="Q22" s="275"/>
+      <c r="H22" s="278"/>
+      <c r="I22" s="278"/>
+      <c r="J22" s="279"/>
+      <c r="K22" s="279"/>
+      <c r="L22" s="286"/>
+      <c r="M22" s="286"/>
+      <c r="N22" s="286"/>
+      <c r="O22" s="286"/>
+      <c r="P22" s="286"/>
+      <c r="Q22" s="286"/>
       <c r="R22" s="101"/>
       <c r="S22" s="101"/>
       <c r="T22" s="101"/>
-      <c r="U22" s="304"/>
+      <c r="U22" s="293"/>
     </row>
     <row r="23" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="287" t="s">
         <v>132</v>
       </c>
       <c r="B23" s="287"/>
-      <c r="C23" s="292"/>
-      <c r="D23" s="292"/>
-      <c r="E23" s="275">
+      <c r="C23" s="288"/>
+      <c r="D23" s="288"/>
+      <c r="E23" s="286">
         <f t="shared" ref="E23" si="0">C23+D23</f>
         <v>0</v>
       </c>
       <c r="F23" s="289"/>
       <c r="G23" s="289"/>
-      <c r="H23" s="290"/>
-      <c r="I23" s="290"/>
-      <c r="J23" s="288">
+      <c r="H23" s="278"/>
+      <c r="I23" s="278"/>
+      <c r="J23" s="279">
         <f t="shared" ref="J23" si="1">F23+H23</f>
         <v>0</v>
       </c>
-      <c r="K23" s="288"/>
-      <c r="L23" s="275">
+      <c r="K23" s="279"/>
+      <c r="L23" s="286">
         <f t="shared" ref="L23" si="2">C23+F23</f>
         <v>0</v>
       </c>
-      <c r="M23" s="275"/>
-      <c r="N23" s="275">
+      <c r="M23" s="286"/>
+      <c r="N23" s="286">
         <f t="shared" ref="N23" si="3">D23+H23</f>
         <v>0</v>
       </c>
-      <c r="O23" s="275"/>
-      <c r="P23" s="275">
+      <c r="O23" s="286"/>
+      <c r="P23" s="286">
         <f t="shared" ref="P23" si="4">L23+N23</f>
         <v>0</v>
       </c>
-      <c r="Q23" s="275"/>
+      <c r="Q23" s="286"/>
       <c r="R23" s="101"/>
       <c r="S23" s="101"/>
       <c r="T23" s="101"/>
@@ -12784,21 +12784,21 @@
     <row r="24" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="287"/>
       <c r="B24" s="287"/>
-      <c r="C24" s="292"/>
-      <c r="D24" s="292"/>
-      <c r="E24" s="275"/>
+      <c r="C24" s="288"/>
+      <c r="D24" s="288"/>
+      <c r="E24" s="286"/>
       <c r="F24" s="289"/>
       <c r="G24" s="289"/>
-      <c r="H24" s="290"/>
-      <c r="I24" s="290"/>
-      <c r="J24" s="288"/>
-      <c r="K24" s="288"/>
-      <c r="L24" s="275"/>
-      <c r="M24" s="275"/>
-      <c r="N24" s="275"/>
-      <c r="O24" s="275"/>
-      <c r="P24" s="275"/>
-      <c r="Q24" s="275"/>
+      <c r="H24" s="278"/>
+      <c r="I24" s="278"/>
+      <c r="J24" s="279"/>
+      <c r="K24" s="279"/>
+      <c r="L24" s="286"/>
+      <c r="M24" s="286"/>
+      <c r="N24" s="286"/>
+      <c r="O24" s="286"/>
+      <c r="P24" s="286"/>
+      <c r="Q24" s="286"/>
       <c r="R24" s="101"/>
       <c r="S24" s="101"/>
       <c r="T24" s="101"/>
@@ -12807,21 +12807,21 @@
     <row r="25" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="287"/>
       <c r="B25" s="287"/>
-      <c r="C25" s="292"/>
-      <c r="D25" s="292"/>
-      <c r="E25" s="275"/>
+      <c r="C25" s="288"/>
+      <c r="D25" s="288"/>
+      <c r="E25" s="286"/>
       <c r="F25" s="289"/>
       <c r="G25" s="289"/>
-      <c r="H25" s="290"/>
-      <c r="I25" s="290"/>
-      <c r="J25" s="288"/>
-      <c r="K25" s="288"/>
-      <c r="L25" s="275"/>
-      <c r="M25" s="275"/>
-      <c r="N25" s="275"/>
-      <c r="O25" s="275"/>
-      <c r="P25" s="275"/>
-      <c r="Q25" s="275"/>
+      <c r="H25" s="278"/>
+      <c r="I25" s="278"/>
+      <c r="J25" s="279"/>
+      <c r="K25" s="279"/>
+      <c r="L25" s="286"/>
+      <c r="M25" s="286"/>
+      <c r="N25" s="286"/>
+      <c r="O25" s="286"/>
+      <c r="P25" s="286"/>
+      <c r="Q25" s="286"/>
       <c r="R25" s="101"/>
       <c r="S25" s="101"/>
       <c r="T25" s="101"/>
@@ -12832,36 +12832,36 @@
         <v>133</v>
       </c>
       <c r="B26" s="287"/>
-      <c r="C26" s="292"/>
-      <c r="D26" s="292"/>
-      <c r="E26" s="275">
+      <c r="C26" s="288"/>
+      <c r="D26" s="288"/>
+      <c r="E26" s="286">
         <f t="shared" ref="E26" si="5">C26+D26</f>
         <v>0</v>
       </c>
       <c r="F26" s="289"/>
       <c r="G26" s="289"/>
-      <c r="H26" s="290"/>
-      <c r="I26" s="290"/>
-      <c r="J26" s="288">
+      <c r="H26" s="278"/>
+      <c r="I26" s="278"/>
+      <c r="J26" s="279">
         <f t="shared" ref="J26" si="6">F26+H26</f>
         <v>0</v>
       </c>
-      <c r="K26" s="288"/>
-      <c r="L26" s="275">
+      <c r="K26" s="279"/>
+      <c r="L26" s="286">
         <f t="shared" ref="L26" si="7">C26+F26</f>
         <v>0</v>
       </c>
-      <c r="M26" s="275"/>
-      <c r="N26" s="275">
+      <c r="M26" s="286"/>
+      <c r="N26" s="286">
         <f t="shared" ref="N26" si="8">D26+H26</f>
         <v>0</v>
       </c>
-      <c r="O26" s="275"/>
-      <c r="P26" s="275">
+      <c r="O26" s="286"/>
+      <c r="P26" s="286">
         <f t="shared" ref="P26" si="9">L26+N26</f>
         <v>0</v>
       </c>
-      <c r="Q26" s="275"/>
+      <c r="Q26" s="286"/>
       <c r="R26" s="125"/>
       <c r="S26" s="135"/>
       <c r="T26" s="135"/>
@@ -12870,21 +12870,21 @@
     <row r="27" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="287"/>
       <c r="B27" s="287"/>
-      <c r="C27" s="292"/>
-      <c r="D27" s="292"/>
-      <c r="E27" s="275"/>
+      <c r="C27" s="288"/>
+      <c r="D27" s="288"/>
+      <c r="E27" s="286"/>
       <c r="F27" s="289"/>
       <c r="G27" s="289"/>
-      <c r="H27" s="290"/>
-      <c r="I27" s="290"/>
-      <c r="J27" s="288"/>
-      <c r="K27" s="288"/>
-      <c r="L27" s="275"/>
-      <c r="M27" s="275"/>
-      <c r="N27" s="275"/>
-      <c r="O27" s="275"/>
-      <c r="P27" s="275"/>
-      <c r="Q27" s="275"/>
+      <c r="H27" s="278"/>
+      <c r="I27" s="278"/>
+      <c r="J27" s="279"/>
+      <c r="K27" s="279"/>
+      <c r="L27" s="286"/>
+      <c r="M27" s="286"/>
+      <c r="N27" s="286"/>
+      <c r="O27" s="286"/>
+      <c r="P27" s="286"/>
+      <c r="Q27" s="286"/>
       <c r="R27" s="125"/>
       <c r="S27" s="135"/>
       <c r="T27" s="135"/>
@@ -12893,21 +12893,21 @@
     <row r="28" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="287"/>
       <c r="B28" s="287"/>
-      <c r="C28" s="292"/>
-      <c r="D28" s="292"/>
-      <c r="E28" s="275"/>
+      <c r="C28" s="288"/>
+      <c r="D28" s="288"/>
+      <c r="E28" s="286"/>
       <c r="F28" s="289"/>
       <c r="G28" s="289"/>
-      <c r="H28" s="290"/>
-      <c r="I28" s="290"/>
-      <c r="J28" s="288"/>
-      <c r="K28" s="288"/>
-      <c r="L28" s="275"/>
-      <c r="M28" s="275"/>
-      <c r="N28" s="275"/>
-      <c r="O28" s="275"/>
-      <c r="P28" s="275"/>
-      <c r="Q28" s="275"/>
+      <c r="H28" s="278"/>
+      <c r="I28" s="278"/>
+      <c r="J28" s="279"/>
+      <c r="K28" s="279"/>
+      <c r="L28" s="286"/>
+      <c r="M28" s="286"/>
+      <c r="N28" s="286"/>
+      <c r="O28" s="286"/>
+      <c r="P28" s="286"/>
+      <c r="Q28" s="286"/>
       <c r="R28" s="125"/>
       <c r="S28" s="135"/>
       <c r="T28" s="135"/>
@@ -12951,13 +12951,13 @@
       <c r="J30" s="106"/>
       <c r="K30" s="106"/>
       <c r="L30" s="106"/>
-      <c r="M30" s="310"/>
-      <c r="N30" s="310"/>
-      <c r="O30" s="310"/>
-      <c r="P30" s="310"/>
-      <c r="Q30" s="310"/>
-      <c r="R30" s="310"/>
-      <c r="S30" s="310"/>
+      <c r="M30" s="284"/>
+      <c r="N30" s="284"/>
+      <c r="O30" s="284"/>
+      <c r="P30" s="284"/>
+      <c r="Q30" s="284"/>
+      <c r="R30" s="284"/>
+      <c r="S30" s="284"/>
       <c r="T30" s="101"/>
       <c r="U30" s="101"/>
     </row>
@@ -12972,17 +12972,17 @@
       <c r="H31" s="105" t="s">
         <v>59</v>
       </c>
-      <c r="I31" s="313"/>
-      <c r="J31" s="313"/>
-      <c r="K31" s="313"/>
-      <c r="L31" s="313"/>
+      <c r="I31" s="277"/>
+      <c r="J31" s="277"/>
+      <c r="K31" s="277"/>
+      <c r="L31" s="277"/>
       <c r="M31" s="101"/>
       <c r="N31" s="119" t="s">
         <v>60</v>
       </c>
-      <c r="O31" s="311"/>
-      <c r="P31" s="311"/>
-      <c r="Q31" s="311"/>
+      <c r="O31" s="285"/>
+      <c r="P31" s="285"/>
+      <c r="Q31" s="285"/>
     </row>
     <row r="32" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A32" s="128"/>
@@ -12995,11 +12995,11 @@
       <c r="H32" s="105" t="s">
         <v>61</v>
       </c>
-      <c r="I32" s="312"/>
-      <c r="J32" s="312"/>
-      <c r="K32" s="312"/>
-      <c r="L32" s="312"/>
-      <c r="M32" s="312"/>
+      <c r="I32" s="276"/>
+      <c r="J32" s="276"/>
+      <c r="K32" s="276"/>
+      <c r="L32" s="276"/>
+      <c r="M32" s="276"/>
       <c r="N32" s="101"/>
       <c r="O32" s="101"/>
       <c r="P32" s="101"/>
@@ -13026,11 +13026,57 @@
     </row>
   </sheetData>
   <mergeCells count="72">
-    <mergeCell ref="I32:M32"/>
-    <mergeCell ref="I31:L31"/>
-    <mergeCell ref="H23:I25"/>
-    <mergeCell ref="J26:K28"/>
-    <mergeCell ref="H20:I22"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="L26:M28"/>
+    <mergeCell ref="N26:O28"/>
+    <mergeCell ref="P26:Q28"/>
+    <mergeCell ref="H13:K14"/>
+    <mergeCell ref="L13:N13"/>
+    <mergeCell ref="O13:P13"/>
+    <mergeCell ref="O14:P14"/>
+    <mergeCell ref="N18:O19"/>
+    <mergeCell ref="J20:K22"/>
+    <mergeCell ref="F26:G28"/>
+    <mergeCell ref="H26:I28"/>
+    <mergeCell ref="A17:B19"/>
+    <mergeCell ref="C20:C22"/>
+    <mergeCell ref="D20:D22"/>
+    <mergeCell ref="F20:G22"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="N8:S8"/>
+    <mergeCell ref="M9:S9"/>
+    <mergeCell ref="M10:N10"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="Q11:S11"/>
+    <mergeCell ref="U17:U19"/>
+    <mergeCell ref="U20:U22"/>
+    <mergeCell ref="J23:K25"/>
+    <mergeCell ref="F18:G19"/>
+    <mergeCell ref="H18:I19"/>
+    <mergeCell ref="J18:K19"/>
+    <mergeCell ref="F17:K17"/>
+    <mergeCell ref="L18:M19"/>
+    <mergeCell ref="L17:Q17"/>
+    <mergeCell ref="P18:Q19"/>
+    <mergeCell ref="L20:M22"/>
+    <mergeCell ref="L23:M25"/>
+    <mergeCell ref="N20:O22"/>
+    <mergeCell ref="N23:O25"/>
+    <mergeCell ref="P20:Q22"/>
+    <mergeCell ref="P23:Q25"/>
+    <mergeCell ref="A5:U5"/>
+    <mergeCell ref="A2:U2"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="N7:O7"/>
+    <mergeCell ref="C7:G7"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="P1:S1"/>
     <mergeCell ref="D14:E14"/>
@@ -13047,57 +13093,11 @@
     <mergeCell ref="D26:D28"/>
     <mergeCell ref="E26:E28"/>
     <mergeCell ref="A23:B25"/>
-    <mergeCell ref="A5:U5"/>
-    <mergeCell ref="A2:U2"/>
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="N7:O7"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="U17:U19"/>
-    <mergeCell ref="U20:U22"/>
-    <mergeCell ref="J23:K25"/>
-    <mergeCell ref="F18:G19"/>
-    <mergeCell ref="H18:I19"/>
-    <mergeCell ref="J18:K19"/>
-    <mergeCell ref="F17:K17"/>
-    <mergeCell ref="L18:M19"/>
-    <mergeCell ref="L17:Q17"/>
-    <mergeCell ref="P18:Q19"/>
-    <mergeCell ref="L20:M22"/>
-    <mergeCell ref="L23:M25"/>
-    <mergeCell ref="N20:O22"/>
-    <mergeCell ref="N23:O25"/>
-    <mergeCell ref="P20:Q22"/>
-    <mergeCell ref="P23:Q25"/>
-    <mergeCell ref="N8:S8"/>
-    <mergeCell ref="M9:S9"/>
-    <mergeCell ref="M10:N10"/>
-    <mergeCell ref="K11:L11"/>
-    <mergeCell ref="Q11:S11"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="L26:M28"/>
-    <mergeCell ref="N26:O28"/>
-    <mergeCell ref="P26:Q28"/>
-    <mergeCell ref="H13:K14"/>
-    <mergeCell ref="L13:N13"/>
-    <mergeCell ref="O13:P13"/>
-    <mergeCell ref="O14:P14"/>
-    <mergeCell ref="N18:O19"/>
-    <mergeCell ref="J20:K22"/>
-    <mergeCell ref="F26:G28"/>
-    <mergeCell ref="H26:I28"/>
-    <mergeCell ref="A17:B19"/>
-    <mergeCell ref="C20:C22"/>
-    <mergeCell ref="D20:D22"/>
-    <mergeCell ref="F20:G22"/>
+    <mergeCell ref="I32:M32"/>
+    <mergeCell ref="I31:L31"/>
+    <mergeCell ref="H23:I25"/>
+    <mergeCell ref="J26:K28"/>
+    <mergeCell ref="H20:I22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
text change in Excel cell caption
</commit_message>
<xml_diff>
--- a/api/templates/results_dr_tb_10a/en.xlsx
+++ b/api/templates/results_dr_tb_10a/en.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect\api\templates\results_dr_tb_10a\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect-2\api\templates\results_dr_tb_10a\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -170,9 +170,6 @@
   </si>
   <si>
     <t>Column (3)</t>
-  </si>
-  <si>
-    <t>Non converters of CAT II (remain positive at month 3)</t>
   </si>
   <si>
     <t>Column (4)</t>
@@ -784,6 +781,9 @@
   </si>
   <si>
     <t>Date Of Enrollment</t>
+  </si>
+  <si>
+    <t>Non converters of CAT II (remain positive at month 2-3)</t>
   </si>
 </sst>
 </file>
@@ -2735,6 +2735,417 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="6" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="6" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="1"/>
@@ -2839,417 +3250,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="53" fillId="6" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="53" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="53" fillId="6" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
@@ -3261,6 +3265,162 @@
     <xf numFmtId="0" fontId="40" fillId="0" borderId="56" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="76" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="58" fillId="0" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" shrinkToFit="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="59" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" shrinkToFit="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="57" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <protection locked="0" hidden="1"/>
     </xf>
     <xf numFmtId="49" fontId="57" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
@@ -3269,166 +3429,6 @@
     <xf numFmtId="0" fontId="50" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="52" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="57" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="57" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="52" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="58" fillId="0" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" shrinkToFit="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="59" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" shrinkToFit="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="76" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="21">
@@ -3887,28 +3887,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="232" t="s">
-        <v>71</v>
-      </c>
-      <c r="B1" s="232"/>
-      <c r="C1" s="232"/>
-      <c r="D1" s="232"/>
-      <c r="E1" s="232"/>
-      <c r="F1" s="232"/>
-      <c r="G1" s="232"/>
-      <c r="H1" s="232"/>
-      <c r="I1" s="232"/>
-      <c r="J1" s="232"/>
-      <c r="K1" s="232"/>
-      <c r="L1" s="232"/>
-      <c r="M1" s="232"/>
-      <c r="N1" s="232"/>
-      <c r="O1" s="232"/>
-      <c r="P1" s="232"/>
-      <c r="Q1" s="232"/>
-      <c r="R1" s="232"/>
+      <c r="A1" s="165" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="165"/>
+      <c r="C1" s="165"/>
+      <c r="D1" s="165"/>
+      <c r="E1" s="165"/>
+      <c r="F1" s="165"/>
+      <c r="G1" s="165"/>
+      <c r="H1" s="165"/>
+      <c r="I1" s="165"/>
+      <c r="J1" s="165"/>
+      <c r="K1" s="165"/>
+      <c r="L1" s="165"/>
+      <c r="M1" s="165"/>
+      <c r="N1" s="165"/>
+      <c r="O1" s="165"/>
+      <c r="P1" s="165"/>
+      <c r="Q1" s="165"/>
+      <c r="R1" s="165"/>
       <c r="S1" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
@@ -3916,54 +3916,54 @@
       <c r="X1" s="1"/>
     </row>
     <row r="2" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="232" t="s">
-        <v>67</v>
-      </c>
-      <c r="B2" s="232"/>
-      <c r="C2" s="232"/>
-      <c r="D2" s="232"/>
-      <c r="E2" s="232"/>
-      <c r="F2" s="232"/>
-      <c r="G2" s="232"/>
-      <c r="H2" s="232"/>
-      <c r="I2" s="232"/>
-      <c r="J2" s="232"/>
-      <c r="K2" s="232"/>
-      <c r="L2" s="232"/>
-      <c r="M2" s="232"/>
-      <c r="N2" s="232"/>
-      <c r="O2" s="232"/>
-      <c r="P2" s="232"/>
-      <c r="Q2" s="232"/>
-      <c r="R2" s="232"/>
-      <c r="S2" s="232"/>
-      <c r="T2" s="232"/>
-      <c r="U2" s="232"/>
+      <c r="A2" s="165" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="165"/>
+      <c r="C2" s="165"/>
+      <c r="D2" s="165"/>
+      <c r="E2" s="165"/>
+      <c r="F2" s="165"/>
+      <c r="G2" s="165"/>
+      <c r="H2" s="165"/>
+      <c r="I2" s="165"/>
+      <c r="J2" s="165"/>
+      <c r="K2" s="165"/>
+      <c r="L2" s="165"/>
+      <c r="M2" s="165"/>
+      <c r="N2" s="165"/>
+      <c r="O2" s="165"/>
+      <c r="P2" s="165"/>
+      <c r="Q2" s="165"/>
+      <c r="R2" s="165"/>
+      <c r="S2" s="165"/>
+      <c r="T2" s="165"/>
+      <c r="U2" s="165"/>
       <c r="V2" s="1"/>
       <c r="W2" s="1"/>
       <c r="X2" s="1"/>
     </row>
     <row r="3" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="232" t="s">
-        <v>80</v>
-      </c>
-      <c r="B3" s="232"/>
-      <c r="C3" s="232"/>
-      <c r="D3" s="232"/>
-      <c r="E3" s="232"/>
-      <c r="F3" s="232"/>
-      <c r="G3" s="232"/>
-      <c r="H3" s="232"/>
-      <c r="I3" s="232"/>
-      <c r="J3" s="232"/>
-      <c r="K3" s="232"/>
-      <c r="L3" s="232"/>
-      <c r="M3" s="232"/>
-      <c r="N3" s="232"/>
-      <c r="O3" s="232"/>
-      <c r="P3" s="232"/>
-      <c r="Q3" s="232"/>
-      <c r="R3" s="232"/>
+      <c r="A3" s="165" t="s">
+        <v>79</v>
+      </c>
+      <c r="B3" s="165"/>
+      <c r="C3" s="165"/>
+      <c r="D3" s="165"/>
+      <c r="E3" s="165"/>
+      <c r="F3" s="165"/>
+      <c r="G3" s="165"/>
+      <c r="H3" s="165"/>
+      <c r="I3" s="165"/>
+      <c r="J3" s="165"/>
+      <c r="K3" s="165"/>
+      <c r="L3" s="165"/>
+      <c r="M3" s="165"/>
+      <c r="N3" s="165"/>
+      <c r="O3" s="165"/>
+      <c r="P3" s="165"/>
+      <c r="Q3" s="165"/>
+      <c r="R3" s="165"/>
       <c r="S3" s="43"/>
       <c r="T3" s="43"/>
       <c r="U3" s="43"/>
@@ -3972,29 +3972,29 @@
       <c r="X3" s="1"/>
     </row>
     <row r="4" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="244" t="s">
-        <v>72</v>
-      </c>
-      <c r="B4" s="244"/>
-      <c r="C4" s="244"/>
-      <c r="D4" s="244"/>
-      <c r="E4" s="244"/>
-      <c r="F4" s="244"/>
-      <c r="G4" s="244"/>
-      <c r="H4" s="244"/>
-      <c r="I4" s="244"/>
-      <c r="J4" s="244"/>
-      <c r="K4" s="244"/>
-      <c r="L4" s="244"/>
-      <c r="M4" s="244"/>
-      <c r="N4" s="244"/>
-      <c r="O4" s="244"/>
-      <c r="P4" s="244"/>
-      <c r="Q4" s="244"/>
-      <c r="R4" s="244"/>
-      <c r="S4" s="244"/>
-      <c r="T4" s="244"/>
-      <c r="U4" s="244"/>
+      <c r="A4" s="177" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="177"/>
+      <c r="C4" s="177"/>
+      <c r="D4" s="177"/>
+      <c r="E4" s="177"/>
+      <c r="F4" s="177"/>
+      <c r="G4" s="177"/>
+      <c r="H4" s="177"/>
+      <c r="I4" s="177"/>
+      <c r="J4" s="177"/>
+      <c r="K4" s="177"/>
+      <c r="L4" s="177"/>
+      <c r="M4" s="177"/>
+      <c r="N4" s="177"/>
+      <c r="O4" s="177"/>
+      <c r="P4" s="177"/>
+      <c r="Q4" s="177"/>
+      <c r="R4" s="177"/>
+      <c r="S4" s="177"/>
+      <c r="T4" s="177"/>
+      <c r="U4" s="177"/>
       <c r="V4" s="4"/>
       <c r="W4" s="4"/>
       <c r="X4" s="4"/>
@@ -4027,14 +4027,14 @@
     </row>
     <row r="6" spans="1:603" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B6" s="5"/>
-      <c r="C6" s="255"/>
-      <c r="D6" s="255"/>
-      <c r="E6" s="255"/>
-      <c r="F6" s="255"/>
-      <c r="G6" s="255"/>
+      <c r="C6" s="141"/>
+      <c r="D6" s="141"/>
+      <c r="E6" s="141"/>
+      <c r="F6" s="141"/>
+      <c r="G6" s="141"/>
       <c r="I6" s="1"/>
       <c r="J6" s="7" t="s">
         <v>16</v>
@@ -4043,8 +4043,8 @@
       <c r="M6" s="62" t="s">
         <v>14</v>
       </c>
-      <c r="N6" s="317"/>
-      <c r="O6" s="317"/>
+      <c r="N6" s="219"/>
+      <c r="O6" s="219"/>
       <c r="P6" s="8" t="s">
         <v>15</v>
       </c>
@@ -4055,48 +4055,48 @@
         <v>9</v>
       </c>
       <c r="B7" s="5"/>
-      <c r="C7" s="256"/>
-      <c r="D7" s="256"/>
-      <c r="E7" s="256"/>
-      <c r="F7" s="256"/>
-      <c r="G7" s="256"/>
+      <c r="C7" s="142"/>
+      <c r="D7" s="142"/>
+      <c r="E7" s="142"/>
+      <c r="F7" s="142"/>
+      <c r="G7" s="142"/>
       <c r="I7" s="6"/>
       <c r="J7" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K7" s="9"/>
       <c r="L7" s="9"/>
       <c r="M7" s="9"/>
-      <c r="N7" s="261"/>
-      <c r="O7" s="261"/>
-      <c r="P7" s="261"/>
-      <c r="Q7" s="261"/>
-      <c r="R7" s="261"/>
-      <c r="S7" s="261"/>
+      <c r="N7" s="147"/>
+      <c r="O7" s="147"/>
+      <c r="P7" s="147"/>
+      <c r="Q7" s="147"/>
+      <c r="R7" s="147"/>
+      <c r="S7" s="147"/>
     </row>
     <row r="8" spans="1:603" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="5"/>
-      <c r="C8" s="257"/>
-      <c r="D8" s="257"/>
-      <c r="E8" s="257"/>
-      <c r="F8" s="257"/>
-      <c r="G8" s="257"/>
+      <c r="C8" s="143"/>
+      <c r="D8" s="143"/>
+      <c r="E8" s="143"/>
+      <c r="F8" s="143"/>
+      <c r="G8" s="143"/>
       <c r="I8" s="6"/>
       <c r="J8" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K8" s="9"/>
       <c r="L8" s="9"/>
-      <c r="M8" s="261"/>
-      <c r="N8" s="261"/>
-      <c r="O8" s="261"/>
-      <c r="P8" s="261"/>
-      <c r="Q8" s="261"/>
-      <c r="R8" s="261"/>
-      <c r="S8" s="261"/>
+      <c r="M8" s="147"/>
+      <c r="N8" s="147"/>
+      <c r="O8" s="147"/>
+      <c r="P8" s="147"/>
+      <c r="Q8" s="147"/>
+      <c r="R8" s="147"/>
+      <c r="S8" s="147"/>
     </row>
     <row r="9" spans="1:603" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="J9" s="9" t="s">
@@ -4104,25 +4104,25 @@
       </c>
       <c r="K9" s="9"/>
       <c r="L9" s="9"/>
-      <c r="M9" s="262"/>
-      <c r="N9" s="262"/>
+      <c r="M9" s="148"/>
+      <c r="N9" s="148"/>
       <c r="O9" s="64"/>
       <c r="P9" s="63"/>
     </row>
     <row r="10" spans="1:603" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="J10" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="K10" s="263"/>
-      <c r="L10" s="263"/>
+        <v>74</v>
+      </c>
+      <c r="K10" s="149"/>
+      <c r="L10" s="149"/>
       <c r="M10" s="10"/>
       <c r="N10" s="11"/>
       <c r="O10" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="Q10" s="264"/>
-      <c r="R10" s="264"/>
-      <c r="S10" s="264"/>
+      <c r="Q10" s="150"/>
+      <c r="R10" s="150"/>
+      <c r="S10" s="150"/>
       <c r="T10" s="19"/>
     </row>
     <row r="11" spans="1:603" s="11" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -4726,27 +4726,27 @@
       <c r="WE11" s="24"/>
     </row>
     <row r="12" spans="1:603" s="25" customFormat="1" ht="13.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="188" t="s">
-        <v>74</v>
-      </c>
-      <c r="B12" s="189"/>
-      <c r="C12" s="190"/>
-      <c r="D12" s="175" t="s">
-        <v>85</v>
-      </c>
-      <c r="E12" s="175"/>
-      <c r="F12" s="175"/>
-      <c r="G12" s="175"/>
+      <c r="A12" s="234" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="235"/>
+      <c r="C12" s="236"/>
+      <c r="D12" s="221" t="s">
+        <v>84</v>
+      </c>
+      <c r="E12" s="221"/>
+      <c r="F12" s="221"/>
+      <c r="G12" s="221"/>
       <c r="H12" s="67">
         <f>D26+E39</f>
         <v>0</v>
       </c>
       <c r="I12" s="24"/>
-      <c r="J12" s="251" t="s">
-        <v>137</v>
-      </c>
-      <c r="K12" s="251"/>
-      <c r="L12" s="251"/>
+      <c r="J12" s="185" t="s">
+        <v>136</v>
+      </c>
+      <c r="K12" s="185"/>
+      <c r="L12" s="185"/>
       <c r="M12" s="140"/>
       <c r="N12" s="24"/>
       <c r="O12" s="24"/>
@@ -5340,45 +5340,45 @@
       <c r="WE12" s="24"/>
     </row>
     <row r="13" spans="1:603" s="24" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="191"/>
-      <c r="B13" s="192"/>
-      <c r="C13" s="193"/>
-      <c r="D13" s="176" t="s">
-        <v>77</v>
-      </c>
-      <c r="E13" s="176"/>
-      <c r="F13" s="176"/>
-      <c r="G13" s="176"/>
+      <c r="A13" s="237"/>
+      <c r="B13" s="238"/>
+      <c r="C13" s="239"/>
+      <c r="D13" s="222" t="s">
+        <v>76</v>
+      </c>
+      <c r="E13" s="222"/>
+      <c r="F13" s="222"/>
+      <c r="G13" s="222"/>
       <c r="H13" s="68">
         <f>U26</f>
         <v>0</v>
       </c>
-      <c r="J13" s="251" t="s">
-        <v>139</v>
-      </c>
-      <c r="K13" s="251"/>
-      <c r="L13" s="251"/>
+      <c r="J13" s="185" t="s">
+        <v>138</v>
+      </c>
+      <c r="K13" s="185"/>
+      <c r="L13" s="185"/>
       <c r="M13" s="140"/>
     </row>
     <row r="14" spans="1:603" s="24" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="194"/>
-      <c r="B14" s="195"/>
-      <c r="C14" s="196"/>
-      <c r="D14" s="177" t="s">
+      <c r="A14" s="240"/>
+      <c r="B14" s="241"/>
+      <c r="C14" s="242"/>
+      <c r="D14" s="223" t="s">
         <v>3</v>
       </c>
-      <c r="E14" s="177"/>
-      <c r="F14" s="177"/>
-      <c r="G14" s="177"/>
+      <c r="E14" s="223"/>
+      <c r="F14" s="223"/>
+      <c r="G14" s="223"/>
       <c r="H14" s="69">
         <f>H12+H13</f>
         <v>0</v>
       </c>
-      <c r="J14" s="252" t="s">
-        <v>138</v>
-      </c>
-      <c r="K14" s="253"/>
-      <c r="L14" s="254"/>
+      <c r="J14" s="186" t="s">
+        <v>137</v>
+      </c>
+      <c r="K14" s="187"/>
+      <c r="L14" s="188"/>
       <c r="M14" s="140"/>
     </row>
     <row r="15" spans="1:603" s="25" customFormat="1" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -5988,15 +5988,15 @@
     </row>
     <row r="16" spans="1:603" s="11" customFormat="1" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B16" s="28"/>
       <c r="C16" s="28"/>
       <c r="D16" s="22" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F16" s="58" t="s">
         <v>3</v>
@@ -6589,11 +6589,11 @@
       <c r="WE16" s="24"/>
     </row>
     <row r="17" spans="1:603" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="151" t="s">
-        <v>63</v>
-      </c>
-      <c r="B17" s="152"/>
-      <c r="C17" s="152"/>
+      <c r="A17" s="257" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17" s="258"/>
+      <c r="C17" s="258"/>
       <c r="D17" s="70">
         <f>D29+E41-D32-E43</f>
         <v>0</v>
@@ -6607,22 +6607,22 @@
         <v>0</v>
       </c>
       <c r="G17" s="24"/>
-      <c r="H17" s="181" t="s">
-        <v>66</v>
-      </c>
-      <c r="I17" s="181"/>
-      <c r="J17" s="181"/>
-      <c r="K17" s="181"/>
-      <c r="L17" s="182" t="s">
-        <v>83</v>
-      </c>
-      <c r="M17" s="183"/>
-      <c r="N17" s="184"/>
-      <c r="O17" s="185" t="s">
-        <v>73</v>
-      </c>
-      <c r="P17" s="186"/>
-      <c r="Q17" s="187"/>
+      <c r="H17" s="227" t="s">
+        <v>65</v>
+      </c>
+      <c r="I17" s="227"/>
+      <c r="J17" s="227"/>
+      <c r="K17" s="227"/>
+      <c r="L17" s="228" t="s">
+        <v>82</v>
+      </c>
+      <c r="M17" s="229"/>
+      <c r="N17" s="230"/>
+      <c r="O17" s="231" t="s">
+        <v>72</v>
+      </c>
+      <c r="P17" s="232"/>
+      <c r="Q17" s="233"/>
       <c r="R17" s="55" t="s">
         <v>3</v>
       </c>
@@ -7202,11 +7202,11 @@
       <c r="WE17" s="24"/>
     </row>
     <row r="18" spans="1:603" s="11" customFormat="1" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="151" t="s">
-        <v>64</v>
-      </c>
-      <c r="B18" s="152"/>
-      <c r="C18" s="152"/>
+      <c r="A18" s="257" t="s">
+        <v>63</v>
+      </c>
+      <c r="B18" s="258"/>
+      <c r="C18" s="258"/>
       <c r="D18" s="72">
         <f>D32+E43</f>
         <v>0</v>
@@ -7220,10 +7220,10 @@
         <v>0</v>
       </c>
       <c r="G18" s="24"/>
-      <c r="H18" s="181"/>
-      <c r="I18" s="181"/>
-      <c r="J18" s="181"/>
-      <c r="K18" s="181"/>
+      <c r="H18" s="227"/>
+      <c r="I18" s="227"/>
+      <c r="J18" s="227"/>
+      <c r="K18" s="227"/>
       <c r="L18" s="56"/>
       <c r="M18" s="57"/>
       <c r="N18" s="57"/>
@@ -7810,11 +7810,11 @@
       <c r="WE18" s="24"/>
     </row>
     <row r="19" spans="1:603" s="11" customFormat="1" ht="13.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="151" t="s">
-        <v>65</v>
-      </c>
-      <c r="B19" s="152"/>
-      <c r="C19" s="152"/>
+      <c r="A19" s="257" t="s">
+        <v>64</v>
+      </c>
+      <c r="B19" s="258"/>
+      <c r="C19" s="258"/>
       <c r="D19" s="51"/>
       <c r="E19" s="59"/>
       <c r="F19" s="71">
@@ -8409,11 +8409,11 @@
       <c r="WE19" s="24"/>
     </row>
     <row r="20" spans="1:603" s="11" customFormat="1" ht="13.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="197" t="s">
-        <v>114</v>
-      </c>
-      <c r="B20" s="198"/>
-      <c r="C20" s="198"/>
+      <c r="A20" s="243" t="s">
+        <v>113</v>
+      </c>
+      <c r="B20" s="244"/>
+      <c r="C20" s="244"/>
       <c r="D20" s="74">
         <f>H12-D29-E41</f>
         <v>0</v>
@@ -9617,46 +9617,46 @@
       <c r="E22" s="37"/>
     </row>
     <row r="23" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="164" t="s">
+      <c r="A23" s="270" t="s">
         <v>1</v>
       </c>
-      <c r="B23" s="160" t="s">
-        <v>86</v>
-      </c>
-      <c r="C23" s="161"/>
-      <c r="D23" s="162"/>
-      <c r="E23" s="271" t="s">
+      <c r="B23" s="266" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" s="267"/>
+      <c r="D23" s="268"/>
+      <c r="E23" s="163" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="272"/>
-      <c r="G23" s="272"/>
-      <c r="H23" s="272"/>
-      <c r="I23" s="272"/>
-      <c r="J23" s="272"/>
-      <c r="K23" s="272"/>
-      <c r="L23" s="272"/>
-      <c r="M23" s="272"/>
-      <c r="N23" s="272"/>
-      <c r="O23" s="272"/>
-      <c r="P23" s="272"/>
-      <c r="Q23" s="272"/>
-      <c r="R23" s="272"/>
-      <c r="S23" s="272"/>
-      <c r="T23" s="272"/>
-      <c r="U23" s="265" t="s">
-        <v>82</v>
+      <c r="F23" s="164"/>
+      <c r="G23" s="164"/>
+      <c r="H23" s="164"/>
+      <c r="I23" s="164"/>
+      <c r="J23" s="164"/>
+      <c r="K23" s="164"/>
+      <c r="L23" s="164"/>
+      <c r="M23" s="164"/>
+      <c r="N23" s="164"/>
+      <c r="O23" s="164"/>
+      <c r="P23" s="164"/>
+      <c r="Q23" s="164"/>
+      <c r="R23" s="164"/>
+      <c r="S23" s="164"/>
+      <c r="T23" s="164"/>
+      <c r="U23" s="151" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:603" ht="66.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="165"/>
+      <c r="A24" s="271"/>
       <c r="B24" s="100" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="C24" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="D24" s="158" t="s">
-        <v>81</v>
+      <c r="D24" s="264" t="s">
+        <v>80</v>
       </c>
       <c r="E24" s="20" t="s">
         <v>20</v>
@@ -9668,490 +9668,490 @@
         <v>22</v>
       </c>
       <c r="H24" s="46" t="s">
-        <v>24</v>
+        <v>140</v>
       </c>
       <c r="I24" s="46" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J24" s="46" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="K24" s="46" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="L24" s="46" t="s">
-        <v>32</v>
-      </c>
-      <c r="M24" s="201" t="s">
-        <v>34</v>
-      </c>
-      <c r="N24" s="201"/>
-      <c r="O24" s="201"/>
-      <c r="P24" s="201" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q24" s="201"/>
-      <c r="R24" s="201"/>
-      <c r="S24" s="230" t="s">
-        <v>38</v>
-      </c>
-      <c r="T24" s="230"/>
-      <c r="U24" s="266"/>
+        <v>31</v>
+      </c>
+      <c r="M24" s="189" t="s">
+        <v>33</v>
+      </c>
+      <c r="N24" s="189"/>
+      <c r="O24" s="189"/>
+      <c r="P24" s="189" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q24" s="189"/>
+      <c r="R24" s="189"/>
+      <c r="S24" s="191" t="s">
+        <v>37</v>
+      </c>
+      <c r="T24" s="191"/>
+      <c r="U24" s="152"/>
     </row>
     <row r="25" spans="1:603" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="166"/>
+      <c r="A25" s="272"/>
       <c r="B25" s="52" t="s">
         <v>18</v>
       </c>
       <c r="C25" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="D25" s="159"/>
+      <c r="D25" s="265"/>
       <c r="E25" s="52" t="s">
         <v>23</v>
       </c>
       <c r="F25" s="53" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G25" s="53" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H25" s="53" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I25" s="53" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J25" s="53" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K25" s="53" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="L25" s="53" t="s">
-        <v>37</v>
-      </c>
-      <c r="M25" s="202" t="s">
-        <v>39</v>
-      </c>
-      <c r="N25" s="202"/>
-      <c r="O25" s="202"/>
-      <c r="P25" s="202" t="s">
+        <v>36</v>
+      </c>
+      <c r="M25" s="190" t="s">
+        <v>38</v>
+      </c>
+      <c r="N25" s="190"/>
+      <c r="O25" s="190"/>
+      <c r="P25" s="190" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q25" s="190"/>
+      <c r="R25" s="190"/>
+      <c r="S25" s="190" t="s">
         <v>78</v>
       </c>
-      <c r="Q25" s="202"/>
-      <c r="R25" s="202"/>
-      <c r="S25" s="202" t="s">
-        <v>79</v>
-      </c>
-      <c r="T25" s="202"/>
-      <c r="U25" s="267"/>
+      <c r="T25" s="190"/>
+      <c r="U25" s="153"/>
     </row>
     <row r="26" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="245" t="s">
-        <v>76</v>
-      </c>
-      <c r="B26" s="153"/>
-      <c r="C26" s="239"/>
-      <c r="D26" s="234">
+      <c r="A26" s="178" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="259"/>
+      <c r="C26" s="172"/>
+      <c r="D26" s="167">
         <f>B26+C26</f>
         <v>0</v>
       </c>
-      <c r="E26" s="248"/>
-      <c r="F26" s="219"/>
-      <c r="G26" s="219"/>
-      <c r="H26" s="219"/>
-      <c r="I26" s="219"/>
-      <c r="J26" s="219"/>
-      <c r="K26" s="219"/>
-      <c r="L26" s="219"/>
-      <c r="M26" s="226" t="s">
-        <v>40</v>
-      </c>
-      <c r="N26" s="227"/>
+      <c r="E26" s="181"/>
+      <c r="F26" s="154"/>
+      <c r="G26" s="154"/>
+      <c r="H26" s="154"/>
+      <c r="I26" s="154"/>
+      <c r="J26" s="154"/>
+      <c r="K26" s="154"/>
+      <c r="L26" s="154"/>
+      <c r="M26" s="194" t="s">
+        <v>39</v>
+      </c>
+      <c r="N26" s="195"/>
       <c r="O26" s="54"/>
-      <c r="P26" s="226" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q26" s="227"/>
+      <c r="P26" s="194" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q26" s="195"/>
       <c r="R26" s="54"/>
-      <c r="S26" s="231">
+      <c r="S26" s="192">
         <f>M40+M41+M42+N40+N41+N42+O40+O41</f>
         <v>0</v>
       </c>
-      <c r="T26" s="231"/>
-      <c r="U26" s="268">
+      <c r="T26" s="192"/>
+      <c r="U26" s="156">
         <f>E26+F26+G26+H26+I26+J26+K26+L26+O26+O27+O28+R26+R27+R28+S26</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="246"/>
-      <c r="B27" s="154"/>
-      <c r="C27" s="240"/>
-      <c r="D27" s="235"/>
-      <c r="E27" s="249"/>
-      <c r="F27" s="203"/>
-      <c r="G27" s="203"/>
-      <c r="H27" s="203"/>
-      <c r="I27" s="203"/>
-      <c r="J27" s="203"/>
-      <c r="K27" s="203"/>
-      <c r="L27" s="203"/>
-      <c r="M27" s="199" t="s">
+      <c r="A27" s="179"/>
+      <c r="B27" s="260"/>
+      <c r="C27" s="173"/>
+      <c r="D27" s="168"/>
+      <c r="E27" s="182"/>
+      <c r="F27" s="155"/>
+      <c r="G27" s="155"/>
+      <c r="H27" s="155"/>
+      <c r="I27" s="155"/>
+      <c r="J27" s="155"/>
+      <c r="K27" s="155"/>
+      <c r="L27" s="155"/>
+      <c r="M27" s="159" t="s">
         <v>13</v>
       </c>
-      <c r="N27" s="200"/>
+      <c r="N27" s="160"/>
       <c r="O27" s="49"/>
-      <c r="P27" s="199" t="s">
+      <c r="P27" s="159" t="s">
         <v>13</v>
       </c>
-      <c r="Q27" s="200"/>
+      <c r="Q27" s="160"/>
       <c r="R27" s="49"/>
-      <c r="S27" s="223"/>
-      <c r="T27" s="223"/>
-      <c r="U27" s="269"/>
+      <c r="S27" s="193"/>
+      <c r="T27" s="193"/>
+      <c r="U27" s="157"/>
     </row>
     <row r="28" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="246"/>
-      <c r="B28" s="155"/>
-      <c r="C28" s="241"/>
-      <c r="D28" s="236"/>
-      <c r="E28" s="249"/>
-      <c r="F28" s="203"/>
-      <c r="G28" s="203"/>
-      <c r="H28" s="203"/>
-      <c r="I28" s="203"/>
-      <c r="J28" s="203"/>
-      <c r="K28" s="203"/>
-      <c r="L28" s="203"/>
-      <c r="M28" s="199" t="s">
-        <v>49</v>
-      </c>
-      <c r="N28" s="200"/>
+      <c r="A28" s="179"/>
+      <c r="B28" s="261"/>
+      <c r="C28" s="174"/>
+      <c r="D28" s="169"/>
+      <c r="E28" s="182"/>
+      <c r="F28" s="155"/>
+      <c r="G28" s="155"/>
+      <c r="H28" s="155"/>
+      <c r="I28" s="155"/>
+      <c r="J28" s="155"/>
+      <c r="K28" s="155"/>
+      <c r="L28" s="155"/>
+      <c r="M28" s="159" t="s">
+        <v>48</v>
+      </c>
+      <c r="N28" s="160"/>
       <c r="O28" s="49"/>
-      <c r="P28" s="199" t="s">
-        <v>49</v>
-      </c>
-      <c r="Q28" s="200"/>
+      <c r="P28" s="159" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q28" s="160"/>
       <c r="R28" s="49"/>
-      <c r="S28" s="223"/>
-      <c r="T28" s="223"/>
-      <c r="U28" s="269"/>
+      <c r="S28" s="193"/>
+      <c r="T28" s="193"/>
+      <c r="U28" s="157"/>
     </row>
     <row r="29" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="246" t="s">
+      <c r="A29" s="179" t="s">
         <v>4</v>
       </c>
-      <c r="B29" s="156"/>
-      <c r="C29" s="242"/>
-      <c r="D29" s="237">
+      <c r="B29" s="262"/>
+      <c r="C29" s="175"/>
+      <c r="D29" s="170">
         <f>B29+C29</f>
         <v>0</v>
       </c>
-      <c r="E29" s="249"/>
-      <c r="F29" s="203"/>
-      <c r="G29" s="203"/>
-      <c r="H29" s="203"/>
-      <c r="I29" s="203"/>
-      <c r="J29" s="203"/>
-      <c r="K29" s="203"/>
-      <c r="L29" s="203"/>
-      <c r="M29" s="199" t="s">
-        <v>40</v>
-      </c>
-      <c r="N29" s="200"/>
+      <c r="E29" s="182"/>
+      <c r="F29" s="155"/>
+      <c r="G29" s="155"/>
+      <c r="H29" s="155"/>
+      <c r="I29" s="155"/>
+      <c r="J29" s="155"/>
+      <c r="K29" s="155"/>
+      <c r="L29" s="155"/>
+      <c r="M29" s="159" t="s">
+        <v>39</v>
+      </c>
+      <c r="N29" s="160"/>
       <c r="O29" s="49"/>
-      <c r="P29" s="199" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q29" s="200"/>
+      <c r="P29" s="159" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q29" s="160"/>
       <c r="R29" s="49"/>
-      <c r="S29" s="223">
+      <c r="S29" s="193">
         <f>P40+P41+P42+Q40+Q41+Q42+R40+R41</f>
         <v>0</v>
       </c>
-      <c r="T29" s="223"/>
-      <c r="U29" s="269">
+      <c r="T29" s="193"/>
+      <c r="U29" s="157">
         <f>E29+F29+G29+H29+I29+J29+K29+L29+O29+O30+O31+R29+R30+R31+S29</f>
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="246"/>
-      <c r="B30" s="154"/>
-      <c r="C30" s="240"/>
-      <c r="D30" s="235"/>
-      <c r="E30" s="249"/>
-      <c r="F30" s="203"/>
-      <c r="G30" s="203"/>
-      <c r="H30" s="203"/>
-      <c r="I30" s="203"/>
-      <c r="J30" s="203"/>
-      <c r="K30" s="203"/>
-      <c r="L30" s="203"/>
-      <c r="M30" s="199" t="s">
+      <c r="A30" s="179"/>
+      <c r="B30" s="260"/>
+      <c r="C30" s="173"/>
+      <c r="D30" s="168"/>
+      <c r="E30" s="182"/>
+      <c r="F30" s="155"/>
+      <c r="G30" s="155"/>
+      <c r="H30" s="155"/>
+      <c r="I30" s="155"/>
+      <c r="J30" s="155"/>
+      <c r="K30" s="155"/>
+      <c r="L30" s="155"/>
+      <c r="M30" s="159" t="s">
         <v>13</v>
       </c>
-      <c r="N30" s="200"/>
+      <c r="N30" s="160"/>
       <c r="O30" s="49"/>
-      <c r="P30" s="199" t="s">
+      <c r="P30" s="159" t="s">
         <v>13</v>
       </c>
-      <c r="Q30" s="200"/>
+      <c r="Q30" s="160"/>
       <c r="R30" s="49"/>
-      <c r="S30" s="223"/>
-      <c r="T30" s="223"/>
-      <c r="U30" s="269"/>
+      <c r="S30" s="193"/>
+      <c r="T30" s="193"/>
+      <c r="U30" s="157"/>
     </row>
     <row r="31" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="246"/>
-      <c r="B31" s="155"/>
-      <c r="C31" s="241"/>
-      <c r="D31" s="236"/>
-      <c r="E31" s="249"/>
-      <c r="F31" s="203"/>
-      <c r="G31" s="203"/>
-      <c r="H31" s="203"/>
-      <c r="I31" s="203"/>
-      <c r="J31" s="203"/>
-      <c r="K31" s="203"/>
-      <c r="L31" s="203"/>
-      <c r="M31" s="199" t="s">
-        <v>49</v>
-      </c>
-      <c r="N31" s="200"/>
+      <c r="A31" s="179"/>
+      <c r="B31" s="261"/>
+      <c r="C31" s="174"/>
+      <c r="D31" s="169"/>
+      <c r="E31" s="182"/>
+      <c r="F31" s="155"/>
+      <c r="G31" s="155"/>
+      <c r="H31" s="155"/>
+      <c r="I31" s="155"/>
+      <c r="J31" s="155"/>
+      <c r="K31" s="155"/>
+      <c r="L31" s="155"/>
+      <c r="M31" s="159" t="s">
+        <v>48</v>
+      </c>
+      <c r="N31" s="160"/>
       <c r="O31" s="49"/>
-      <c r="P31" s="199" t="s">
-        <v>49</v>
-      </c>
-      <c r="Q31" s="200"/>
+      <c r="P31" s="159" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q31" s="160"/>
       <c r="R31" s="49"/>
-      <c r="S31" s="223"/>
-      <c r="T31" s="223"/>
-      <c r="U31" s="269"/>
+      <c r="S31" s="193"/>
+      <c r="T31" s="193"/>
+      <c r="U31" s="157"/>
     </row>
     <row r="32" spans="1:603" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="246" t="s">
+      <c r="A32" s="179" t="s">
         <v>5</v>
       </c>
-      <c r="B32" s="156"/>
-      <c r="C32" s="242"/>
-      <c r="D32" s="237">
+      <c r="B32" s="262"/>
+      <c r="C32" s="175"/>
+      <c r="D32" s="170">
         <f>B32+C32</f>
         <v>0</v>
       </c>
-      <c r="E32" s="249"/>
-      <c r="F32" s="203"/>
-      <c r="G32" s="203"/>
-      <c r="H32" s="203"/>
-      <c r="I32" s="203"/>
-      <c r="J32" s="203"/>
-      <c r="K32" s="203"/>
-      <c r="L32" s="203"/>
-      <c r="M32" s="199" t="s">
-        <v>40</v>
-      </c>
-      <c r="N32" s="200"/>
+      <c r="E32" s="182"/>
+      <c r="F32" s="155"/>
+      <c r="G32" s="155"/>
+      <c r="H32" s="155"/>
+      <c r="I32" s="155"/>
+      <c r="J32" s="155"/>
+      <c r="K32" s="155"/>
+      <c r="L32" s="155"/>
+      <c r="M32" s="159" t="s">
+        <v>39</v>
+      </c>
+      <c r="N32" s="160"/>
       <c r="O32" s="49"/>
-      <c r="P32" s="199" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q32" s="200"/>
+      <c r="P32" s="159" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q32" s="160"/>
       <c r="R32" s="49"/>
-      <c r="S32" s="223">
+      <c r="S32" s="193">
         <f>S40+S41+S42+T40+T41+T42+U40+U41</f>
         <v>0</v>
       </c>
-      <c r="T32" s="223"/>
-      <c r="U32" s="269">
+      <c r="T32" s="193"/>
+      <c r="U32" s="157">
         <f>E32+F32+G32+H32+I32+J32+K32+L32+O32+O33+O34+R32+R33+R34+S32</f>
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:24" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="246"/>
-      <c r="B33" s="154"/>
-      <c r="C33" s="240"/>
-      <c r="D33" s="235"/>
-      <c r="E33" s="249"/>
-      <c r="F33" s="203"/>
-      <c r="G33" s="203"/>
-      <c r="H33" s="203"/>
-      <c r="I33" s="203"/>
-      <c r="J33" s="203"/>
-      <c r="K33" s="203"/>
-      <c r="L33" s="203"/>
-      <c r="M33" s="199" t="s">
+      <c r="A33" s="179"/>
+      <c r="B33" s="260"/>
+      <c r="C33" s="173"/>
+      <c r="D33" s="168"/>
+      <c r="E33" s="182"/>
+      <c r="F33" s="155"/>
+      <c r="G33" s="155"/>
+      <c r="H33" s="155"/>
+      <c r="I33" s="155"/>
+      <c r="J33" s="155"/>
+      <c r="K33" s="155"/>
+      <c r="L33" s="155"/>
+      <c r="M33" s="159" t="s">
         <v>13</v>
       </c>
-      <c r="N33" s="200"/>
+      <c r="N33" s="160"/>
       <c r="O33" s="49"/>
-      <c r="P33" s="199" t="s">
+      <c r="P33" s="159" t="s">
         <v>13</v>
       </c>
-      <c r="Q33" s="200"/>
+      <c r="Q33" s="160"/>
       <c r="R33" s="49"/>
-      <c r="S33" s="223"/>
-      <c r="T33" s="223"/>
-      <c r="U33" s="269"/>
+      <c r="S33" s="193"/>
+      <c r="T33" s="193"/>
+      <c r="U33" s="157"/>
     </row>
     <row r="34" spans="1:24" ht="13.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="247"/>
-      <c r="B34" s="157"/>
-      <c r="C34" s="243"/>
-      <c r="D34" s="238"/>
-      <c r="E34" s="250"/>
-      <c r="F34" s="204"/>
-      <c r="G34" s="204"/>
-      <c r="H34" s="204"/>
-      <c r="I34" s="204"/>
-      <c r="J34" s="204"/>
-      <c r="K34" s="204"/>
-      <c r="L34" s="204"/>
-      <c r="M34" s="228" t="s">
-        <v>49</v>
-      </c>
-      <c r="N34" s="229"/>
+      <c r="A34" s="180"/>
+      <c r="B34" s="263"/>
+      <c r="C34" s="176"/>
+      <c r="D34" s="171"/>
+      <c r="E34" s="183"/>
+      <c r="F34" s="184"/>
+      <c r="G34" s="184"/>
+      <c r="H34" s="184"/>
+      <c r="I34" s="184"/>
+      <c r="J34" s="184"/>
+      <c r="K34" s="184"/>
+      <c r="L34" s="184"/>
+      <c r="M34" s="161" t="s">
+        <v>48</v>
+      </c>
+      <c r="N34" s="162"/>
       <c r="O34" s="50"/>
-      <c r="P34" s="228" t="s">
-        <v>49</v>
-      </c>
-      <c r="Q34" s="229"/>
+      <c r="P34" s="161" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q34" s="162"/>
       <c r="R34" s="50"/>
-      <c r="S34" s="224"/>
-      <c r="T34" s="224"/>
-      <c r="U34" s="270"/>
+      <c r="S34" s="218"/>
+      <c r="T34" s="218"/>
+      <c r="U34" s="158"/>
     </row>
     <row r="35" spans="1:24" ht="4.6500000000000004" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="36" spans="1:24" ht="13.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
     </row>
     <row r="37" spans="1:24" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="178" t="s">
-        <v>45</v>
-      </c>
-      <c r="B37" s="179"/>
-      <c r="C37" s="179"/>
-      <c r="D37" s="179"/>
-      <c r="E37" s="180"/>
+      <c r="A37" s="224" t="s">
+        <v>44</v>
+      </c>
+      <c r="B37" s="225"/>
+      <c r="C37" s="225"/>
+      <c r="D37" s="225"/>
+      <c r="E37" s="226"/>
       <c r="F37" s="18"/>
       <c r="G37" s="18"/>
       <c r="H37" s="18"/>
-      <c r="J37" s="207" t="s">
-        <v>50</v>
-      </c>
-      <c r="K37" s="208"/>
-      <c r="L37" s="208"/>
-      <c r="M37" s="208"/>
-      <c r="N37" s="208"/>
-      <c r="O37" s="208"/>
-      <c r="P37" s="208"/>
-      <c r="Q37" s="208"/>
-      <c r="R37" s="208"/>
-      <c r="S37" s="208"/>
-      <c r="T37" s="208"/>
-      <c r="U37" s="209"/>
+      <c r="J37" s="203" t="s">
+        <v>49</v>
+      </c>
+      <c r="K37" s="204"/>
+      <c r="L37" s="204"/>
+      <c r="M37" s="204"/>
+      <c r="N37" s="204"/>
+      <c r="O37" s="204"/>
+      <c r="P37" s="204"/>
+      <c r="Q37" s="204"/>
+      <c r="R37" s="204"/>
+      <c r="S37" s="204"/>
+      <c r="T37" s="204"/>
+      <c r="U37" s="205"/>
     </row>
     <row r="38" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="14"/>
       <c r="B38" s="44" t="s">
+        <v>45</v>
+      </c>
+      <c r="C38" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="C38" s="44" t="s">
+      <c r="D38" s="44" t="s">
         <v>47</v>
-      </c>
-      <c r="D38" s="44" t="s">
-        <v>48</v>
       </c>
       <c r="E38" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="J38" s="210" t="s">
+      <c r="J38" s="206" t="s">
         <v>2</v>
       </c>
-      <c r="K38" s="211"/>
-      <c r="L38" s="212"/>
-      <c r="M38" s="205" t="s">
+      <c r="K38" s="207"/>
+      <c r="L38" s="208"/>
+      <c r="M38" s="201" t="s">
         <v>6</v>
       </c>
-      <c r="N38" s="205"/>
-      <c r="O38" s="205"/>
-      <c r="P38" s="205" t="s">
+      <c r="N38" s="201"/>
+      <c r="O38" s="201"/>
+      <c r="P38" s="201" t="s">
         <v>4</v>
       </c>
-      <c r="Q38" s="205"/>
-      <c r="R38" s="205"/>
-      <c r="S38" s="205" t="s">
+      <c r="Q38" s="201"/>
+      <c r="R38" s="201"/>
+      <c r="S38" s="201" t="s">
         <v>5</v>
       </c>
-      <c r="T38" s="205"/>
-      <c r="U38" s="206"/>
+      <c r="T38" s="201"/>
+      <c r="U38" s="202"/>
     </row>
     <row r="39" spans="1:24" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="169" t="s">
-        <v>42</v>
-      </c>
-      <c r="B39" s="172"/>
-      <c r="C39" s="172"/>
-      <c r="D39" s="172"/>
-      <c r="E39" s="171">
+      <c r="A39" s="246" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="196"/>
+      <c r="C39" s="196"/>
+      <c r="D39" s="196"/>
+      <c r="E39" s="198">
         <f>B39+C39+D39</f>
         <v>0</v>
       </c>
-      <c r="F39" s="168"/>
-      <c r="G39" s="168"/>
-      <c r="H39" s="167"/>
-      <c r="J39" s="213"/>
-      <c r="K39" s="214"/>
-      <c r="L39" s="215"/>
+      <c r="F39" s="200"/>
+      <c r="G39" s="200"/>
+      <c r="H39" s="245"/>
+      <c r="J39" s="209"/>
+      <c r="K39" s="210"/>
+      <c r="L39" s="211"/>
       <c r="M39" s="44" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="N39" s="44" t="s">
         <v>7</v>
       </c>
       <c r="O39" s="44" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="P39" s="44" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="Q39" s="44" t="s">
         <v>7</v>
       </c>
       <c r="R39" s="44" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="S39" s="44" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="T39" s="44" t="s">
         <v>7</v>
       </c>
       <c r="U39" s="45" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="40" spans="1:24" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="169"/>
-      <c r="B40" s="174"/>
-      <c r="C40" s="174"/>
-      <c r="D40" s="174"/>
-      <c r="E40" s="171"/>
-      <c r="F40" s="168"/>
-      <c r="G40" s="168"/>
-      <c r="H40" s="167"/>
-      <c r="J40" s="216" t="s">
-        <v>53</v>
-      </c>
-      <c r="K40" s="217"/>
-      <c r="L40" s="218"/>
+      <c r="A40" s="246"/>
+      <c r="B40" s="220"/>
+      <c r="C40" s="220"/>
+      <c r="D40" s="220"/>
+      <c r="E40" s="198"/>
+      <c r="F40" s="200"/>
+      <c r="G40" s="200"/>
+      <c r="H40" s="245"/>
+      <c r="J40" s="212" t="s">
+        <v>52</v>
+      </c>
+      <c r="K40" s="213"/>
+      <c r="L40" s="214"/>
       <c r="M40" s="38"/>
       <c r="N40" s="38"/>
       <c r="O40" s="38"/>
@@ -10163,24 +10163,24 @@
       <c r="U40" s="39"/>
     </row>
     <row r="41" spans="1:24" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="169" t="s">
-        <v>43</v>
-      </c>
-      <c r="B41" s="172"/>
-      <c r="C41" s="172"/>
-      <c r="D41" s="172"/>
-      <c r="E41" s="171">
+      <c r="A41" s="246" t="s">
+        <v>42</v>
+      </c>
+      <c r="B41" s="196"/>
+      <c r="C41" s="196"/>
+      <c r="D41" s="196"/>
+      <c r="E41" s="198">
         <f>B41+C41+D41</f>
         <v>0</v>
       </c>
-      <c r="F41" s="168"/>
-      <c r="G41" s="168"/>
-      <c r="H41" s="167"/>
-      <c r="J41" s="216" t="s">
-        <v>54</v>
-      </c>
-      <c r="K41" s="217"/>
-      <c r="L41" s="218"/>
+      <c r="F41" s="200"/>
+      <c r="G41" s="200"/>
+      <c r="H41" s="245"/>
+      <c r="J41" s="212" t="s">
+        <v>53</v>
+      </c>
+      <c r="K41" s="213"/>
+      <c r="L41" s="214"/>
       <c r="M41" s="38"/>
       <c r="N41" s="38"/>
       <c r="O41" s="38"/>
@@ -10192,19 +10192,19 @@
       <c r="U41" s="39"/>
     </row>
     <row r="42" spans="1:24" ht="13.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="169"/>
-      <c r="B42" s="174"/>
-      <c r="C42" s="174"/>
-      <c r="D42" s="174"/>
-      <c r="E42" s="171"/>
-      <c r="F42" s="168"/>
-      <c r="G42" s="168"/>
-      <c r="H42" s="167"/>
-      <c r="J42" s="220" t="s">
-        <v>55</v>
-      </c>
-      <c r="K42" s="221"/>
-      <c r="L42" s="222"/>
+      <c r="A42" s="246"/>
+      <c r="B42" s="220"/>
+      <c r="C42" s="220"/>
+      <c r="D42" s="220"/>
+      <c r="E42" s="198"/>
+      <c r="F42" s="200"/>
+      <c r="G42" s="200"/>
+      <c r="H42" s="245"/>
+      <c r="J42" s="215" t="s">
+        <v>54</v>
+      </c>
+      <c r="K42" s="216"/>
+      <c r="L42" s="217"/>
       <c r="M42" s="40"/>
       <c r="N42" s="40"/>
       <c r="O42" s="41"/>
@@ -10216,21 +10216,21 @@
       <c r="U42" s="42"/>
     </row>
     <row r="43" spans="1:24" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="169" t="s">
-        <v>44</v>
-      </c>
-      <c r="B43" s="172"/>
-      <c r="C43" s="172"/>
-      <c r="D43" s="172"/>
-      <c r="E43" s="171">
+      <c r="A43" s="246" t="s">
+        <v>43</v>
+      </c>
+      <c r="B43" s="196"/>
+      <c r="C43" s="196"/>
+      <c r="D43" s="196"/>
+      <c r="E43" s="198">
         <f>B43+C43+D43</f>
         <v>0</v>
       </c>
-      <c r="F43" s="168"/>
-      <c r="G43" s="168"/>
-      <c r="H43" s="167"/>
+      <c r="F43" s="200"/>
+      <c r="G43" s="200"/>
+      <c r="H43" s="245"/>
       <c r="J43" s="15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K43" s="16"/>
       <c r="L43" s="16"/>
@@ -10248,123 +10248,239 @@
       <c r="X43" s="16"/>
     </row>
     <row r="44" spans="1:24" ht="13.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="170"/>
-      <c r="B44" s="173"/>
-      <c r="C44" s="173"/>
-      <c r="D44" s="173"/>
-      <c r="E44" s="225"/>
-      <c r="F44" s="168"/>
-      <c r="G44" s="168"/>
-      <c r="H44" s="167"/>
+      <c r="A44" s="273"/>
+      <c r="B44" s="197"/>
+      <c r="C44" s="197"/>
+      <c r="D44" s="197"/>
+      <c r="E44" s="199"/>
+      <c r="F44" s="200"/>
+      <c r="G44" s="200"/>
+      <c r="H44" s="245"/>
     </row>
     <row r="45" spans="1:24" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
-      <c r="F45" s="150" t="s">
-        <v>115</v>
-      </c>
-      <c r="G45" s="150"/>
-      <c r="H45" s="150"/>
+      <c r="F45" s="256" t="s">
+        <v>114</v>
+      </c>
+      <c r="G45" s="256"/>
+      <c r="H45" s="256"/>
       <c r="L45" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M45" s="16"/>
       <c r="N45" s="16"/>
       <c r="O45" s="16"/>
       <c r="P45" s="16"/>
-      <c r="Q45" s="260"/>
-      <c r="R45" s="260"/>
-      <c r="S45" s="260"/>
-      <c r="T45" s="260"/>
-      <c r="U45" s="260"/>
+      <c r="Q45" s="146"/>
+      <c r="R45" s="146"/>
+      <c r="S45" s="146"/>
+      <c r="T45" s="146"/>
+      <c r="U45" s="146"/>
     </row>
     <row r="46" spans="1:24" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="163"/>
+      <c r="A46" s="269"/>
       <c r="B46" s="48"/>
       <c r="C46" s="48"/>
       <c r="D46" s="48"/>
-      <c r="E46" s="141"/>
-      <c r="F46" s="142"/>
-      <c r="G46" s="142"/>
-      <c r="H46" s="142"/>
-      <c r="I46" s="142"/>
-      <c r="J46" s="143"/>
+      <c r="E46" s="247"/>
+      <c r="F46" s="248"/>
+      <c r="G46" s="248"/>
+      <c r="H46" s="248"/>
+      <c r="I46" s="248"/>
+      <c r="J46" s="249"/>
       <c r="K46" s="16"/>
       <c r="L46" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="M46" s="260"/>
-      <c r="N46" s="260"/>
-      <c r="O46" s="260"/>
-      <c r="P46" s="260"/>
+        <v>57</v>
+      </c>
+      <c r="M46" s="146"/>
+      <c r="N46" s="146"/>
+      <c r="O46" s="146"/>
+      <c r="P46" s="146"/>
       <c r="Q46" s="16"/>
       <c r="R46" s="16"/>
     </row>
     <row r="47" spans="1:24" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="163"/>
+      <c r="A47" s="269"/>
       <c r="B47" s="48"/>
       <c r="C47" s="48"/>
       <c r="D47" s="48"/>
-      <c r="E47" s="144"/>
-      <c r="F47" s="145"/>
-      <c r="G47" s="145"/>
-      <c r="H47" s="145"/>
-      <c r="I47" s="145"/>
-      <c r="J47" s="146"/>
+      <c r="E47" s="250"/>
+      <c r="F47" s="251"/>
+      <c r="G47" s="251"/>
+      <c r="H47" s="251"/>
+      <c r="I47" s="251"/>
+      <c r="J47" s="252"/>
       <c r="K47" s="16"/>
       <c r="L47" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="M47" s="259"/>
-      <c r="N47" s="259"/>
-      <c r="O47" s="259"/>
-      <c r="P47" s="259"/>
+        <v>58</v>
+      </c>
+      <c r="M47" s="145"/>
+      <c r="N47" s="145"/>
+      <c r="O47" s="145"/>
+      <c r="P47" s="145"/>
       <c r="Q47" s="16"/>
       <c r="R47" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="S47" s="258"/>
-      <c r="T47" s="258"/>
+        <v>59</v>
+      </c>
+      <c r="S47" s="144"/>
+      <c r="T47" s="144"/>
     </row>
     <row r="48" spans="1:24" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="167"/>
+      <c r="A48" s="245"/>
       <c r="B48" s="47"/>
       <c r="C48" s="47"/>
       <c r="D48" s="47"/>
-      <c r="E48" s="144"/>
-      <c r="F48" s="145"/>
-      <c r="G48" s="145"/>
-      <c r="H48" s="145"/>
-      <c r="I48" s="145"/>
-      <c r="J48" s="146"/>
+      <c r="E48" s="250"/>
+      <c r="F48" s="251"/>
+      <c r="G48" s="251"/>
+      <c r="H48" s="251"/>
+      <c r="I48" s="251"/>
+      <c r="J48" s="252"/>
       <c r="K48" s="16"/>
       <c r="L48" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="M48" s="233"/>
-      <c r="N48" s="233"/>
-      <c r="O48" s="233"/>
-      <c r="P48" s="233"/>
+        <v>60</v>
+      </c>
+      <c r="M48" s="166"/>
+      <c r="N48" s="166"/>
+      <c r="O48" s="166"/>
+      <c r="P48" s="166"/>
       <c r="Q48" s="16"/>
       <c r="R48" s="16"/>
     </row>
     <row r="49" spans="1:11" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="167"/>
+      <c r="A49" s="245"/>
       <c r="B49" s="47"/>
       <c r="C49" s="47"/>
       <c r="D49" s="47"/>
-      <c r="E49" s="147"/>
-      <c r="F49" s="148"/>
-      <c r="G49" s="148"/>
-      <c r="H49" s="148"/>
-      <c r="I49" s="148"/>
-      <c r="J49" s="149"/>
+      <c r="E49" s="253"/>
+      <c r="F49" s="254"/>
+      <c r="G49" s="254"/>
+      <c r="H49" s="254"/>
+      <c r="I49" s="254"/>
+      <c r="J49" s="255"/>
       <c r="K49" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="140">
+    <mergeCell ref="E46:J49"/>
+    <mergeCell ref="F45:H45"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="B26:B28"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="A48:A49"/>
+    <mergeCell ref="G43:G44"/>
+    <mergeCell ref="H43:H44"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="G39:G40"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="G41:G42"/>
+    <mergeCell ref="H41:H42"/>
+    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="N6:O6"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="D39:D40"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="D41:D42"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="D13:G13"/>
+    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="H17:K18"/>
+    <mergeCell ref="L17:N17"/>
+    <mergeCell ref="O17:Q17"/>
+    <mergeCell ref="A12:C14"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="P27:Q27"/>
+    <mergeCell ref="M24:O24"/>
+    <mergeCell ref="M25:O25"/>
+    <mergeCell ref="P25:R25"/>
+    <mergeCell ref="L32:L34"/>
+    <mergeCell ref="H39:H40"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="S38:U38"/>
+    <mergeCell ref="J37:U37"/>
+    <mergeCell ref="J38:L39"/>
+    <mergeCell ref="J40:L40"/>
+    <mergeCell ref="J41:L41"/>
+    <mergeCell ref="J32:J34"/>
+    <mergeCell ref="G26:G28"/>
+    <mergeCell ref="J26:J28"/>
+    <mergeCell ref="J42:L42"/>
+    <mergeCell ref="M38:O38"/>
+    <mergeCell ref="P38:R38"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="I29:I31"/>
+    <mergeCell ref="I32:I34"/>
+    <mergeCell ref="M27:N27"/>
+    <mergeCell ref="P32:Q32"/>
+    <mergeCell ref="H26:H28"/>
+    <mergeCell ref="H29:H31"/>
+    <mergeCell ref="S29:T31"/>
+    <mergeCell ref="S32:T34"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="D43:D44"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="F29:F31"/>
+    <mergeCell ref="P26:Q26"/>
+    <mergeCell ref="P33:Q33"/>
+    <mergeCell ref="K32:K34"/>
+    <mergeCell ref="F32:F34"/>
+    <mergeCell ref="G29:G31"/>
+    <mergeCell ref="P24:R24"/>
+    <mergeCell ref="S25:T25"/>
+    <mergeCell ref="P34:Q34"/>
+    <mergeCell ref="P30:Q30"/>
+    <mergeCell ref="P31:Q31"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="S24:T24"/>
+    <mergeCell ref="S26:T28"/>
+    <mergeCell ref="M26:N26"/>
+    <mergeCell ref="P28:Q28"/>
+    <mergeCell ref="P29:Q29"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="M48:P48"/>
+    <mergeCell ref="D26:D28"/>
+    <mergeCell ref="D29:D31"/>
+    <mergeCell ref="D32:D34"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="C29:C31"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="A4:U4"/>
+    <mergeCell ref="A2:U2"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="A29:A31"/>
+    <mergeCell ref="A32:A34"/>
+    <mergeCell ref="E26:E28"/>
+    <mergeCell ref="E29:E31"/>
+    <mergeCell ref="E32:E34"/>
+    <mergeCell ref="F26:F28"/>
+    <mergeCell ref="G32:G34"/>
+    <mergeCell ref="J29:J31"/>
+    <mergeCell ref="K29:K31"/>
+    <mergeCell ref="J12:L12"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="J14:L14"/>
     <mergeCell ref="C6:G6"/>
     <mergeCell ref="C7:G7"/>
     <mergeCell ref="C8:G8"/>
@@ -10389,125 +10505,9 @@
     <mergeCell ref="E23:T23"/>
     <mergeCell ref="K26:K28"/>
     <mergeCell ref="M32:N32"/>
-    <mergeCell ref="A1:R1"/>
-    <mergeCell ref="M48:P48"/>
-    <mergeCell ref="D26:D28"/>
-    <mergeCell ref="D29:D31"/>
-    <mergeCell ref="D32:D34"/>
-    <mergeCell ref="C26:C28"/>
-    <mergeCell ref="C29:C31"/>
-    <mergeCell ref="C32:C34"/>
-    <mergeCell ref="A4:U4"/>
-    <mergeCell ref="A2:U2"/>
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="A29:A31"/>
-    <mergeCell ref="A32:A34"/>
-    <mergeCell ref="E26:E28"/>
-    <mergeCell ref="E29:E31"/>
-    <mergeCell ref="E32:E34"/>
-    <mergeCell ref="F26:F28"/>
-    <mergeCell ref="G32:G34"/>
-    <mergeCell ref="J29:J31"/>
-    <mergeCell ref="K29:K31"/>
-    <mergeCell ref="J12:L12"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="P24:R24"/>
-    <mergeCell ref="S25:T25"/>
-    <mergeCell ref="P34:Q34"/>
-    <mergeCell ref="P30:Q30"/>
-    <mergeCell ref="P31:Q31"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="S24:T24"/>
-    <mergeCell ref="S26:T28"/>
-    <mergeCell ref="M26:N26"/>
-    <mergeCell ref="P28:Q28"/>
-    <mergeCell ref="P29:Q29"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="D43:D44"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="H32:H34"/>
-    <mergeCell ref="F29:F31"/>
-    <mergeCell ref="P26:Q26"/>
-    <mergeCell ref="P33:Q33"/>
-    <mergeCell ref="K32:K34"/>
-    <mergeCell ref="F32:F34"/>
-    <mergeCell ref="G29:G31"/>
-    <mergeCell ref="S38:U38"/>
-    <mergeCell ref="J37:U37"/>
-    <mergeCell ref="J38:L39"/>
-    <mergeCell ref="J40:L40"/>
-    <mergeCell ref="J41:L41"/>
-    <mergeCell ref="J32:J34"/>
-    <mergeCell ref="G26:G28"/>
-    <mergeCell ref="J26:J28"/>
-    <mergeCell ref="J42:L42"/>
-    <mergeCell ref="M38:O38"/>
-    <mergeCell ref="P38:R38"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="I29:I31"/>
-    <mergeCell ref="I32:I34"/>
-    <mergeCell ref="M27:N27"/>
-    <mergeCell ref="P32:Q32"/>
-    <mergeCell ref="H26:H28"/>
-    <mergeCell ref="H29:H31"/>
-    <mergeCell ref="S29:T31"/>
-    <mergeCell ref="S32:T34"/>
-    <mergeCell ref="N6:O6"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="D39:D40"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="D41:D42"/>
-    <mergeCell ref="D12:G12"/>
-    <mergeCell ref="D13:G13"/>
-    <mergeCell ref="D14:G14"/>
-    <mergeCell ref="A37:E37"/>
-    <mergeCell ref="H17:K18"/>
-    <mergeCell ref="L17:N17"/>
-    <mergeCell ref="O17:Q17"/>
-    <mergeCell ref="A12:C14"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="P27:Q27"/>
-    <mergeCell ref="M24:O24"/>
-    <mergeCell ref="M25:O25"/>
-    <mergeCell ref="P25:R25"/>
-    <mergeCell ref="L32:L34"/>
-    <mergeCell ref="H39:H40"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="E46:J49"/>
-    <mergeCell ref="F45:H45"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="B26:B28"/>
-    <mergeCell ref="B29:B31"/>
-    <mergeCell ref="B32:B34"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="A46:A47"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="A48:A49"/>
-    <mergeCell ref="G43:G44"/>
-    <mergeCell ref="H43:H44"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="E39:E40"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="G39:G40"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="G41:G42"/>
-    <mergeCell ref="H41:H42"/>
-    <mergeCell ref="B43:B44"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
-  <dataValidations count="5">
+  <dataValidations disablePrompts="1" count="5">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Date Format:_x000a_DD/MM/YYYY" sqref="S47 P9"/>
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E26:L34 M40:U42 B39:D44 L18:N18 R26:R34 O26:O34 C26:C34 B26:B28 B32:B34">
       <formula1>0</formula1>
@@ -11439,23 +11439,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:42" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="274" t="s">
-        <v>88</v>
-      </c>
-      <c r="B1" s="274"/>
-      <c r="C1" s="274"/>
-      <c r="D1" s="274"/>
-      <c r="E1" s="274"/>
-      <c r="F1" s="274"/>
-      <c r="G1" s="274"/>
-      <c r="H1" s="274"/>
-      <c r="I1" s="274"/>
-      <c r="J1" s="274"/>
-      <c r="K1" s="274"/>
-      <c r="L1" s="274"/>
-      <c r="M1" s="274"/>
-      <c r="N1" s="274"/>
-      <c r="O1" s="274"/>
+      <c r="A1" s="275" t="s">
+        <v>87</v>
+      </c>
+      <c r="B1" s="275"/>
+      <c r="C1" s="275"/>
+      <c r="D1" s="275"/>
+      <c r="E1" s="275"/>
+      <c r="F1" s="275"/>
+      <c r="G1" s="275"/>
+      <c r="H1" s="275"/>
+      <c r="I1" s="275"/>
+      <c r="J1" s="275"/>
+      <c r="K1" s="275"/>
+      <c r="L1" s="275"/>
+      <c r="M1" s="275"/>
+      <c r="N1" s="275"/>
+      <c r="O1" s="275"/>
       <c r="P1" s="76"/>
       <c r="Q1" s="76"/>
       <c r="R1" s="76"/>
@@ -11485,23 +11485,23 @@
       <c r="AP1" s="76"/>
     </row>
     <row r="2" spans="1:42" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="274" t="s">
-        <v>89</v>
-      </c>
-      <c r="B2" s="274"/>
-      <c r="C2" s="274"/>
-      <c r="D2" s="274"/>
-      <c r="E2" s="274"/>
-      <c r="F2" s="274"/>
-      <c r="G2" s="274"/>
-      <c r="H2" s="274"/>
-      <c r="I2" s="274"/>
-      <c r="J2" s="274"/>
-      <c r="K2" s="274"/>
-      <c r="L2" s="274"/>
-      <c r="M2" s="274"/>
-      <c r="N2" s="274"/>
-      <c r="O2" s="274"/>
+      <c r="A2" s="275" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="275"/>
+      <c r="C2" s="275"/>
+      <c r="D2" s="275"/>
+      <c r="E2" s="275"/>
+      <c r="F2" s="275"/>
+      <c r="G2" s="275"/>
+      <c r="H2" s="275"/>
+      <c r="I2" s="275"/>
+      <c r="J2" s="275"/>
+      <c r="K2" s="275"/>
+      <c r="L2" s="275"/>
+      <c r="M2" s="275"/>
+      <c r="N2" s="275"/>
+      <c r="O2" s="275"/>
       <c r="P2" s="76"/>
       <c r="Q2" s="76"/>
       <c r="R2" s="76"/>
@@ -11531,23 +11531,23 @@
       <c r="AP2" s="76"/>
     </row>
     <row r="3" spans="1:42" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="274" t="s">
-        <v>90</v>
-      </c>
-      <c r="B3" s="274"/>
-      <c r="C3" s="274"/>
-      <c r="D3" s="274"/>
-      <c r="E3" s="274"/>
-      <c r="F3" s="274"/>
-      <c r="G3" s="274"/>
-      <c r="H3" s="274"/>
-      <c r="I3" s="274"/>
-      <c r="J3" s="274"/>
-      <c r="K3" s="274"/>
-      <c r="L3" s="274"/>
-      <c r="M3" s="274"/>
-      <c r="N3" s="274"/>
-      <c r="O3" s="274"/>
+      <c r="A3" s="275" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" s="275"/>
+      <c r="C3" s="275"/>
+      <c r="D3" s="275"/>
+      <c r="E3" s="275"/>
+      <c r="F3" s="275"/>
+      <c r="G3" s="275"/>
+      <c r="H3" s="275"/>
+      <c r="I3" s="275"/>
+      <c r="J3" s="275"/>
+      <c r="K3" s="275"/>
+      <c r="L3" s="275"/>
+      <c r="M3" s="275"/>
+      <c r="N3" s="275"/>
+      <c r="O3" s="275"/>
       <c r="P3" s="76"/>
       <c r="Q3" s="76"/>
       <c r="R3" s="76"/>
@@ -11577,23 +11577,23 @@
       <c r="AP3" s="76"/>
     </row>
     <row r="4" spans="1:42" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="274" t="s">
-        <v>91</v>
-      </c>
-      <c r="B4" s="274"/>
-      <c r="C4" s="274"/>
-      <c r="D4" s="274"/>
-      <c r="E4" s="274"/>
-      <c r="F4" s="274"/>
-      <c r="G4" s="274"/>
-      <c r="H4" s="274"/>
-      <c r="I4" s="274"/>
-      <c r="J4" s="274"/>
-      <c r="K4" s="274"/>
-      <c r="L4" s="274"/>
-      <c r="M4" s="274"/>
-      <c r="N4" s="274"/>
-      <c r="O4" s="274"/>
+      <c r="A4" s="275" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" s="275"/>
+      <c r="C4" s="275"/>
+      <c r="D4" s="275"/>
+      <c r="E4" s="275"/>
+      <c r="F4" s="275"/>
+      <c r="G4" s="275"/>
+      <c r="H4" s="275"/>
+      <c r="I4" s="275"/>
+      <c r="J4" s="275"/>
+      <c r="K4" s="275"/>
+      <c r="L4" s="275"/>
+      <c r="M4" s="275"/>
+      <c r="N4" s="275"/>
+      <c r="O4" s="275"/>
       <c r="P4" s="76"/>
       <c r="Q4" s="76"/>
       <c r="R4" s="76"/>
@@ -11623,57 +11623,57 @@
       <c r="AP4" s="76"/>
     </row>
     <row r="5" spans="1:42" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="274" t="s">
-        <v>92</v>
-      </c>
-      <c r="B5" s="274"/>
-      <c r="C5" s="274"/>
-      <c r="D5" s="274"/>
-      <c r="E5" s="274"/>
-      <c r="F5" s="274"/>
-      <c r="G5" s="274"/>
-      <c r="H5" s="274"/>
-      <c r="I5" s="274"/>
-      <c r="J5" s="274"/>
-      <c r="K5" s="274"/>
-      <c r="L5" s="274"/>
-      <c r="M5" s="274"/>
-      <c r="N5" s="274"/>
-      <c r="O5" s="274"/>
+      <c r="A5" s="275" t="s">
+        <v>91</v>
+      </c>
+      <c r="B5" s="275"/>
+      <c r="C5" s="275"/>
+      <c r="D5" s="275"/>
+      <c r="E5" s="275"/>
+      <c r="F5" s="275"/>
+      <c r="G5" s="275"/>
+      <c r="H5" s="275"/>
+      <c r="I5" s="275"/>
+      <c r="J5" s="275"/>
+      <c r="K5" s="275"/>
+      <c r="L5" s="275"/>
+      <c r="M5" s="275"/>
+      <c r="N5" s="275"/>
+      <c r="O5" s="275"/>
     </row>
     <row r="6" spans="1:42" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="7" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A7" s="78" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:42" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="86" t="s">
-        <v>94</v>
-      </c>
-      <c r="D8" s="275" t="str">
+        <v>93</v>
+      </c>
+      <c r="D8" s="276" t="str">
         <f>IF('DR-TB 10A'!C8="","",'DR-TB 10A'!C8)</f>
         <v/>
       </c>
-      <c r="E8" s="275"/>
-      <c r="F8" s="275"/>
+      <c r="E8" s="276"/>
+      <c r="F8" s="276"/>
       <c r="G8" s="85"/>
       <c r="H8" s="79" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I8" s="92" t="str">
         <f>IF('DR-TB 10A'!L6="","",'DR-TB 10A'!L6)</f>
         <v/>
       </c>
       <c r="J8" s="79" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K8" s="93" t="str">
         <f>IF('DR-TB 10A'!N6="","",'DR-TB 10A'!N6)</f>
         <v/>
       </c>
       <c r="L8" s="87" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M8" s="87"/>
       <c r="O8" s="94" t="str">
@@ -11683,7 +11683,7 @@
     </row>
     <row r="9" spans="1:42" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="90" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F9" s="91">
         <f>'DR-TB 10A'!F18</f>
@@ -11693,49 +11693,49 @@
     <row r="10" spans="1:42" ht="4.6500000000000004" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="1:42" ht="76.650000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="88" t="s">
+        <v>97</v>
+      </c>
+      <c r="B11" s="89" t="s">
         <v>98</v>
       </c>
-      <c r="B11" s="89" t="s">
+      <c r="C11" s="89" t="s">
         <v>99</v>
       </c>
-      <c r="C11" s="89" t="s">
+      <c r="D11" s="89" t="s">
+        <v>111</v>
+      </c>
+      <c r="E11" s="89" t="s">
+        <v>115</v>
+      </c>
+      <c r="F11" s="89" t="s">
         <v>100</v>
       </c>
-      <c r="D11" s="89" t="s">
+      <c r="G11" s="89" t="s">
+        <v>101</v>
+      </c>
+      <c r="H11" s="89" t="s">
+        <v>102</v>
+      </c>
+      <c r="I11" s="89" t="s">
+        <v>103</v>
+      </c>
+      <c r="J11" s="89" t="s">
+        <v>104</v>
+      </c>
+      <c r="K11" s="89" t="s">
+        <v>105</v>
+      </c>
+      <c r="L11" s="89" t="s">
         <v>112</v>
       </c>
-      <c r="E11" s="89" t="s">
-        <v>116</v>
-      </c>
-      <c r="F11" s="89" t="s">
-        <v>101</v>
-      </c>
-      <c r="G11" s="89" t="s">
-        <v>102</v>
-      </c>
-      <c r="H11" s="89" t="s">
-        <v>103</v>
-      </c>
-      <c r="I11" s="89" t="s">
-        <v>104</v>
-      </c>
-      <c r="J11" s="89" t="s">
-        <v>105</v>
-      </c>
-      <c r="K11" s="89" t="s">
+      <c r="M11" s="89" t="s">
+        <v>139</v>
+      </c>
+      <c r="N11" s="89" t="s">
         <v>106</v>
       </c>
-      <c r="L11" s="89" t="s">
-        <v>113</v>
-      </c>
-      <c r="M11" s="89" t="s">
-        <v>140</v>
-      </c>
-      <c r="N11" s="89" t="s">
+      <c r="O11" s="89" t="s">
         <v>107</v>
-      </c>
-      <c r="O11" s="89" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="12" spans="1:42" s="99" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -12031,27 +12031,27 @@
       <c r="C29" s="80"/>
     </row>
     <row r="30" spans="1:15" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="273" t="s">
-        <v>109</v>
-      </c>
-      <c r="B30" s="273"/>
-      <c r="C30" s="273"/>
-      <c r="D30" s="273"/>
-      <c r="E30" s="273"/>
-      <c r="F30" s="273"/>
-      <c r="G30" s="273"/>
-      <c r="H30" s="273"/>
-      <c r="I30" s="273"/>
-      <c r="J30" s="273"/>
-      <c r="K30" s="273"/>
-      <c r="L30" s="273"/>
-      <c r="M30" s="273"/>
-      <c r="N30" s="273"/>
-      <c r="O30" s="273"/>
+      <c r="A30" s="274" t="s">
+        <v>108</v>
+      </c>
+      <c r="B30" s="274"/>
+      <c r="C30" s="274"/>
+      <c r="D30" s="274"/>
+      <c r="E30" s="274"/>
+      <c r="F30" s="274"/>
+      <c r="G30" s="274"/>
+      <c r="H30" s="274"/>
+      <c r="I30" s="274"/>
+      <c r="J30" s="274"/>
+      <c r="K30" s="274"/>
+      <c r="L30" s="274"/>
+      <c r="M30" s="274"/>
+      <c r="N30" s="274"/>
+      <c r="O30" s="274"/>
     </row>
     <row r="31" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="81" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B31" s="82"/>
       <c r="C31" s="82"/>
@@ -12070,7 +12070,7 @@
     </row>
     <row r="32" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="83" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B32" s="84"/>
       <c r="C32" s="84"/>
@@ -12130,78 +12130,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" s="65" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="280" t="s">
-        <v>136</v>
-      </c>
-      <c r="B1" s="280"/>
-      <c r="C1" s="280"/>
-      <c r="D1" s="280"/>
-      <c r="E1" s="280"/>
-      <c r="F1" s="280"/>
-      <c r="G1" s="280"/>
-      <c r="H1" s="280"/>
-      <c r="I1" s="280"/>
-      <c r="J1" s="280"/>
-      <c r="K1" s="280"/>
-      <c r="L1" s="280"/>
-      <c r="M1" s="280"/>
-      <c r="N1" s="280"/>
-      <c r="O1" s="280"/>
-      <c r="P1" s="281" t="s">
+      <c r="A1" s="311" t="s">
         <v>135</v>
       </c>
-      <c r="Q1" s="281"/>
-      <c r="R1" s="281"/>
-      <c r="S1" s="281"/>
+      <c r="B1" s="311"/>
+      <c r="C1" s="311"/>
+      <c r="D1" s="311"/>
+      <c r="E1" s="311"/>
+      <c r="F1" s="311"/>
+      <c r="G1" s="311"/>
+      <c r="H1" s="311"/>
+      <c r="I1" s="311"/>
+      <c r="J1" s="311"/>
+      <c r="K1" s="311"/>
+      <c r="L1" s="311"/>
+      <c r="M1" s="311"/>
+      <c r="N1" s="311"/>
+      <c r="O1" s="311"/>
+      <c r="P1" s="310" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q1" s="310"/>
+      <c r="R1" s="310"/>
+      <c r="S1" s="310"/>
       <c r="T1" s="130"/>
       <c r="U1" s="130"/>
     </row>
     <row r="2" spans="1:21" s="65" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A2" s="280" t="s">
-        <v>67</v>
-      </c>
-      <c r="B2" s="280"/>
-      <c r="C2" s="280"/>
-      <c r="D2" s="280"/>
-      <c r="E2" s="280"/>
-      <c r="F2" s="280"/>
-      <c r="G2" s="280"/>
-      <c r="H2" s="280"/>
-      <c r="I2" s="280"/>
-      <c r="J2" s="280"/>
-      <c r="K2" s="280"/>
-      <c r="L2" s="280"/>
-      <c r="M2" s="280"/>
-      <c r="N2" s="280"/>
-      <c r="O2" s="280"/>
-      <c r="P2" s="280"/>
-      <c r="Q2" s="280"/>
-      <c r="R2" s="280"/>
-      <c r="S2" s="280"/>
-      <c r="T2" s="280"/>
-      <c r="U2" s="280"/>
+      <c r="A2" s="311" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="311"/>
+      <c r="C2" s="311"/>
+      <c r="D2" s="311"/>
+      <c r="E2" s="311"/>
+      <c r="F2" s="311"/>
+      <c r="G2" s="311"/>
+      <c r="H2" s="311"/>
+      <c r="I2" s="311"/>
+      <c r="J2" s="311"/>
+      <c r="K2" s="311"/>
+      <c r="L2" s="311"/>
+      <c r="M2" s="311"/>
+      <c r="N2" s="311"/>
+      <c r="O2" s="311"/>
+      <c r="P2" s="311"/>
+      <c r="Q2" s="311"/>
+      <c r="R2" s="311"/>
+      <c r="S2" s="311"/>
+      <c r="T2" s="311"/>
+      <c r="U2" s="311"/>
     </row>
     <row r="3" spans="1:21" s="65" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A3" s="280" t="s">
-        <v>118</v>
-      </c>
-      <c r="B3" s="280"/>
-      <c r="C3" s="280"/>
-      <c r="D3" s="280"/>
-      <c r="E3" s="280"/>
-      <c r="F3" s="280"/>
-      <c r="G3" s="280"/>
-      <c r="H3" s="280"/>
-      <c r="I3" s="280"/>
-      <c r="J3" s="280"/>
-      <c r="K3" s="280"/>
-      <c r="L3" s="280"/>
-      <c r="M3" s="280"/>
-      <c r="N3" s="280"/>
-      <c r="O3" s="280"/>
-      <c r="P3" s="280"/>
-      <c r="Q3" s="280"/>
-      <c r="R3" s="280"/>
+      <c r="A3" s="311" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3" s="311"/>
+      <c r="C3" s="311"/>
+      <c r="D3" s="311"/>
+      <c r="E3" s="311"/>
+      <c r="F3" s="311"/>
+      <c r="G3" s="311"/>
+      <c r="H3" s="311"/>
+      <c r="I3" s="311"/>
+      <c r="J3" s="311"/>
+      <c r="K3" s="311"/>
+      <c r="L3" s="311"/>
+      <c r="M3" s="311"/>
+      <c r="N3" s="311"/>
+      <c r="O3" s="311"/>
+      <c r="P3" s="311"/>
+      <c r="Q3" s="311"/>
+      <c r="R3" s="311"/>
       <c r="S3" s="131"/>
       <c r="T3" s="131"/>
       <c r="U3" s="131"/>
@@ -12230,29 +12230,29 @@
       <c r="U4" s="131"/>
     </row>
     <row r="5" spans="1:21" s="65" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A5" s="281" t="s">
-        <v>119</v>
-      </c>
-      <c r="B5" s="281"/>
-      <c r="C5" s="281"/>
-      <c r="D5" s="281"/>
-      <c r="E5" s="281"/>
-      <c r="F5" s="281"/>
-      <c r="G5" s="281"/>
-      <c r="H5" s="281"/>
-      <c r="I5" s="281"/>
-      <c r="J5" s="281"/>
-      <c r="K5" s="281"/>
-      <c r="L5" s="281"/>
-      <c r="M5" s="281"/>
-      <c r="N5" s="281"/>
-      <c r="O5" s="281"/>
-      <c r="P5" s="281"/>
-      <c r="Q5" s="281"/>
-      <c r="R5" s="281"/>
-      <c r="S5" s="281"/>
-      <c r="T5" s="281"/>
-      <c r="U5" s="281"/>
+      <c r="A5" s="310" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="310"/>
+      <c r="C5" s="310"/>
+      <c r="D5" s="310"/>
+      <c r="E5" s="310"/>
+      <c r="F5" s="310"/>
+      <c r="G5" s="310"/>
+      <c r="H5" s="310"/>
+      <c r="I5" s="310"/>
+      <c r="J5" s="310"/>
+      <c r="K5" s="310"/>
+      <c r="L5" s="310"/>
+      <c r="M5" s="310"/>
+      <c r="N5" s="310"/>
+      <c r="O5" s="310"/>
+      <c r="P5" s="310"/>
+      <c r="Q5" s="310"/>
+      <c r="R5" s="310"/>
+      <c r="S5" s="310"/>
+      <c r="T5" s="310"/>
+      <c r="U5" s="310"/>
     </row>
     <row r="6" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="103"/>
@@ -12279,17 +12279,17 @@
     </row>
     <row r="7" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="104" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B7" s="104"/>
-      <c r="C7" s="291">
+      <c r="C7" s="313">
         <f>'DR-TB 10A'!C6:G6</f>
         <v>0</v>
       </c>
-      <c r="D7" s="291"/>
-      <c r="E7" s="291"/>
-      <c r="F7" s="291"/>
-      <c r="G7" s="291"/>
+      <c r="D7" s="313"/>
+      <c r="E7" s="313"/>
+      <c r="F7" s="313"/>
+      <c r="G7" s="313"/>
       <c r="H7" s="101"/>
       <c r="I7" s="104"/>
       <c r="J7" s="107" t="s">
@@ -12303,11 +12303,11 @@
       <c r="M7" s="108" t="s">
         <v>14</v>
       </c>
-      <c r="N7" s="290">
+      <c r="N7" s="312">
         <f>'DR-TB 10A'!N6:O6</f>
         <v>0</v>
       </c>
-      <c r="O7" s="290"/>
+      <c r="O7" s="312"/>
       <c r="P7" s="109" t="s">
         <v>15</v>
       </c>
@@ -12325,28 +12325,28 @@
         <v>9</v>
       </c>
       <c r="B8" s="104"/>
-      <c r="C8" s="300">
+      <c r="C8" s="297">
         <f>'DR-TB 10A'!C7:G7</f>
         <v>0</v>
       </c>
-      <c r="D8" s="300"/>
-      <c r="E8" s="300"/>
-      <c r="F8" s="300"/>
-      <c r="G8" s="300"/>
+      <c r="D8" s="297"/>
+      <c r="E8" s="297"/>
+      <c r="F8" s="297"/>
+      <c r="G8" s="297"/>
       <c r="H8" s="101"/>
       <c r="I8" s="110"/>
       <c r="J8" s="124" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="K8" s="123"/>
       <c r="L8" s="123"/>
       <c r="M8" s="123"/>
-      <c r="N8" s="296"/>
-      <c r="O8" s="296"/>
-      <c r="P8" s="296"/>
-      <c r="Q8" s="296"/>
-      <c r="R8" s="296"/>
-      <c r="S8" s="296"/>
+      <c r="N8" s="303"/>
+      <c r="O8" s="303"/>
+      <c r="P8" s="303"/>
+      <c r="Q8" s="303"/>
+      <c r="R8" s="303"/>
+      <c r="S8" s="303"/>
       <c r="T8" s="101"/>
       <c r="U8" s="101"/>
     </row>
@@ -12355,28 +12355,28 @@
         <v>10</v>
       </c>
       <c r="B9" s="104"/>
-      <c r="C9" s="301">
+      <c r="C9" s="299">
         <f>'DR-TB 10A'!C8:G8</f>
         <v>0</v>
       </c>
-      <c r="D9" s="301"/>
-      <c r="E9" s="301"/>
-      <c r="F9" s="301"/>
-      <c r="G9" s="301"/>
+      <c r="D9" s="299"/>
+      <c r="E9" s="299"/>
+      <c r="F9" s="299"/>
+      <c r="G9" s="299"/>
       <c r="H9" s="101"/>
       <c r="I9" s="110"/>
       <c r="J9" s="110" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K9" s="110"/>
       <c r="L9" s="110"/>
-      <c r="M9" s="296"/>
-      <c r="N9" s="296"/>
-      <c r="O9" s="296"/>
-      <c r="P9" s="296"/>
-      <c r="Q9" s="296"/>
-      <c r="R9" s="296"/>
-      <c r="S9" s="296"/>
+      <c r="M9" s="303"/>
+      <c r="N9" s="303"/>
+      <c r="O9" s="303"/>
+      <c r="P9" s="303"/>
+      <c r="Q9" s="303"/>
+      <c r="R9" s="303"/>
+      <c r="S9" s="303"/>
       <c r="T9" s="101"/>
       <c r="U9" s="101"/>
     </row>
@@ -12395,8 +12395,8 @@
       </c>
       <c r="K10" s="110"/>
       <c r="L10" s="110"/>
-      <c r="M10" s="297"/>
-      <c r="N10" s="297"/>
+      <c r="M10" s="304"/>
+      <c r="N10" s="304"/>
       <c r="O10" s="111"/>
       <c r="P10" s="102"/>
       <c r="Q10" s="101"/>
@@ -12416,19 +12416,19 @@
       <c r="H11" s="101"/>
       <c r="I11" s="101"/>
       <c r="J11" s="112" t="s">
-        <v>75</v>
-      </c>
-      <c r="K11" s="298"/>
-      <c r="L11" s="298"/>
+        <v>74</v>
+      </c>
+      <c r="K11" s="305"/>
+      <c r="L11" s="305"/>
       <c r="M11" s="112"/>
       <c r="N11" s="113"/>
       <c r="O11" s="110" t="s">
         <v>12</v>
       </c>
       <c r="P11" s="101"/>
-      <c r="Q11" s="299"/>
-      <c r="R11" s="299"/>
-      <c r="S11" s="299"/>
+      <c r="Q11" s="306"/>
+      <c r="R11" s="306"/>
+      <c r="S11" s="306"/>
       <c r="T11" s="106"/>
       <c r="U11" s="101"/>
     </row>
@@ -12456,34 +12456,34 @@
       <c r="U12" s="101"/>
     </row>
     <row r="13" spans="1:21" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="303" t="s">
+      <c r="A13" s="277" t="s">
+        <v>120</v>
+      </c>
+      <c r="B13" s="300" t="s">
         <v>121</v>
       </c>
-      <c r="B13" s="302" t="s">
+      <c r="C13" s="300"/>
+      <c r="D13" s="300" t="s">
         <v>122</v>
       </c>
-      <c r="C13" s="302"/>
-      <c r="D13" s="302" t="s">
-        <v>123</v>
-      </c>
-      <c r="E13" s="302"/>
+      <c r="E13" s="300"/>
       <c r="F13" s="101"/>
       <c r="G13" s="101"/>
-      <c r="H13" s="305" t="s">
+      <c r="H13" s="280" t="s">
+        <v>123</v>
+      </c>
+      <c r="I13" s="281"/>
+      <c r="J13" s="281"/>
+      <c r="K13" s="282"/>
+      <c r="L13" s="286" t="s">
         <v>124</v>
       </c>
-      <c r="I13" s="306"/>
-      <c r="J13" s="306"/>
-      <c r="K13" s="307"/>
-      <c r="L13" s="311" t="s">
-        <v>125</v>
-      </c>
-      <c r="M13" s="311"/>
-      <c r="N13" s="311"/>
-      <c r="O13" s="312" t="s">
+      <c r="M13" s="286"/>
+      <c r="N13" s="286"/>
+      <c r="O13" s="287" t="s">
         <v>3</v>
       </c>
-      <c r="P13" s="313"/>
+      <c r="P13" s="288"/>
       <c r="Q13" s="106"/>
       <c r="R13" s="101"/>
       <c r="S13" s="101"/>
@@ -12491,25 +12491,25 @@
       <c r="U13" s="101"/>
     </row>
     <row r="14" spans="1:21" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="304"/>
-      <c r="B14" s="282"/>
-      <c r="C14" s="283"/>
-      <c r="D14" s="282"/>
-      <c r="E14" s="283"/>
+      <c r="A14" s="278"/>
+      <c r="B14" s="301"/>
+      <c r="C14" s="302"/>
+      <c r="D14" s="301"/>
+      <c r="E14" s="302"/>
       <c r="F14" s="101"/>
       <c r="G14" s="101"/>
-      <c r="H14" s="308"/>
-      <c r="I14" s="309"/>
-      <c r="J14" s="309"/>
-      <c r="K14" s="310"/>
+      <c r="H14" s="283"/>
+      <c r="I14" s="284"/>
+      <c r="J14" s="284"/>
+      <c r="K14" s="285"/>
       <c r="L14" s="136"/>
       <c r="M14" s="137"/>
       <c r="N14" s="138"/>
-      <c r="O14" s="314">
+      <c r="O14" s="289">
         <f>L14+M14+N14</f>
         <v>0</v>
       </c>
-      <c r="P14" s="315"/>
+      <c r="P14" s="290"/>
       <c r="Q14" s="106"/>
       <c r="R14" s="101"/>
       <c r="S14" s="101"/>
@@ -12563,351 +12563,351 @@
       <c r="U16" s="118"/>
     </row>
     <row r="17" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="316"/>
-      <c r="B17" s="316"/>
-      <c r="C17" s="287" t="s">
+      <c r="A17" s="295"/>
+      <c r="B17" s="295"/>
+      <c r="C17" s="291" t="s">
+        <v>125</v>
+      </c>
+      <c r="D17" s="291"/>
+      <c r="E17" s="291"/>
+      <c r="F17" s="309" t="s">
         <v>126</v>
       </c>
-      <c r="D17" s="287"/>
-      <c r="E17" s="287"/>
-      <c r="F17" s="294" t="s">
+      <c r="G17" s="309"/>
+      <c r="H17" s="309"/>
+      <c r="I17" s="309"/>
+      <c r="J17" s="309"/>
+      <c r="K17" s="309"/>
+      <c r="L17" s="291" t="s">
         <v>127</v>
       </c>
-      <c r="G17" s="294"/>
-      <c r="H17" s="294"/>
-      <c r="I17" s="294"/>
-      <c r="J17" s="294"/>
-      <c r="K17" s="294"/>
-      <c r="L17" s="287" t="s">
-        <v>128</v>
-      </c>
-      <c r="M17" s="287"/>
-      <c r="N17" s="287"/>
-      <c r="O17" s="287"/>
-      <c r="P17" s="287"/>
-      <c r="Q17" s="287"/>
+      <c r="M17" s="291"/>
+      <c r="N17" s="291"/>
+      <c r="O17" s="291"/>
+      <c r="P17" s="291"/>
+      <c r="Q17" s="291"/>
       <c r="R17" s="101"/>
       <c r="S17" s="101"/>
       <c r="T17" s="101"/>
-      <c r="U17" s="292"/>
+      <c r="U17" s="307"/>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A18" s="316"/>
-      <c r="B18" s="316"/>
-      <c r="C18" s="295" t="s">
+      <c r="A18" s="295"/>
+      <c r="B18" s="295"/>
+      <c r="C18" s="298" t="s">
+        <v>128</v>
+      </c>
+      <c r="D18" s="298" t="s">
         <v>129</v>
       </c>
-      <c r="D18" s="295" t="s">
-        <v>130</v>
-      </c>
-      <c r="E18" s="295" t="s">
+      <c r="E18" s="298" t="s">
         <v>3</v>
       </c>
-      <c r="F18" s="294" t="s">
+      <c r="F18" s="309" t="s">
+        <v>128</v>
+      </c>
+      <c r="G18" s="309"/>
+      <c r="H18" s="309" t="s">
         <v>129</v>
       </c>
-      <c r="G18" s="294"/>
-      <c r="H18" s="294" t="s">
-        <v>130</v>
-      </c>
-      <c r="I18" s="294"/>
-      <c r="J18" s="294" t="s">
+      <c r="I18" s="309"/>
+      <c r="J18" s="309" t="s">
         <v>3</v>
       </c>
-      <c r="K18" s="294"/>
-      <c r="L18" s="287" t="s">
+      <c r="K18" s="309"/>
+      <c r="L18" s="291" t="s">
+        <v>128</v>
+      </c>
+      <c r="M18" s="291"/>
+      <c r="N18" s="291" t="s">
         <v>129</v>
       </c>
-      <c r="M18" s="287"/>
-      <c r="N18" s="287" t="s">
-        <v>130</v>
-      </c>
-      <c r="O18" s="287"/>
-      <c r="P18" s="295" t="s">
+      <c r="O18" s="291"/>
+      <c r="P18" s="298" t="s">
         <v>3</v>
       </c>
-      <c r="Q18" s="295"/>
+      <c r="Q18" s="298"/>
       <c r="R18" s="101"/>
       <c r="S18" s="101"/>
       <c r="T18" s="101"/>
-      <c r="U18" s="292"/>
+      <c r="U18" s="307"/>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A19" s="316"/>
-      <c r="B19" s="316"/>
-      <c r="C19" s="295"/>
-      <c r="D19" s="295"/>
-      <c r="E19" s="295"/>
-      <c r="F19" s="294"/>
-      <c r="G19" s="294"/>
-      <c r="H19" s="294"/>
-      <c r="I19" s="294"/>
-      <c r="J19" s="294"/>
-      <c r="K19" s="294"/>
-      <c r="L19" s="287"/>
-      <c r="M19" s="287"/>
-      <c r="N19" s="287"/>
-      <c r="O19" s="287"/>
-      <c r="P19" s="295"/>
-      <c r="Q19" s="295"/>
+      <c r="A19" s="295"/>
+      <c r="B19" s="295"/>
+      <c r="C19" s="298"/>
+      <c r="D19" s="298"/>
+      <c r="E19" s="298"/>
+      <c r="F19" s="309"/>
+      <c r="G19" s="309"/>
+      <c r="H19" s="309"/>
+      <c r="I19" s="309"/>
+      <c r="J19" s="309"/>
+      <c r="K19" s="309"/>
+      <c r="L19" s="291"/>
+      <c r="M19" s="291"/>
+      <c r="N19" s="291"/>
+      <c r="O19" s="291"/>
+      <c r="P19" s="298"/>
+      <c r="Q19" s="298"/>
       <c r="R19" s="101"/>
       <c r="S19" s="101"/>
       <c r="T19" s="101"/>
-      <c r="U19" s="292"/>
+      <c r="U19" s="307"/>
     </row>
     <row r="20" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="287" t="s">
-        <v>131</v>
-      </c>
-      <c r="B20" s="287"/>
-      <c r="C20" s="288"/>
-      <c r="D20" s="288"/>
-      <c r="E20" s="286">
+      <c r="A20" s="291" t="s">
+        <v>130</v>
+      </c>
+      <c r="B20" s="291"/>
+      <c r="C20" s="296"/>
+      <c r="D20" s="296"/>
+      <c r="E20" s="279">
         <f>C20+D20</f>
         <v>0</v>
       </c>
-      <c r="F20" s="289"/>
-      <c r="G20" s="289"/>
-      <c r="H20" s="278"/>
-      <c r="I20" s="278"/>
-      <c r="J20" s="279">
+      <c r="F20" s="293"/>
+      <c r="G20" s="293"/>
+      <c r="H20" s="294"/>
+      <c r="I20" s="294"/>
+      <c r="J20" s="292">
         <f>F20+H20</f>
         <v>0</v>
       </c>
-      <c r="K20" s="279"/>
-      <c r="L20" s="286">
+      <c r="K20" s="292"/>
+      <c r="L20" s="279">
         <f>C20+F20</f>
         <v>0</v>
       </c>
-      <c r="M20" s="286"/>
-      <c r="N20" s="286">
+      <c r="M20" s="279"/>
+      <c r="N20" s="279">
         <f>D20+H20</f>
         <v>0</v>
       </c>
-      <c r="O20" s="286"/>
-      <c r="P20" s="286">
+      <c r="O20" s="279"/>
+      <c r="P20" s="279">
         <f>L20+N20</f>
         <v>0</v>
       </c>
-      <c r="Q20" s="286"/>
+      <c r="Q20" s="279"/>
       <c r="R20" s="101"/>
       <c r="S20" s="101"/>
       <c r="T20" s="101"/>
-      <c r="U20" s="293"/>
+      <c r="U20" s="308"/>
     </row>
     <row r="21" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="287"/>
-      <c r="B21" s="287"/>
-      <c r="C21" s="288"/>
-      <c r="D21" s="288"/>
-      <c r="E21" s="286"/>
-      <c r="F21" s="289"/>
-      <c r="G21" s="289"/>
-      <c r="H21" s="278"/>
-      <c r="I21" s="278"/>
-      <c r="J21" s="279"/>
-      <c r="K21" s="279"/>
-      <c r="L21" s="286"/>
-      <c r="M21" s="286"/>
-      <c r="N21" s="286"/>
-      <c r="O21" s="286"/>
-      <c r="P21" s="286"/>
-      <c r="Q21" s="286"/>
+      <c r="A21" s="291"/>
+      <c r="B21" s="291"/>
+      <c r="C21" s="296"/>
+      <c r="D21" s="296"/>
+      <c r="E21" s="279"/>
+      <c r="F21" s="293"/>
+      <c r="G21" s="293"/>
+      <c r="H21" s="294"/>
+      <c r="I21" s="294"/>
+      <c r="J21" s="292"/>
+      <c r="K21" s="292"/>
+      <c r="L21" s="279"/>
+      <c r="M21" s="279"/>
+      <c r="N21" s="279"/>
+      <c r="O21" s="279"/>
+      <c r="P21" s="279"/>
+      <c r="Q21" s="279"/>
       <c r="R21" s="101"/>
       <c r="S21" s="101"/>
       <c r="T21" s="101"/>
-      <c r="U21" s="293"/>
+      <c r="U21" s="308"/>
     </row>
     <row r="22" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="287"/>
-      <c r="B22" s="287"/>
-      <c r="C22" s="288"/>
-      <c r="D22" s="288"/>
-      <c r="E22" s="286"/>
-      <c r="F22" s="289"/>
-      <c r="G22" s="289"/>
-      <c r="H22" s="278"/>
-      <c r="I22" s="278"/>
-      <c r="J22" s="279"/>
-      <c r="K22" s="279"/>
-      <c r="L22" s="286"/>
-      <c r="M22" s="286"/>
-      <c r="N22" s="286"/>
-      <c r="O22" s="286"/>
-      <c r="P22" s="286"/>
-      <c r="Q22" s="286"/>
+      <c r="A22" s="291"/>
+      <c r="B22" s="291"/>
+      <c r="C22" s="296"/>
+      <c r="D22" s="296"/>
+      <c r="E22" s="279"/>
+      <c r="F22" s="293"/>
+      <c r="G22" s="293"/>
+      <c r="H22" s="294"/>
+      <c r="I22" s="294"/>
+      <c r="J22" s="292"/>
+      <c r="K22" s="292"/>
+      <c r="L22" s="279"/>
+      <c r="M22" s="279"/>
+      <c r="N22" s="279"/>
+      <c r="O22" s="279"/>
+      <c r="P22" s="279"/>
+      <c r="Q22" s="279"/>
       <c r="R22" s="101"/>
       <c r="S22" s="101"/>
       <c r="T22" s="101"/>
-      <c r="U22" s="293"/>
+      <c r="U22" s="308"/>
     </row>
     <row r="23" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="287" t="s">
-        <v>132</v>
-      </c>
-      <c r="B23" s="287"/>
-      <c r="C23" s="288"/>
-      <c r="D23" s="288"/>
-      <c r="E23" s="286">
+      <c r="A23" s="291" t="s">
+        <v>131</v>
+      </c>
+      <c r="B23" s="291"/>
+      <c r="C23" s="296"/>
+      <c r="D23" s="296"/>
+      <c r="E23" s="279">
         <f t="shared" ref="E23" si="0">C23+D23</f>
         <v>0</v>
       </c>
-      <c r="F23" s="289"/>
-      <c r="G23" s="289"/>
-      <c r="H23" s="278"/>
-      <c r="I23" s="278"/>
-      <c r="J23" s="279">
+      <c r="F23" s="293"/>
+      <c r="G23" s="293"/>
+      <c r="H23" s="294"/>
+      <c r="I23" s="294"/>
+      <c r="J23" s="292">
         <f t="shared" ref="J23" si="1">F23+H23</f>
         <v>0</v>
       </c>
-      <c r="K23" s="279"/>
-      <c r="L23" s="286">
+      <c r="K23" s="292"/>
+      <c r="L23" s="279">
         <f t="shared" ref="L23" si="2">C23+F23</f>
         <v>0</v>
       </c>
-      <c r="M23" s="286"/>
-      <c r="N23" s="286">
+      <c r="M23" s="279"/>
+      <c r="N23" s="279">
         <f t="shared" ref="N23" si="3">D23+H23</f>
         <v>0</v>
       </c>
-      <c r="O23" s="286"/>
-      <c r="P23" s="286">
+      <c r="O23" s="279"/>
+      <c r="P23" s="279">
         <f t="shared" ref="P23" si="4">L23+N23</f>
         <v>0</v>
       </c>
-      <c r="Q23" s="286"/>
+      <c r="Q23" s="279"/>
       <c r="R23" s="101"/>
       <c r="S23" s="101"/>
       <c r="T23" s="101"/>
       <c r="U23" s="134"/>
     </row>
     <row r="24" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="287"/>
-      <c r="B24" s="287"/>
-      <c r="C24" s="288"/>
-      <c r="D24" s="288"/>
-      <c r="E24" s="286"/>
-      <c r="F24" s="289"/>
-      <c r="G24" s="289"/>
-      <c r="H24" s="278"/>
-      <c r="I24" s="278"/>
-      <c r="J24" s="279"/>
-      <c r="K24" s="279"/>
-      <c r="L24" s="286"/>
-      <c r="M24" s="286"/>
-      <c r="N24" s="286"/>
-      <c r="O24" s="286"/>
-      <c r="P24" s="286"/>
-      <c r="Q24" s="286"/>
+      <c r="A24" s="291"/>
+      <c r="B24" s="291"/>
+      <c r="C24" s="296"/>
+      <c r="D24" s="296"/>
+      <c r="E24" s="279"/>
+      <c r="F24" s="293"/>
+      <c r="G24" s="293"/>
+      <c r="H24" s="294"/>
+      <c r="I24" s="294"/>
+      <c r="J24" s="292"/>
+      <c r="K24" s="292"/>
+      <c r="L24" s="279"/>
+      <c r="M24" s="279"/>
+      <c r="N24" s="279"/>
+      <c r="O24" s="279"/>
+      <c r="P24" s="279"/>
+      <c r="Q24" s="279"/>
       <c r="R24" s="101"/>
       <c r="S24" s="101"/>
       <c r="T24" s="101"/>
       <c r="U24" s="134"/>
     </row>
     <row r="25" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="287"/>
-      <c r="B25" s="287"/>
-      <c r="C25" s="288"/>
-      <c r="D25" s="288"/>
-      <c r="E25" s="286"/>
-      <c r="F25" s="289"/>
-      <c r="G25" s="289"/>
-      <c r="H25" s="278"/>
-      <c r="I25" s="278"/>
-      <c r="J25" s="279"/>
-      <c r="K25" s="279"/>
-      <c r="L25" s="286"/>
-      <c r="M25" s="286"/>
-      <c r="N25" s="286"/>
-      <c r="O25" s="286"/>
-      <c r="P25" s="286"/>
-      <c r="Q25" s="286"/>
+      <c r="A25" s="291"/>
+      <c r="B25" s="291"/>
+      <c r="C25" s="296"/>
+      <c r="D25" s="296"/>
+      <c r="E25" s="279"/>
+      <c r="F25" s="293"/>
+      <c r="G25" s="293"/>
+      <c r="H25" s="294"/>
+      <c r="I25" s="294"/>
+      <c r="J25" s="292"/>
+      <c r="K25" s="292"/>
+      <c r="L25" s="279"/>
+      <c r="M25" s="279"/>
+      <c r="N25" s="279"/>
+      <c r="O25" s="279"/>
+      <c r="P25" s="279"/>
+      <c r="Q25" s="279"/>
       <c r="R25" s="101"/>
       <c r="S25" s="101"/>
       <c r="T25" s="101"/>
       <c r="U25" s="134"/>
     </row>
     <row r="26" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="287" t="s">
-        <v>133</v>
-      </c>
-      <c r="B26" s="287"/>
-      <c r="C26" s="288"/>
-      <c r="D26" s="288"/>
-      <c r="E26" s="286">
+      <c r="A26" s="291" t="s">
+        <v>132</v>
+      </c>
+      <c r="B26" s="291"/>
+      <c r="C26" s="296"/>
+      <c r="D26" s="296"/>
+      <c r="E26" s="279">
         <f t="shared" ref="E26" si="5">C26+D26</f>
         <v>0</v>
       </c>
-      <c r="F26" s="289"/>
-      <c r="G26" s="289"/>
-      <c r="H26" s="278"/>
-      <c r="I26" s="278"/>
-      <c r="J26" s="279">
+      <c r="F26" s="293"/>
+      <c r="G26" s="293"/>
+      <c r="H26" s="294"/>
+      <c r="I26" s="294"/>
+      <c r="J26" s="292">
         <f t="shared" ref="J26" si="6">F26+H26</f>
         <v>0</v>
       </c>
-      <c r="K26" s="279"/>
-      <c r="L26" s="286">
+      <c r="K26" s="292"/>
+      <c r="L26" s="279">
         <f t="shared" ref="L26" si="7">C26+F26</f>
         <v>0</v>
       </c>
-      <c r="M26" s="286"/>
-      <c r="N26" s="286">
+      <c r="M26" s="279"/>
+      <c r="N26" s="279">
         <f t="shared" ref="N26" si="8">D26+H26</f>
         <v>0</v>
       </c>
-      <c r="O26" s="286"/>
-      <c r="P26" s="286">
+      <c r="O26" s="279"/>
+      <c r="P26" s="279">
         <f t="shared" ref="P26" si="9">L26+N26</f>
         <v>0</v>
       </c>
-      <c r="Q26" s="286"/>
+      <c r="Q26" s="279"/>
       <c r="R26" s="125"/>
       <c r="S26" s="135"/>
       <c r="T26" s="135"/>
       <c r="U26" s="134"/>
     </row>
     <row r="27" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="287"/>
-      <c r="B27" s="287"/>
-      <c r="C27" s="288"/>
-      <c r="D27" s="288"/>
-      <c r="E27" s="286"/>
-      <c r="F27" s="289"/>
-      <c r="G27" s="289"/>
-      <c r="H27" s="278"/>
-      <c r="I27" s="278"/>
-      <c r="J27" s="279"/>
-      <c r="K27" s="279"/>
-      <c r="L27" s="286"/>
-      <c r="M27" s="286"/>
-      <c r="N27" s="286"/>
-      <c r="O27" s="286"/>
-      <c r="P27" s="286"/>
-      <c r="Q27" s="286"/>
+      <c r="A27" s="291"/>
+      <c r="B27" s="291"/>
+      <c r="C27" s="296"/>
+      <c r="D27" s="296"/>
+      <c r="E27" s="279"/>
+      <c r="F27" s="293"/>
+      <c r="G27" s="293"/>
+      <c r="H27" s="294"/>
+      <c r="I27" s="294"/>
+      <c r="J27" s="292"/>
+      <c r="K27" s="292"/>
+      <c r="L27" s="279"/>
+      <c r="M27" s="279"/>
+      <c r="N27" s="279"/>
+      <c r="O27" s="279"/>
+      <c r="P27" s="279"/>
+      <c r="Q27" s="279"/>
       <c r="R27" s="125"/>
       <c r="S27" s="135"/>
       <c r="T27" s="135"/>
       <c r="U27" s="134"/>
     </row>
     <row r="28" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="287"/>
-      <c r="B28" s="287"/>
-      <c r="C28" s="288"/>
-      <c r="D28" s="288"/>
-      <c r="E28" s="286"/>
-      <c r="F28" s="289"/>
-      <c r="G28" s="289"/>
-      <c r="H28" s="278"/>
-      <c r="I28" s="278"/>
-      <c r="J28" s="279"/>
-      <c r="K28" s="279"/>
-      <c r="L28" s="286"/>
-      <c r="M28" s="286"/>
-      <c r="N28" s="286"/>
-      <c r="O28" s="286"/>
-      <c r="P28" s="286"/>
-      <c r="Q28" s="286"/>
+      <c r="A28" s="291"/>
+      <c r="B28" s="291"/>
+      <c r="C28" s="296"/>
+      <c r="D28" s="296"/>
+      <c r="E28" s="279"/>
+      <c r="F28" s="293"/>
+      <c r="G28" s="293"/>
+      <c r="H28" s="294"/>
+      <c r="I28" s="294"/>
+      <c r="J28" s="292"/>
+      <c r="K28" s="292"/>
+      <c r="L28" s="279"/>
+      <c r="M28" s="279"/>
+      <c r="N28" s="279"/>
+      <c r="O28" s="279"/>
+      <c r="P28" s="279"/>
+      <c r="Q28" s="279"/>
       <c r="R28" s="125"/>
       <c r="S28" s="135"/>
       <c r="T28" s="135"/>
@@ -12945,19 +12945,19 @@
       <c r="F30" s="101"/>
       <c r="G30" s="101"/>
       <c r="H30" s="105" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I30" s="106"/>
       <c r="J30" s="106"/>
       <c r="K30" s="106"/>
       <c r="L30" s="106"/>
-      <c r="M30" s="284"/>
-      <c r="N30" s="284"/>
-      <c r="O30" s="284"/>
-      <c r="P30" s="284"/>
-      <c r="Q30" s="284"/>
-      <c r="R30" s="284"/>
-      <c r="S30" s="284"/>
+      <c r="M30" s="314"/>
+      <c r="N30" s="314"/>
+      <c r="O30" s="314"/>
+      <c r="P30" s="314"/>
+      <c r="Q30" s="314"/>
+      <c r="R30" s="314"/>
+      <c r="S30" s="314"/>
       <c r="T30" s="101"/>
       <c r="U30" s="101"/>
     </row>
@@ -12970,19 +12970,19 @@
       <c r="F31" s="126"/>
       <c r="G31" s="127"/>
       <c r="H31" s="105" t="s">
-        <v>59</v>
-      </c>
-      <c r="I31" s="277"/>
-      <c r="J31" s="277"/>
-      <c r="K31" s="277"/>
-      <c r="L31" s="277"/>
+        <v>58</v>
+      </c>
+      <c r="I31" s="317"/>
+      <c r="J31" s="317"/>
+      <c r="K31" s="317"/>
+      <c r="L31" s="317"/>
       <c r="M31" s="101"/>
       <c r="N31" s="119" t="s">
-        <v>60</v>
-      </c>
-      <c r="O31" s="285"/>
-      <c r="P31" s="285"/>
-      <c r="Q31" s="285"/>
+        <v>59</v>
+      </c>
+      <c r="O31" s="315"/>
+      <c r="P31" s="315"/>
+      <c r="Q31" s="315"/>
     </row>
     <row r="32" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A32" s="128"/>
@@ -12993,13 +12993,13 @@
       <c r="F32" s="127"/>
       <c r="G32" s="129"/>
       <c r="H32" s="105" t="s">
-        <v>61</v>
-      </c>
-      <c r="I32" s="276"/>
-      <c r="J32" s="276"/>
-      <c r="K32" s="276"/>
-      <c r="L32" s="276"/>
-      <c r="M32" s="276"/>
+        <v>60</v>
+      </c>
+      <c r="I32" s="316"/>
+      <c r="J32" s="316"/>
+      <c r="K32" s="316"/>
+      <c r="L32" s="316"/>
+      <c r="M32" s="316"/>
       <c r="N32" s="101"/>
       <c r="O32" s="101"/>
       <c r="P32" s="101"/>
@@ -13026,6 +13026,62 @@
     </row>
   </sheetData>
   <mergeCells count="72">
+    <mergeCell ref="I32:M32"/>
+    <mergeCell ref="I31:L31"/>
+    <mergeCell ref="H23:I25"/>
+    <mergeCell ref="J26:K28"/>
+    <mergeCell ref="H20:I22"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="P1:S1"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="M30:S30"/>
+    <mergeCell ref="O31:Q31"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="A20:B22"/>
+    <mergeCell ref="C23:C25"/>
+    <mergeCell ref="D23:D25"/>
+    <mergeCell ref="E23:E25"/>
+    <mergeCell ref="F23:G25"/>
+    <mergeCell ref="A26:B28"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="D26:D28"/>
+    <mergeCell ref="E26:E28"/>
+    <mergeCell ref="A23:B25"/>
+    <mergeCell ref="A5:U5"/>
+    <mergeCell ref="A2:U2"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="N7:O7"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="U17:U19"/>
+    <mergeCell ref="U20:U22"/>
+    <mergeCell ref="J23:K25"/>
+    <mergeCell ref="F18:G19"/>
+    <mergeCell ref="H18:I19"/>
+    <mergeCell ref="J18:K19"/>
+    <mergeCell ref="F17:K17"/>
+    <mergeCell ref="L18:M19"/>
+    <mergeCell ref="L17:Q17"/>
+    <mergeCell ref="P18:Q19"/>
+    <mergeCell ref="L20:M22"/>
+    <mergeCell ref="L23:M25"/>
+    <mergeCell ref="N20:O22"/>
+    <mergeCell ref="N23:O25"/>
+    <mergeCell ref="P20:Q22"/>
+    <mergeCell ref="P23:Q25"/>
+    <mergeCell ref="N8:S8"/>
+    <mergeCell ref="M9:S9"/>
+    <mergeCell ref="M10:N10"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="Q11:S11"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="B14:C14"/>
     <mergeCell ref="A13:A14"/>
     <mergeCell ref="L26:M28"/>
     <mergeCell ref="N26:O28"/>
@@ -13042,62 +13098,6 @@
     <mergeCell ref="C20:C22"/>
     <mergeCell ref="D20:D22"/>
     <mergeCell ref="F20:G22"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="N8:S8"/>
-    <mergeCell ref="M9:S9"/>
-    <mergeCell ref="M10:N10"/>
-    <mergeCell ref="K11:L11"/>
-    <mergeCell ref="Q11:S11"/>
-    <mergeCell ref="U17:U19"/>
-    <mergeCell ref="U20:U22"/>
-    <mergeCell ref="J23:K25"/>
-    <mergeCell ref="F18:G19"/>
-    <mergeCell ref="H18:I19"/>
-    <mergeCell ref="J18:K19"/>
-    <mergeCell ref="F17:K17"/>
-    <mergeCell ref="L18:M19"/>
-    <mergeCell ref="L17:Q17"/>
-    <mergeCell ref="P18:Q19"/>
-    <mergeCell ref="L20:M22"/>
-    <mergeCell ref="L23:M25"/>
-    <mergeCell ref="N20:O22"/>
-    <mergeCell ref="N23:O25"/>
-    <mergeCell ref="P20:Q22"/>
-    <mergeCell ref="P23:Q25"/>
-    <mergeCell ref="A5:U5"/>
-    <mergeCell ref="A2:U2"/>
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="N7:O7"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="P1:S1"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="M30:S30"/>
-    <mergeCell ref="O31:Q31"/>
-    <mergeCell ref="E20:E22"/>
-    <mergeCell ref="A20:B22"/>
-    <mergeCell ref="C23:C25"/>
-    <mergeCell ref="D23:D25"/>
-    <mergeCell ref="E23:E25"/>
-    <mergeCell ref="F23:G25"/>
-    <mergeCell ref="A26:B28"/>
-    <mergeCell ref="C26:C28"/>
-    <mergeCell ref="D26:D28"/>
-    <mergeCell ref="E26:E28"/>
-    <mergeCell ref="A23:B25"/>
-    <mergeCell ref="I32:M32"/>
-    <mergeCell ref="I31:L31"/>
-    <mergeCell ref="H23:I25"/>
-    <mergeCell ref="J26:K28"/>
-    <mergeCell ref="H20:I22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>